<commit_message>
feat: watchdog for reload
</commit_message>
<xml_diff>
--- a/users/uzuran/burn_table.xlsx
+++ b/users/uzuran/burn_table.xlsx
@@ -67,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -101,6 +101,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -538,506 +547,506 @@
       <c r="J1" s="3" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="14" t="n"/>
-      <c r="B2" s="14" t="n"/>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="14" t="n"/>
-      <c r="G2" s="14" t="n"/>
-      <c r="H2" s="14" t="n"/>
+      <c r="A2" s="17" t="n"/>
+      <c r="B2" s="17" t="n"/>
+      <c r="C2" s="17" t="n"/>
+      <c r="D2" s="17" t="n"/>
+      <c r="E2" s="17" t="n"/>
+      <c r="F2" s="17" t="n"/>
+      <c r="G2" s="17" t="n"/>
+      <c r="H2" s="17" t="n"/>
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>14.07.2026</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>4039-95</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>1.0026-2X2500X1250</t>
         </is>
       </c>
-      <c r="D3" s="14" t="n">
+      <c r="D3" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>00:04:03</t>
         </is>
       </c>
-      <c r="F3" s="14" t="n"/>
-      <c r="G3" s="14" t="n"/>
-      <c r="H3" s="14" t="n"/>
+      <c r="F3" s="17" t="n"/>
+      <c r="G3" s="17" t="n"/>
+      <c r="H3" s="17" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="15" t="n"/>
-      <c r="B4" s="15" t="n"/>
-      <c r="C4" s="15" t="n"/>
-      <c r="D4" s="15" t="n"/>
-      <c r="E4" s="15" t="n"/>
-      <c r="F4" s="15" t="n"/>
-      <c r="G4" s="15" t="n"/>
-      <c r="H4" s="15" t="n"/>
+      <c r="A4" s="18" t="n"/>
+      <c r="B4" s="18" t="n"/>
+      <c r="C4" s="18" t="n"/>
+      <c r="D4" s="18" t="n"/>
+      <c r="E4" s="18" t="n"/>
+      <c r="F4" s="18" t="n"/>
+      <c r="G4" s="18" t="n"/>
+      <c r="H4" s="18" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>14.07.2026</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>4039-95</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>-----</t>
         </is>
       </c>
-      <c r="D5" s="14" t="n">
+      <c r="D5" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>00:04:03</t>
         </is>
       </c>
-      <c r="F5" s="14" t="n"/>
-      <c r="G5" s="14" t="n"/>
-      <c r="H5" s="14" t="n"/>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="17" t="n"/>
+      <c r="H5" s="17" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="15" t="n"/>
-      <c r="B6" s="15" t="n"/>
-      <c r="C6" s="15" t="n"/>
-      <c r="D6" s="15" t="n"/>
-      <c r="E6" s="15" t="n"/>
-      <c r="F6" s="15" t="n"/>
-      <c r="G6" s="15" t="n"/>
-      <c r="H6" s="15" t="n"/>
+      <c r="A6" s="18" t="n"/>
+      <c r="B6" s="18" t="n"/>
+      <c r="C6" s="18" t="n"/>
+      <c r="D6" s="18" t="n"/>
+      <c r="E6" s="18" t="n"/>
+      <c r="F6" s="18" t="n"/>
+      <c r="G6" s="18" t="n"/>
+      <c r="H6" s="18" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="14" t="n"/>
-      <c r="B7" s="14" t="n"/>
-      <c r="C7" s="14" t="n"/>
-      <c r="D7" s="14" t="n"/>
-      <c r="E7" s="14" t="n"/>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="14" t="n"/>
-      <c r="H7" s="14" t="n"/>
+      <c r="A7" s="17" t="n"/>
+      <c r="B7" s="17" t="n"/>
+      <c r="C7" s="17" t="n"/>
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="17" t="n"/>
+      <c r="F7" s="17" t="n"/>
+      <c r="G7" s="17" t="n"/>
+      <c r="H7" s="17" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="14" t="n"/>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
-      <c r="E8" s="14" t="n"/>
-      <c r="F8" s="14" t="n"/>
-      <c r="G8" s="14" t="n"/>
-      <c r="H8" s="14" t="n"/>
+      <c r="A8" s="17" t="n"/>
+      <c r="B8" s="17" t="n"/>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="17" t="n"/>
+      <c r="F8" s="17" t="n"/>
+      <c r="G8" s="17" t="n"/>
+      <c r="H8" s="17" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="14" t="n"/>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
-      <c r="E9" s="14" t="n"/>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="14" t="n"/>
+      <c r="A9" s="17" t="n"/>
+      <c r="B9" s="17" t="n"/>
+      <c r="C9" s="17" t="n"/>
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="17" t="n"/>
+      <c r="F9" s="17" t="n"/>
+      <c r="G9" s="17" t="n"/>
+      <c r="H9" s="17" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="14" t="n"/>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="14" t="n"/>
-      <c r="E10" s="14" t="n"/>
-      <c r="F10" s="14" t="n"/>
-      <c r="G10" s="14" t="n"/>
-      <c r="H10" s="14" t="n"/>
+      <c r="A10" s="17" t="n"/>
+      <c r="B10" s="17" t="n"/>
+      <c r="C10" s="17" t="n"/>
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="17" t="n"/>
+      <c r="F10" s="17" t="n"/>
+      <c r="G10" s="17" t="n"/>
+      <c r="H10" s="17" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="14" t="n"/>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="14" t="n"/>
-      <c r="D11" s="14" t="n"/>
-      <c r="E11" s="14" t="n"/>
-      <c r="F11" s="14" t="n"/>
-      <c r="G11" s="14" t="n"/>
-      <c r="H11" s="14" t="n"/>
+      <c r="A11" s="17" t="n"/>
+      <c r="B11" s="17" t="n"/>
+      <c r="C11" s="17" t="n"/>
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="17" t="n"/>
+      <c r="F11" s="17" t="n"/>
+      <c r="G11" s="17" t="n"/>
+      <c r="H11" s="17" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="14" t="n"/>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="14" t="n"/>
-      <c r="E12" s="14" t="n"/>
-      <c r="F12" s="14" t="n"/>
-      <c r="G12" s="14" t="n"/>
-      <c r="H12" s="14" t="n"/>
+      <c r="A12" s="17" t="n"/>
+      <c r="B12" s="17" t="n"/>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n"/>
+      <c r="G12" s="17" t="n"/>
+      <c r="H12" s="17" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="14" t="n"/>
-      <c r="B13" s="14" t="n"/>
-      <c r="C13" s="14" t="n"/>
-      <c r="D13" s="14" t="n"/>
-      <c r="E13" s="14" t="n"/>
-      <c r="F13" s="14" t="n"/>
-      <c r="G13" s="14" t="n"/>
-      <c r="H13" s="14" t="n"/>
+      <c r="A13" s="17" t="n"/>
+      <c r="B13" s="17" t="n"/>
+      <c r="C13" s="17" t="n"/>
+      <c r="D13" s="17" t="n"/>
+      <c r="E13" s="17" t="n"/>
+      <c r="F13" s="17" t="n"/>
+      <c r="G13" s="17" t="n"/>
+      <c r="H13" s="17" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="14" t="n"/>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="14" t="n"/>
-      <c r="E14" s="14" t="n"/>
-      <c r="F14" s="14" t="n"/>
-      <c r="G14" s="14" t="n"/>
-      <c r="H14" s="14" t="n"/>
+      <c r="A14" s="17" t="n"/>
+      <c r="B14" s="17" t="n"/>
+      <c r="C14" s="17" t="n"/>
+      <c r="D14" s="17" t="n"/>
+      <c r="E14" s="17" t="n"/>
+      <c r="F14" s="17" t="n"/>
+      <c r="G14" s="17" t="n"/>
+      <c r="H14" s="17" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="14" t="n"/>
-      <c r="B15" s="14" t="n"/>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="14" t="n"/>
-      <c r="E15" s="14" t="n"/>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="14" t="n"/>
-      <c r="H15" s="14" t="n"/>
+      <c r="A15" s="17" t="n"/>
+      <c r="B15" s="17" t="n"/>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="17" t="n"/>
+      <c r="E15" s="17" t="n"/>
+      <c r="F15" s="17" t="n"/>
+      <c r="G15" s="17" t="n"/>
+      <c r="H15" s="17" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="14" t="n"/>
-      <c r="B16" s="14" t="n"/>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="14" t="n"/>
-      <c r="E16" s="14" t="n"/>
-      <c r="F16" s="14" t="n"/>
-      <c r="G16" s="14" t="n"/>
-      <c r="H16" s="14" t="n"/>
+      <c r="A16" s="17" t="n"/>
+      <c r="B16" s="17" t="n"/>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="17" t="n"/>
+      <c r="H16" s="17" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="14" t="n"/>
-      <c r="B17" s="14" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="14" t="n"/>
-      <c r="E17" s="14" t="n"/>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="14" t="n"/>
-      <c r="H17" s="14" t="n"/>
+      <c r="A17" s="17" t="n"/>
+      <c r="B17" s="17" t="n"/>
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="17" t="n"/>
+      <c r="E17" s="17" t="n"/>
+      <c r="F17" s="17" t="n"/>
+      <c r="G17" s="17" t="n"/>
+      <c r="H17" s="17" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="14" t="n"/>
-      <c r="B18" s="14" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="14" t="n"/>
-      <c r="E18" s="14" t="n"/>
-      <c r="F18" s="14" t="n"/>
-      <c r="G18" s="14" t="n"/>
-      <c r="H18" s="14" t="n"/>
+      <c r="A18" s="17" t="n"/>
+      <c r="B18" s="17" t="n"/>
+      <c r="C18" s="17" t="n"/>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="17" t="n"/>
+      <c r="F18" s="17" t="n"/>
+      <c r="G18" s="17" t="n"/>
+      <c r="H18" s="17" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="14" t="n"/>
-      <c r="B19" s="14" t="n"/>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="14" t="n"/>
-      <c r="E19" s="14" t="n"/>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="14" t="n"/>
-      <c r="H19" s="14" t="n"/>
+      <c r="A19" s="17" t="n"/>
+      <c r="B19" s="17" t="n"/>
+      <c r="C19" s="17" t="n"/>
+      <c r="D19" s="17" t="n"/>
+      <c r="E19" s="17" t="n"/>
+      <c r="F19" s="17" t="n"/>
+      <c r="G19" s="17" t="n"/>
+      <c r="H19" s="17" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="14" t="n"/>
-      <c r="B20" s="14" t="n"/>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="14" t="n"/>
-      <c r="E20" s="14" t="n"/>
-      <c r="F20" s="14" t="n"/>
-      <c r="G20" s="14" t="n"/>
-      <c r="H20" s="14" t="n"/>
+      <c r="A20" s="17" t="n"/>
+      <c r="B20" s="17" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="17" t="n"/>
+      <c r="G20" s="17" t="n"/>
+      <c r="H20" s="17" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="14" t="n"/>
-      <c r="B21" s="14" t="n"/>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="14" t="n"/>
-      <c r="E21" s="14" t="n"/>
-      <c r="F21" s="14" t="n"/>
-      <c r="G21" s="14" t="n"/>
-      <c r="H21" s="14" t="n"/>
+      <c r="A21" s="17" t="n"/>
+      <c r="B21" s="17" t="n"/>
+      <c r="C21" s="17" t="n"/>
+      <c r="D21" s="17" t="n"/>
+      <c r="E21" s="17" t="n"/>
+      <c r="F21" s="17" t="n"/>
+      <c r="G21" s="17" t="n"/>
+      <c r="H21" s="17" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="14" t="n"/>
-      <c r="B22" s="14" t="n"/>
-      <c r="C22" s="14" t="n"/>
-      <c r="D22" s="14" t="n"/>
-      <c r="E22" s="14" t="n"/>
-      <c r="F22" s="14" t="n"/>
-      <c r="G22" s="14" t="n"/>
-      <c r="H22" s="14" t="n"/>
+      <c r="A22" s="17" t="n"/>
+      <c r="B22" s="17" t="n"/>
+      <c r="C22" s="17" t="n"/>
+      <c r="D22" s="17" t="n"/>
+      <c r="E22" s="17" t="n"/>
+      <c r="F22" s="17" t="n"/>
+      <c r="G22" s="17" t="n"/>
+      <c r="H22" s="17" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="14" t="n"/>
-      <c r="B23" s="14" t="n"/>
-      <c r="C23" s="14" t="n"/>
-      <c r="D23" s="14" t="n"/>
-      <c r="E23" s="14" t="n"/>
-      <c r="F23" s="14" t="n"/>
-      <c r="G23" s="14" t="n"/>
-      <c r="H23" s="14" t="n"/>
+      <c r="A23" s="17" t="n"/>
+      <c r="B23" s="17" t="n"/>
+      <c r="C23" s="17" t="n"/>
+      <c r="D23" s="17" t="n"/>
+      <c r="E23" s="17" t="n"/>
+      <c r="F23" s="17" t="n"/>
+      <c r="G23" s="17" t="n"/>
+      <c r="H23" s="17" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="14" t="n"/>
-      <c r="B24" s="14" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="14" t="n"/>
-      <c r="E24" s="14" t="n"/>
-      <c r="F24" s="14" t="n"/>
-      <c r="G24" s="14" t="n"/>
-      <c r="H24" s="14" t="n"/>
+      <c r="A24" s="17" t="n"/>
+      <c r="B24" s="17" t="n"/>
+      <c r="C24" s="17" t="n"/>
+      <c r="D24" s="17" t="n"/>
+      <c r="E24" s="17" t="n"/>
+      <c r="F24" s="17" t="n"/>
+      <c r="G24" s="17" t="n"/>
+      <c r="H24" s="17" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="14" t="n"/>
-      <c r="B25" s="14" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="14" t="n"/>
-      <c r="E25" s="14" t="n"/>
-      <c r="F25" s="14" t="n"/>
-      <c r="G25" s="14" t="n"/>
-      <c r="H25" s="14" t="n"/>
+      <c r="A25" s="17" t="n"/>
+      <c r="B25" s="17" t="n"/>
+      <c r="C25" s="17" t="n"/>
+      <c r="D25" s="17" t="n"/>
+      <c r="E25" s="17" t="n"/>
+      <c r="F25" s="17" t="n"/>
+      <c r="G25" s="17" t="n"/>
+      <c r="H25" s="17" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="14" t="n"/>
-      <c r="B26" s="14" t="n"/>
-      <c r="C26" s="14" t="n"/>
-      <c r="D26" s="14" t="n"/>
-      <c r="E26" s="14" t="n"/>
-      <c r="F26" s="14" t="n"/>
-      <c r="G26" s="14" t="n"/>
-      <c r="H26" s="14" t="n"/>
+      <c r="A26" s="17" t="n"/>
+      <c r="B26" s="17" t="n"/>
+      <c r="C26" s="17" t="n"/>
+      <c r="D26" s="17" t="n"/>
+      <c r="E26" s="17" t="n"/>
+      <c r="F26" s="17" t="n"/>
+      <c r="G26" s="17" t="n"/>
+      <c r="H26" s="17" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="14" t="n"/>
-      <c r="B27" s="14" t="n"/>
-      <c r="C27" s="14" t="n"/>
-      <c r="D27" s="14" t="n"/>
-      <c r="E27" s="14" t="n"/>
-      <c r="F27" s="14" t="n"/>
-      <c r="G27" s="14" t="n"/>
-      <c r="H27" s="14" t="n"/>
+      <c r="A27" s="17" t="n"/>
+      <c r="B27" s="17" t="n"/>
+      <c r="C27" s="17" t="n"/>
+      <c r="D27" s="17" t="n"/>
+      <c r="E27" s="17" t="n"/>
+      <c r="F27" s="17" t="n"/>
+      <c r="G27" s="17" t="n"/>
+      <c r="H27" s="17" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="14" t="n"/>
-      <c r="B28" s="14" t="n"/>
-      <c r="C28" s="14" t="n"/>
-      <c r="D28" s="14" t="n"/>
-      <c r="E28" s="14" t="n"/>
-      <c r="F28" s="14" t="n"/>
-      <c r="G28" s="14" t="n"/>
-      <c r="H28" s="14" t="n"/>
+      <c r="A28" s="17" t="n"/>
+      <c r="B28" s="17" t="n"/>
+      <c r="C28" s="17" t="n"/>
+      <c r="D28" s="17" t="n"/>
+      <c r="E28" s="17" t="n"/>
+      <c r="F28" s="17" t="n"/>
+      <c r="G28" s="17" t="n"/>
+      <c r="H28" s="17" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="14" t="n"/>
-      <c r="B29" s="14" t="n"/>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="14" t="n"/>
-      <c r="F29" s="14" t="n"/>
-      <c r="G29" s="14" t="n"/>
-      <c r="H29" s="14" t="n"/>
+      <c r="A29" s="17" t="n"/>
+      <c r="B29" s="17" t="n"/>
+      <c r="C29" s="17" t="n"/>
+      <c r="D29" s="17" t="n"/>
+      <c r="E29" s="17" t="n"/>
+      <c r="F29" s="17" t="n"/>
+      <c r="G29" s="17" t="n"/>
+      <c r="H29" s="17" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="14" t="n"/>
-      <c r="B30" s="14" t="n"/>
-      <c r="C30" s="14" t="n"/>
-      <c r="D30" s="14" t="n"/>
-      <c r="E30" s="14" t="n"/>
-      <c r="F30" s="14" t="n"/>
-      <c r="G30" s="14" t="n"/>
-      <c r="H30" s="14" t="n"/>
+      <c r="A30" s="17" t="n"/>
+      <c r="B30" s="17" t="n"/>
+      <c r="C30" s="17" t="n"/>
+      <c r="D30" s="17" t="n"/>
+      <c r="E30" s="17" t="n"/>
+      <c r="F30" s="17" t="n"/>
+      <c r="G30" s="17" t="n"/>
+      <c r="H30" s="17" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="14" t="n"/>
-      <c r="B31" s="14" t="n"/>
-      <c r="C31" s="14" t="n"/>
-      <c r="D31" s="14" t="n"/>
-      <c r="E31" s="14" t="n"/>
-      <c r="F31" s="14" t="n"/>
-      <c r="G31" s="14" t="n"/>
-      <c r="H31" s="14" t="n"/>
+      <c r="A31" s="17" t="n"/>
+      <c r="B31" s="17" t="n"/>
+      <c r="C31" s="17" t="n"/>
+      <c r="D31" s="17" t="n"/>
+      <c r="E31" s="17" t="n"/>
+      <c r="F31" s="17" t="n"/>
+      <c r="G31" s="17" t="n"/>
+      <c r="H31" s="17" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="14" t="n"/>
-      <c r="B32" s="14" t="n"/>
-      <c r="C32" s="14" t="n"/>
-      <c r="D32" s="14" t="n"/>
-      <c r="E32" s="14" t="n"/>
-      <c r="F32" s="14" t="n"/>
-      <c r="G32" s="14" t="n"/>
-      <c r="H32" s="14" t="n"/>
+      <c r="A32" s="17" t="n"/>
+      <c r="B32" s="17" t="n"/>
+      <c r="C32" s="17" t="n"/>
+      <c r="D32" s="17" t="n"/>
+      <c r="E32" s="17" t="n"/>
+      <c r="F32" s="17" t="n"/>
+      <c r="G32" s="17" t="n"/>
+      <c r="H32" s="17" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="14" t="n"/>
-      <c r="B33" s="14" t="n"/>
-      <c r="C33" s="14" t="n"/>
-      <c r="D33" s="14" t="n"/>
-      <c r="E33" s="14" t="n"/>
-      <c r="F33" s="14" t="n"/>
-      <c r="G33" s="14" t="n"/>
-      <c r="H33" s="14" t="n"/>
+      <c r="A33" s="17" t="n"/>
+      <c r="B33" s="17" t="n"/>
+      <c r="C33" s="17" t="n"/>
+      <c r="D33" s="17" t="n"/>
+      <c r="E33" s="17" t="n"/>
+      <c r="F33" s="17" t="n"/>
+      <c r="G33" s="17" t="n"/>
+      <c r="H33" s="17" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="14" t="n"/>
-      <c r="B34" s="14" t="n"/>
-      <c r="C34" s="14" t="n"/>
-      <c r="D34" s="14" t="n"/>
-      <c r="E34" s="14" t="n"/>
-      <c r="F34" s="14" t="n"/>
-      <c r="G34" s="14" t="n"/>
-      <c r="H34" s="14" t="n"/>
+      <c r="A34" s="17" t="n"/>
+      <c r="B34" s="17" t="n"/>
+      <c r="C34" s="17" t="n"/>
+      <c r="D34" s="17" t="n"/>
+      <c r="E34" s="17" t="n"/>
+      <c r="F34" s="17" t="n"/>
+      <c r="G34" s="17" t="n"/>
+      <c r="H34" s="17" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="14" t="n"/>
-      <c r="B35" s="14" t="n"/>
-      <c r="C35" s="14" t="n"/>
-      <c r="D35" s="14" t="n"/>
-      <c r="E35" s="14" t="n"/>
-      <c r="F35" s="14" t="n"/>
-      <c r="G35" s="14" t="n"/>
-      <c r="H35" s="14" t="n"/>
+      <c r="A35" s="17" t="n"/>
+      <c r="B35" s="17" t="n"/>
+      <c r="C35" s="17" t="n"/>
+      <c r="D35" s="17" t="n"/>
+      <c r="E35" s="17" t="n"/>
+      <c r="F35" s="17" t="n"/>
+      <c r="G35" s="17" t="n"/>
+      <c r="H35" s="17" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="14" t="n"/>
-      <c r="B36" s="14" t="n"/>
-      <c r="C36" s="14" t="n"/>
-      <c r="D36" s="14" t="n"/>
-      <c r="E36" s="14" t="n"/>
-      <c r="F36" s="14" t="n"/>
-      <c r="G36" s="14" t="n"/>
-      <c r="H36" s="14" t="n"/>
+      <c r="A36" s="17" t="n"/>
+      <c r="B36" s="17" t="n"/>
+      <c r="C36" s="17" t="n"/>
+      <c r="D36" s="17" t="n"/>
+      <c r="E36" s="17" t="n"/>
+      <c r="F36" s="17" t="n"/>
+      <c r="G36" s="17" t="n"/>
+      <c r="H36" s="17" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="14" t="n"/>
-      <c r="B37" s="14" t="n"/>
-      <c r="C37" s="14" t="n"/>
-      <c r="D37" s="14" t="n"/>
-      <c r="E37" s="14" t="n"/>
-      <c r="F37" s="14" t="n"/>
-      <c r="G37" s="14" t="n"/>
-      <c r="H37" s="14" t="n"/>
+      <c r="A37" s="17" t="n"/>
+      <c r="B37" s="17" t="n"/>
+      <c r="C37" s="17" t="n"/>
+      <c r="D37" s="17" t="n"/>
+      <c r="E37" s="17" t="n"/>
+      <c r="F37" s="17" t="n"/>
+      <c r="G37" s="17" t="n"/>
+      <c r="H37" s="17" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="14" t="n"/>
-      <c r="B38" s="14" t="n"/>
-      <c r="C38" s="14" t="n"/>
-      <c r="D38" s="14" t="n"/>
-      <c r="E38" s="14" t="n"/>
-      <c r="F38" s="14" t="n"/>
-      <c r="G38" s="14" t="n"/>
-      <c r="H38" s="14" t="n"/>
+      <c r="A38" s="17" t="n"/>
+      <c r="B38" s="17" t="n"/>
+      <c r="C38" s="17" t="n"/>
+      <c r="D38" s="17" t="n"/>
+      <c r="E38" s="17" t="n"/>
+      <c r="F38" s="17" t="n"/>
+      <c r="G38" s="17" t="n"/>
+      <c r="H38" s="17" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="14" t="n"/>
-      <c r="B39" s="14" t="n"/>
-      <c r="C39" s="14" t="n"/>
-      <c r="D39" s="14" t="n"/>
-      <c r="E39" s="14" t="n"/>
-      <c r="F39" s="14" t="n"/>
-      <c r="G39" s="14" t="n"/>
-      <c r="H39" s="14" t="n"/>
+      <c r="A39" s="17" t="n"/>
+      <c r="B39" s="17" t="n"/>
+      <c r="C39" s="17" t="n"/>
+      <c r="D39" s="17" t="n"/>
+      <c r="E39" s="17" t="n"/>
+      <c r="F39" s="17" t="n"/>
+      <c r="G39" s="17" t="n"/>
+      <c r="H39" s="17" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="14" t="n"/>
-      <c r="B40" s="14" t="n"/>
-      <c r="C40" s="14" t="n"/>
-      <c r="D40" s="14" t="n"/>
-      <c r="E40" s="14" t="n"/>
-      <c r="F40" s="14" t="n"/>
-      <c r="G40" s="14" t="n"/>
-      <c r="H40" s="14" t="n"/>
+      <c r="A40" s="17" t="n"/>
+      <c r="B40" s="17" t="n"/>
+      <c r="C40" s="17" t="n"/>
+      <c r="D40" s="17" t="n"/>
+      <c r="E40" s="17" t="n"/>
+      <c r="F40" s="17" t="n"/>
+      <c r="G40" s="17" t="n"/>
+      <c r="H40" s="17" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
     </row>
@@ -1115,476 +1124,476 @@
       <c r="J2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>14.07.2026</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="19" t="inlineStr">
         <is>
           <t>4039-95</t>
         </is>
       </c>
-      <c r="C3" s="16" t="inlineStr">
+      <c r="C3" s="19" t="inlineStr">
         <is>
           <t>1.0026-2X2500X1250</t>
         </is>
       </c>
-      <c r="D3" s="16" t="n">
+      <c r="D3" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="16" t="inlineStr">
+      <c r="E3" s="19" t="inlineStr">
         <is>
           <t>00:04:03</t>
         </is>
       </c>
-      <c r="F3" s="16" t="n"/>
-      <c r="G3" s="16" t="n"/>
-      <c r="H3" s="16" t="n"/>
+      <c r="F3" s="19" t="n"/>
+      <c r="G3" s="19" t="n"/>
+      <c r="H3" s="19" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="n"/>
-      <c r="B4" s="16" t="n"/>
-      <c r="C4" s="16" t="n"/>
-      <c r="D4" s="16" t="n"/>
-      <c r="E4" s="16" t="n"/>
-      <c r="F4" s="16" t="n"/>
-      <c r="G4" s="16" t="n"/>
-      <c r="H4" s="16" t="n"/>
+      <c r="A4" s="19" t="n"/>
+      <c r="B4" s="19" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+      <c r="E4" s="19" t="n"/>
+      <c r="F4" s="19" t="n"/>
+      <c r="G4" s="19" t="n"/>
+      <c r="H4" s="19" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="n"/>
-      <c r="B5" s="16" t="n"/>
-      <c r="C5" s="16" t="n"/>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="16" t="n"/>
-      <c r="G5" s="16" t="n"/>
-      <c r="H5" s="16" t="n"/>
+      <c r="A5" s="19" t="n"/>
+      <c r="B5" s="19" t="n"/>
+      <c r="C5" s="19" t="n"/>
+      <c r="D5" s="19" t="n"/>
+      <c r="E5" s="19" t="n"/>
+      <c r="F5" s="19" t="n"/>
+      <c r="G5" s="19" t="n"/>
+      <c r="H5" s="19" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="n"/>
-      <c r="B6" s="16" t="n"/>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="16" t="n"/>
-      <c r="E6" s="16" t="n"/>
-      <c r="F6" s="16" t="n"/>
-      <c r="G6" s="16" t="n"/>
-      <c r="H6" s="16" t="n"/>
+      <c r="A6" s="19" t="n"/>
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="19" t="n"/>
+      <c r="D6" s="19" t="n"/>
+      <c r="E6" s="19" t="n"/>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6" s="19" t="n"/>
+      <c r="H6" s="19" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="n"/>
-      <c r="B7" s="16" t="n"/>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="16" t="n"/>
-      <c r="E7" s="16" t="n"/>
-      <c r="F7" s="16" t="n"/>
-      <c r="G7" s="16" t="n"/>
-      <c r="H7" s="16" t="n"/>
+      <c r="A7" s="19" t="n"/>
+      <c r="B7" s="19" t="n"/>
+      <c r="C7" s="19" t="n"/>
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="19" t="n"/>
+      <c r="F7" s="19" t="n"/>
+      <c r="G7" s="19" t="n"/>
+      <c r="H7" s="19" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="n"/>
-      <c r="B8" s="16" t="n"/>
-      <c r="C8" s="16" t="n"/>
-      <c r="D8" s="16" t="n"/>
-      <c r="E8" s="16" t="n"/>
-      <c r="F8" s="16" t="n"/>
-      <c r="G8" s="16" t="n"/>
-      <c r="H8" s="16" t="n"/>
+      <c r="A8" s="19" t="n"/>
+      <c r="B8" s="19" t="n"/>
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="19" t="n"/>
+      <c r="H8" s="19" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="n"/>
-      <c r="B9" s="16" t="n"/>
-      <c r="C9" s="16" t="n"/>
-      <c r="D9" s="16" t="n"/>
-      <c r="E9" s="16" t="n"/>
-      <c r="F9" s="16" t="n"/>
-      <c r="G9" s="16" t="n"/>
-      <c r="H9" s="16" t="n"/>
+      <c r="A9" s="19" t="n"/>
+      <c r="B9" s="19" t="n"/>
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="19" t="n"/>
+      <c r="E9" s="19" t="n"/>
+      <c r="F9" s="19" t="n"/>
+      <c r="G9" s="19" t="n"/>
+      <c r="H9" s="19" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="n"/>
-      <c r="B10" s="16" t="n"/>
-      <c r="C10" s="16" t="n"/>
-      <c r="D10" s="16" t="n"/>
-      <c r="E10" s="16" t="n"/>
-      <c r="F10" s="16" t="n"/>
-      <c r="G10" s="16" t="n"/>
-      <c r="H10" s="16" t="n"/>
+      <c r="A10" s="19" t="n"/>
+      <c r="B10" s="19" t="n"/>
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="19" t="n"/>
+      <c r="H10" s="19" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="n"/>
-      <c r="B11" s="16" t="n"/>
-      <c r="C11" s="16" t="n"/>
-      <c r="D11" s="16" t="n"/>
-      <c r="E11" s="16" t="n"/>
-      <c r="F11" s="16" t="n"/>
-      <c r="G11" s="16" t="n"/>
-      <c r="H11" s="16" t="n"/>
+      <c r="A11" s="19" t="n"/>
+      <c r="B11" s="19" t="n"/>
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="19" t="n"/>
+      <c r="E11" s="19" t="n"/>
+      <c r="F11" s="19" t="n"/>
+      <c r="G11" s="19" t="n"/>
+      <c r="H11" s="19" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="n"/>
-      <c r="B12" s="16" t="n"/>
-      <c r="C12" s="16" t="n"/>
-      <c r="D12" s="16" t="n"/>
-      <c r="E12" s="16" t="n"/>
-      <c r="F12" s="16" t="n"/>
-      <c r="G12" s="16" t="n"/>
-      <c r="H12" s="16" t="n"/>
+      <c r="A12" s="19" t="n"/>
+      <c r="B12" s="19" t="n"/>
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="19" t="n"/>
+      <c r="E12" s="19" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="19" t="n"/>
+      <c r="H12" s="19" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="n"/>
-      <c r="B13" s="16" t="n"/>
-      <c r="C13" s="16" t="n"/>
-      <c r="D13" s="16" t="n"/>
-      <c r="E13" s="16" t="n"/>
-      <c r="F13" s="16" t="n"/>
-      <c r="G13" s="16" t="n"/>
-      <c r="H13" s="16" t="n"/>
+      <c r="A13" s="19" t="n"/>
+      <c r="B13" s="19" t="n"/>
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="19" t="n"/>
+      <c r="E13" s="19" t="n"/>
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="19" t="n"/>
+      <c r="H13" s="19" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="n"/>
-      <c r="B14" s="16" t="n"/>
-      <c r="C14" s="16" t="n"/>
-      <c r="D14" s="16" t="n"/>
-      <c r="E14" s="16" t="n"/>
-      <c r="F14" s="16" t="n"/>
-      <c r="G14" s="16" t="n"/>
-      <c r="H14" s="16" t="n"/>
+      <c r="A14" s="19" t="n"/>
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+      <c r="E14" s="19" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="19" t="n"/>
+      <c r="H14" s="19" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="n"/>
-      <c r="B15" s="16" t="n"/>
-      <c r="C15" s="16" t="n"/>
-      <c r="D15" s="16" t="n"/>
-      <c r="E15" s="16" t="n"/>
-      <c r="F15" s="16" t="n"/>
-      <c r="G15" s="16" t="n"/>
-      <c r="H15" s="16" t="n"/>
+      <c r="A15" s="19" t="n"/>
+      <c r="B15" s="19" t="n"/>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="19" t="n"/>
+      <c r="E15" s="19" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="n"/>
+      <c r="H15" s="19" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="n"/>
-      <c r="B16" s="16" t="n"/>
-      <c r="C16" s="16" t="n"/>
-      <c r="D16" s="16" t="n"/>
-      <c r="E16" s="16" t="n"/>
-      <c r="F16" s="16" t="n"/>
-      <c r="G16" s="16" t="n"/>
-      <c r="H16" s="16" t="n"/>
+      <c r="A16" s="19" t="n"/>
+      <c r="B16" s="19" t="n"/>
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="19" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="n"/>
+      <c r="H16" s="19" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="n"/>
-      <c r="B17" s="16" t="n"/>
-      <c r="C17" s="16" t="n"/>
-      <c r="D17" s="16" t="n"/>
-      <c r="E17" s="16" t="n"/>
-      <c r="F17" s="16" t="n"/>
-      <c r="G17" s="16" t="n"/>
-      <c r="H17" s="16" t="n"/>
+      <c r="A17" s="19" t="n"/>
+      <c r="B17" s="19" t="n"/>
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="19" t="n"/>
+      <c r="E17" s="19" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="19" t="n"/>
+      <c r="H17" s="19" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="n"/>
-      <c r="B18" s="16" t="n"/>
-      <c r="C18" s="16" t="n"/>
-      <c r="D18" s="16" t="n"/>
-      <c r="E18" s="16" t="n"/>
-      <c r="F18" s="16" t="n"/>
-      <c r="G18" s="16" t="n"/>
-      <c r="H18" s="16" t="n"/>
+      <c r="A18" s="19" t="n"/>
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+      <c r="E18" s="19" t="n"/>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="19" t="n"/>
+      <c r="H18" s="19" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="n"/>
-      <c r="B19" s="16" t="n"/>
-      <c r="C19" s="16" t="n"/>
-      <c r="D19" s="16" t="n"/>
-      <c r="E19" s="16" t="n"/>
-      <c r="F19" s="16" t="n"/>
-      <c r="G19" s="16" t="n"/>
-      <c r="H19" s="16" t="n"/>
+      <c r="A19" s="19" t="n"/>
+      <c r="B19" s="19" t="n"/>
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="19" t="n"/>
+      <c r="E19" s="19" t="n"/>
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="19" t="n"/>
+      <c r="H19" s="19" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="n"/>
-      <c r="B20" s="16" t="n"/>
-      <c r="C20" s="16" t="n"/>
-      <c r="D20" s="16" t="n"/>
-      <c r="E20" s="16" t="n"/>
-      <c r="F20" s="16" t="n"/>
-      <c r="G20" s="16" t="n"/>
-      <c r="H20" s="16" t="n"/>
+      <c r="A20" s="19" t="n"/>
+      <c r="B20" s="19" t="n"/>
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="19" t="n"/>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="19" t="n"/>
+      <c r="H20" s="19" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="n"/>
-      <c r="B21" s="16" t="n"/>
-      <c r="C21" s="16" t="n"/>
-      <c r="D21" s="16" t="n"/>
-      <c r="E21" s="16" t="n"/>
-      <c r="F21" s="16" t="n"/>
-      <c r="G21" s="16" t="n"/>
-      <c r="H21" s="16" t="n"/>
+      <c r="A21" s="19" t="n"/>
+      <c r="B21" s="19" t="n"/>
+      <c r="C21" s="19" t="n"/>
+      <c r="D21" s="19" t="n"/>
+      <c r="E21" s="19" t="n"/>
+      <c r="F21" s="19" t="n"/>
+      <c r="G21" s="19" t="n"/>
+      <c r="H21" s="19" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="n"/>
-      <c r="B22" s="16" t="n"/>
-      <c r="C22" s="16" t="n"/>
-      <c r="D22" s="16" t="n"/>
-      <c r="E22" s="16" t="n"/>
-      <c r="F22" s="16" t="n"/>
-      <c r="G22" s="16" t="n"/>
-      <c r="H22" s="16" t="n"/>
+      <c r="A22" s="19" t="n"/>
+      <c r="B22" s="19" t="n"/>
+      <c r="C22" s="19" t="n"/>
+      <c r="D22" s="19" t="n"/>
+      <c r="E22" s="19" t="n"/>
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="19" t="n"/>
+      <c r="H22" s="19" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="n"/>
-      <c r="B23" s="16" t="n"/>
-      <c r="C23" s="16" t="n"/>
-      <c r="D23" s="16" t="n"/>
-      <c r="E23" s="16" t="n"/>
-      <c r="F23" s="16" t="n"/>
-      <c r="G23" s="16" t="n"/>
-      <c r="H23" s="16" t="n"/>
+      <c r="A23" s="19" t="n"/>
+      <c r="B23" s="19" t="n"/>
+      <c r="C23" s="19" t="n"/>
+      <c r="D23" s="19" t="n"/>
+      <c r="E23" s="19" t="n"/>
+      <c r="F23" s="19" t="n"/>
+      <c r="G23" s="19" t="n"/>
+      <c r="H23" s="19" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="n"/>
-      <c r="B24" s="16" t="n"/>
-      <c r="C24" s="16" t="n"/>
-      <c r="D24" s="16" t="n"/>
-      <c r="E24" s="16" t="n"/>
-      <c r="F24" s="16" t="n"/>
-      <c r="G24" s="16" t="n"/>
-      <c r="H24" s="16" t="n"/>
+      <c r="A24" s="19" t="n"/>
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+      <c r="E24" s="19" t="n"/>
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="19" t="n"/>
+      <c r="H24" s="19" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="n"/>
-      <c r="B25" s="16" t="n"/>
-      <c r="C25" s="16" t="n"/>
-      <c r="D25" s="16" t="n"/>
-      <c r="E25" s="16" t="n"/>
-      <c r="F25" s="16" t="n"/>
-      <c r="G25" s="16" t="n"/>
-      <c r="H25" s="16" t="n"/>
+      <c r="A25" s="19" t="n"/>
+      <c r="B25" s="19" t="n"/>
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
+      <c r="F25" s="19" t="n"/>
+      <c r="G25" s="19" t="n"/>
+      <c r="H25" s="19" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="n"/>
-      <c r="B26" s="16" t="n"/>
-      <c r="C26" s="16" t="n"/>
-      <c r="D26" s="16" t="n"/>
-      <c r="E26" s="16" t="n"/>
-      <c r="F26" s="16" t="n"/>
-      <c r="G26" s="16" t="n"/>
-      <c r="H26" s="16" t="n"/>
+      <c r="A26" s="19" t="n"/>
+      <c r="B26" s="19" t="n"/>
+      <c r="C26" s="19" t="n"/>
+      <c r="D26" s="19" t="n"/>
+      <c r="E26" s="19" t="n"/>
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="19" t="n"/>
+      <c r="H26" s="19" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="n"/>
-      <c r="B27" s="16" t="n"/>
-      <c r="C27" s="16" t="n"/>
-      <c r="D27" s="16" t="n"/>
-      <c r="E27" s="16" t="n"/>
-      <c r="F27" s="16" t="n"/>
-      <c r="G27" s="16" t="n"/>
-      <c r="H27" s="16" t="n"/>
+      <c r="A27" s="19" t="n"/>
+      <c r="B27" s="19" t="n"/>
+      <c r="C27" s="19" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="19" t="n"/>
+      <c r="F27" s="19" t="n"/>
+      <c r="G27" s="19" t="n"/>
+      <c r="H27" s="19" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="n"/>
-      <c r="B28" s="16" t="n"/>
-      <c r="C28" s="16" t="n"/>
-      <c r="D28" s="16" t="n"/>
-      <c r="E28" s="16" t="n"/>
-      <c r="F28" s="16" t="n"/>
-      <c r="G28" s="16" t="n"/>
-      <c r="H28" s="16" t="n"/>
+      <c r="A28" s="19" t="n"/>
+      <c r="B28" s="19" t="n"/>
+      <c r="C28" s="19" t="n"/>
+      <c r="D28" s="19" t="n"/>
+      <c r="E28" s="19" t="n"/>
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="19" t="n"/>
+      <c r="H28" s="19" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="n"/>
-      <c r="B29" s="16" t="n"/>
-      <c r="C29" s="16" t="n"/>
-      <c r="D29" s="16" t="n"/>
-      <c r="E29" s="16" t="n"/>
-      <c r="F29" s="16" t="n"/>
-      <c r="G29" s="16" t="n"/>
-      <c r="H29" s="16" t="n"/>
+      <c r="A29" s="19" t="n"/>
+      <c r="B29" s="19" t="n"/>
+      <c r="C29" s="19" t="n"/>
+      <c r="D29" s="19" t="n"/>
+      <c r="E29" s="19" t="n"/>
+      <c r="F29" s="19" t="n"/>
+      <c r="G29" s="19" t="n"/>
+      <c r="H29" s="19" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="n"/>
-      <c r="B30" s="16" t="n"/>
-      <c r="C30" s="16" t="n"/>
-      <c r="D30" s="16" t="n"/>
-      <c r="E30" s="16" t="n"/>
-      <c r="F30" s="16" t="n"/>
-      <c r="G30" s="16" t="n"/>
-      <c r="H30" s="16" t="n"/>
+      <c r="A30" s="19" t="n"/>
+      <c r="B30" s="19" t="n"/>
+      <c r="C30" s="19" t="n"/>
+      <c r="D30" s="19" t="n"/>
+      <c r="E30" s="19" t="n"/>
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="19" t="n"/>
+      <c r="H30" s="19" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="16" t="n"/>
-      <c r="B31" s="16" t="n"/>
-      <c r="C31" s="16" t="n"/>
-      <c r="D31" s="16" t="n"/>
-      <c r="E31" s="16" t="n"/>
-      <c r="F31" s="16" t="n"/>
-      <c r="G31" s="16" t="n"/>
-      <c r="H31" s="16" t="n"/>
+      <c r="A31" s="19" t="n"/>
+      <c r="B31" s="19" t="n"/>
+      <c r="C31" s="19" t="n"/>
+      <c r="D31" s="19" t="n"/>
+      <c r="E31" s="19" t="n"/>
+      <c r="F31" s="19" t="n"/>
+      <c r="G31" s="19" t="n"/>
+      <c r="H31" s="19" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="16" t="n"/>
-      <c r="B32" s="16" t="n"/>
-      <c r="C32" s="16" t="n"/>
-      <c r="D32" s="16" t="n"/>
-      <c r="E32" s="16" t="n"/>
-      <c r="F32" s="16" t="n"/>
-      <c r="G32" s="16" t="n"/>
-      <c r="H32" s="16" t="n"/>
+      <c r="A32" s="19" t="n"/>
+      <c r="B32" s="19" t="n"/>
+      <c r="C32" s="19" t="n"/>
+      <c r="D32" s="19" t="n"/>
+      <c r="E32" s="19" t="n"/>
+      <c r="F32" s="19" t="n"/>
+      <c r="G32" s="19" t="n"/>
+      <c r="H32" s="19" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="n"/>
-      <c r="B33" s="16" t="n"/>
-      <c r="C33" s="16" t="n"/>
-      <c r="D33" s="16" t="n"/>
-      <c r="E33" s="16" t="n"/>
-      <c r="F33" s="16" t="n"/>
-      <c r="G33" s="16" t="n"/>
-      <c r="H33" s="16" t="n"/>
+      <c r="A33" s="19" t="n"/>
+      <c r="B33" s="19" t="n"/>
+      <c r="C33" s="19" t="n"/>
+      <c r="D33" s="19" t="n"/>
+      <c r="E33" s="19" t="n"/>
+      <c r="F33" s="19" t="n"/>
+      <c r="G33" s="19" t="n"/>
+      <c r="H33" s="19" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="n"/>
-      <c r="B34" s="16" t="n"/>
-      <c r="C34" s="16" t="n"/>
-      <c r="D34" s="16" t="n"/>
-      <c r="E34" s="16" t="n"/>
-      <c r="F34" s="16" t="n"/>
-      <c r="G34" s="16" t="n"/>
-      <c r="H34" s="16" t="n"/>
+      <c r="A34" s="19" t="n"/>
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="19" t="n"/>
+      <c r="D34" s="19" t="n"/>
+      <c r="E34" s="19" t="n"/>
+      <c r="F34" s="19" t="n"/>
+      <c r="G34" s="19" t="n"/>
+      <c r="H34" s="19" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="16" t="n"/>
-      <c r="B35" s="16" t="n"/>
-      <c r="C35" s="16" t="n"/>
-      <c r="D35" s="16" t="n"/>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="16" t="n"/>
-      <c r="G35" s="16" t="n"/>
-      <c r="H35" s="16" t="n"/>
+      <c r="A35" s="19" t="n"/>
+      <c r="B35" s="19" t="n"/>
+      <c r="C35" s="19" t="n"/>
+      <c r="D35" s="19" t="n"/>
+      <c r="E35" s="19" t="n"/>
+      <c r="F35" s="19" t="n"/>
+      <c r="G35" s="19" t="n"/>
+      <c r="H35" s="19" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="16" t="n"/>
-      <c r="B36" s="16" t="n"/>
-      <c r="C36" s="16" t="n"/>
-      <c r="D36" s="16" t="n"/>
-      <c r="E36" s="16" t="n"/>
-      <c r="F36" s="16" t="n"/>
-      <c r="G36" s="16" t="n"/>
-      <c r="H36" s="16" t="n"/>
+      <c r="A36" s="19" t="n"/>
+      <c r="B36" s="19" t="n"/>
+      <c r="C36" s="19" t="n"/>
+      <c r="D36" s="19" t="n"/>
+      <c r="E36" s="19" t="n"/>
+      <c r="F36" s="19" t="n"/>
+      <c r="G36" s="19" t="n"/>
+      <c r="H36" s="19" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="16" t="n"/>
-      <c r="B37" s="16" t="n"/>
-      <c r="C37" s="16" t="n"/>
-      <c r="D37" s="16" t="n"/>
-      <c r="E37" s="16" t="n"/>
-      <c r="F37" s="16" t="n"/>
-      <c r="G37" s="16" t="n"/>
-      <c r="H37" s="16" t="n"/>
+      <c r="A37" s="19" t="n"/>
+      <c r="B37" s="19" t="n"/>
+      <c r="C37" s="19" t="n"/>
+      <c r="D37" s="19" t="n"/>
+      <c r="E37" s="19" t="n"/>
+      <c r="F37" s="19" t="n"/>
+      <c r="G37" s="19" t="n"/>
+      <c r="H37" s="19" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="16" t="n"/>
-      <c r="B38" s="16" t="n"/>
-      <c r="C38" s="16" t="n"/>
-      <c r="D38" s="16" t="n"/>
-      <c r="E38" s="16" t="n"/>
-      <c r="F38" s="16" t="n"/>
-      <c r="G38" s="16" t="n"/>
-      <c r="H38" s="16" t="n"/>
+      <c r="A38" s="19" t="n"/>
+      <c r="B38" s="19" t="n"/>
+      <c r="C38" s="19" t="n"/>
+      <c r="D38" s="19" t="n"/>
+      <c r="E38" s="19" t="n"/>
+      <c r="F38" s="19" t="n"/>
+      <c r="G38" s="19" t="n"/>
+      <c r="H38" s="19" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="16" t="n"/>
-      <c r="B39" s="16" t="n"/>
-      <c r="C39" s="16" t="n"/>
-      <c r="D39" s="16" t="n"/>
-      <c r="E39" s="16" t="n"/>
-      <c r="F39" s="16" t="n"/>
-      <c r="G39" s="16" t="n"/>
-      <c r="H39" s="16" t="n"/>
+      <c r="A39" s="19" t="n"/>
+      <c r="B39" s="19" t="n"/>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="19" t="n"/>
+      <c r="F39" s="19" t="n"/>
+      <c r="G39" s="19" t="n"/>
+      <c r="H39" s="19" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="16" t="n"/>
-      <c r="B40" s="16" t="n"/>
-      <c r="C40" s="16" t="n"/>
-      <c r="D40" s="16" t="n"/>
-      <c r="E40" s="16" t="n"/>
-      <c r="F40" s="16" t="n"/>
-      <c r="G40" s="16" t="n"/>
-      <c r="H40" s="16" t="n"/>
+      <c r="A40" s="19" t="n"/>
+      <c r="B40" s="19" t="n"/>
+      <c r="C40" s="19" t="n"/>
+      <c r="D40" s="19" t="n"/>
+      <c r="E40" s="19" t="n"/>
+      <c r="F40" s="19" t="n"/>
+      <c r="G40" s="19" t="n"/>
+      <c r="H40" s="19" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
     </row>

</xml_diff>

<commit_message>
feat: left over parts storage
</commit_message>
<xml_diff>
--- a/users/uzuran/burn_table.xlsx
+++ b/users/uzuran/burn_table.xlsx
@@ -67,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="613">
+  <cellXfs count="657">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1760,6 +1760,138 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2338,532 +2470,532 @@
       <c r="J2" s="3" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="611" t="inlineStr">
+      <c r="A3" s="655" t="inlineStr">
         <is>
           <t>14.07.2026</t>
         </is>
       </c>
-      <c r="B3" s="611" t="inlineStr">
+      <c r="B3" s="655" t="inlineStr">
         <is>
           <t>4039-95</t>
         </is>
       </c>
-      <c r="C3" s="611" t="inlineStr">
+      <c r="C3" s="655" t="inlineStr">
         <is>
           <t>1.0026-2X2500X1250</t>
         </is>
       </c>
-      <c r="D3" s="611" t="n">
+      <c r="D3" s="655" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="611" t="inlineStr">
+      <c r="E3" s="655" t="inlineStr">
         <is>
           <t>00:04:03</t>
         </is>
       </c>
-      <c r="F3" s="611" t="n"/>
-      <c r="G3" s="611" t="n"/>
-      <c r="H3" s="611" t="n"/>
+      <c r="F3" s="655" t="n"/>
+      <c r="G3" s="655" t="n"/>
+      <c r="H3" s="655" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="611" t="n"/>
-      <c r="B4" s="611" t="inlineStr">
+      <c r="A4" s="655" t="n"/>
+      <c r="B4" s="655" t="inlineStr">
         <is>
           <t>4039-96</t>
         </is>
       </c>
-      <c r="C4" s="611" t="inlineStr">
+      <c r="C4" s="655" t="inlineStr">
         <is>
           <t>3.3535-2X2500X1250</t>
         </is>
       </c>
-      <c r="D4" s="611" t="n">
+      <c r="D4" s="655" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="611" t="inlineStr">
+      <c r="E4" s="655" t="inlineStr">
         <is>
           <t>00:03:09</t>
         </is>
       </c>
-      <c r="F4" s="611" t="n"/>
-      <c r="G4" s="611" t="n"/>
-      <c r="H4" s="611" t="n"/>
+      <c r="F4" s="655" t="n"/>
+      <c r="G4" s="655" t="n"/>
+      <c r="H4" s="655" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="611" t="n"/>
-      <c r="B5" s="611" t="inlineStr">
+      <c r="A5" s="655" t="n"/>
+      <c r="B5" s="655" t="inlineStr">
         <is>
           <t>4039-97</t>
         </is>
       </c>
-      <c r="C5" s="611" t="inlineStr">
+      <c r="C5" s="655" t="inlineStr">
         <is>
           <t>-----</t>
         </is>
       </c>
-      <c r="D5" s="611" t="n">
+      <c r="D5" s="655" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="611" t="inlineStr">
+      <c r="E5" s="655" t="inlineStr">
         <is>
           <t>00:03:56</t>
         </is>
       </c>
-      <c r="F5" s="611" t="n"/>
-      <c r="G5" s="611" t="n"/>
-      <c r="H5" s="611" t="n"/>
+      <c r="F5" s="655" t="n"/>
+      <c r="G5" s="655" t="n"/>
+      <c r="H5" s="655" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="611" t="n"/>
-      <c r="B6" s="611" t="inlineStr">
+      <c r="A6" s="655" t="n"/>
+      <c r="B6" s="655" t="inlineStr">
         <is>
           <t>4039-98</t>
         </is>
       </c>
-      <c r="C6" s="611" t="inlineStr">
+      <c r="C6" s="655" t="inlineStr">
         <is>
           <t>-----</t>
         </is>
       </c>
-      <c r="D6" s="611" t="n">
+      <c r="D6" s="655" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="611" t="inlineStr">
+      <c r="E6" s="655" t="inlineStr">
         <is>
           <t>00:03:02</t>
         </is>
       </c>
-      <c r="F6" s="611" t="n"/>
-      <c r="G6" s="611" t="n"/>
-      <c r="H6" s="611" t="n"/>
+      <c r="F6" s="655" t="n"/>
+      <c r="G6" s="655" t="n"/>
+      <c r="H6" s="655" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="611" t="n"/>
-      <c r="B7" s="611" t="inlineStr">
+      <c r="A7" s="655" t="n"/>
+      <c r="B7" s="655" t="inlineStr">
         <is>
           <t>4039-99</t>
         </is>
       </c>
-      <c r="C7" s="611" t="inlineStr">
+      <c r="C7" s="655" t="inlineStr">
         <is>
           <t>3.3535-2X3000X1500</t>
         </is>
       </c>
-      <c r="D7" s="611" t="n">
+      <c r="D7" s="655" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="611" t="inlineStr">
+      <c r="E7" s="655" t="inlineStr">
         <is>
           <t>00:02:44</t>
         </is>
       </c>
-      <c r="F7" s="611" t="n"/>
-      <c r="G7" s="611" t="n"/>
-      <c r="H7" s="611" t="n"/>
+      <c r="F7" s="655" t="n"/>
+      <c r="G7" s="655" t="n"/>
+      <c r="H7" s="655" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="611" t="n"/>
-      <c r="B8" s="611" t="n"/>
-      <c r="C8" s="611" t="n"/>
-      <c r="D8" s="611" t="n"/>
-      <c r="E8" s="611" t="n"/>
-      <c r="F8" s="611" t="n"/>
-      <c r="G8" s="611" t="n"/>
-      <c r="H8" s="611" t="n"/>
+      <c r="A8" s="655" t="n"/>
+      <c r="B8" s="655" t="n"/>
+      <c r="C8" s="655" t="n"/>
+      <c r="D8" s="655" t="n"/>
+      <c r="E8" s="655" t="n"/>
+      <c r="F8" s="655" t="n"/>
+      <c r="G8" s="655" t="n"/>
+      <c r="H8" s="655" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="611" t="n"/>
-      <c r="B9" s="611" t="n"/>
-      <c r="C9" s="611" t="n"/>
-      <c r="D9" s="611" t="n"/>
-      <c r="E9" s="611" t="n"/>
-      <c r="F9" s="611" t="n"/>
-      <c r="G9" s="611" t="n"/>
-      <c r="H9" s="611" t="n"/>
+      <c r="A9" s="655" t="n"/>
+      <c r="B9" s="655" t="n"/>
+      <c r="C9" s="655" t="n"/>
+      <c r="D9" s="655" t="n"/>
+      <c r="E9" s="655" t="n"/>
+      <c r="F9" s="655" t="n"/>
+      <c r="G9" s="655" t="n"/>
+      <c r="H9" s="655" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="611" t="n"/>
-      <c r="B10" s="611" t="n"/>
-      <c r="C10" s="611" t="n"/>
-      <c r="D10" s="611" t="n"/>
-      <c r="E10" s="611" t="n"/>
-      <c r="F10" s="611" t="n"/>
-      <c r="G10" s="611" t="n"/>
-      <c r="H10" s="611" t="n"/>
+      <c r="A10" s="655" t="n"/>
+      <c r="B10" s="655" t="n"/>
+      <c r="C10" s="655" t="n"/>
+      <c r="D10" s="655" t="n"/>
+      <c r="E10" s="655" t="n"/>
+      <c r="F10" s="655" t="n"/>
+      <c r="G10" s="655" t="n"/>
+      <c r="H10" s="655" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="611" t="n"/>
-      <c r="B11" s="611" t="n"/>
-      <c r="C11" s="611" t="n"/>
-      <c r="D11" s="611" t="n"/>
-      <c r="E11" s="611" t="n"/>
-      <c r="F11" s="611" t="n"/>
-      <c r="G11" s="611" t="n"/>
-      <c r="H11" s="611" t="n"/>
+      <c r="A11" s="655" t="n"/>
+      <c r="B11" s="655" t="n"/>
+      <c r="C11" s="655" t="n"/>
+      <c r="D11" s="655" t="n"/>
+      <c r="E11" s="655" t="n"/>
+      <c r="F11" s="655" t="n"/>
+      <c r="G11" s="655" t="n"/>
+      <c r="H11" s="655" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="611" t="n"/>
-      <c r="B12" s="611" t="n"/>
-      <c r="C12" s="611" t="n"/>
-      <c r="D12" s="611" t="n"/>
-      <c r="E12" s="611" t="n"/>
-      <c r="F12" s="611" t="n"/>
-      <c r="G12" s="611" t="n"/>
-      <c r="H12" s="611" t="n"/>
+      <c r="A12" s="655" t="n"/>
+      <c r="B12" s="655" t="n"/>
+      <c r="C12" s="655" t="n"/>
+      <c r="D12" s="655" t="n"/>
+      <c r="E12" s="655" t="n"/>
+      <c r="F12" s="655" t="n"/>
+      <c r="G12" s="655" t="n"/>
+      <c r="H12" s="655" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="611" t="n"/>
-      <c r="B13" s="611" t="n"/>
-      <c r="C13" s="611" t="n"/>
-      <c r="D13" s="611" t="n"/>
-      <c r="E13" s="611" t="n"/>
-      <c r="F13" s="611" t="n"/>
-      <c r="G13" s="611" t="n"/>
-      <c r="H13" s="611" t="n"/>
+      <c r="A13" s="655" t="n"/>
+      <c r="B13" s="655" t="n"/>
+      <c r="C13" s="655" t="n"/>
+      <c r="D13" s="655" t="n"/>
+      <c r="E13" s="655" t="n"/>
+      <c r="F13" s="655" t="n"/>
+      <c r="G13" s="655" t="n"/>
+      <c r="H13" s="655" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="611" t="n"/>
-      <c r="B14" s="611" t="n"/>
-      <c r="C14" s="611" t="n"/>
-      <c r="D14" s="611" t="n"/>
-      <c r="E14" s="611" t="n"/>
-      <c r="F14" s="611" t="n"/>
-      <c r="G14" s="611" t="n"/>
-      <c r="H14" s="611" t="n"/>
+      <c r="A14" s="655" t="n"/>
+      <c r="B14" s="655" t="n"/>
+      <c r="C14" s="655" t="n"/>
+      <c r="D14" s="655" t="n"/>
+      <c r="E14" s="655" t="n"/>
+      <c r="F14" s="655" t="n"/>
+      <c r="G14" s="655" t="n"/>
+      <c r="H14" s="655" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="611" t="n"/>
-      <c r="B15" s="611" t="n"/>
-      <c r="C15" s="611" t="n"/>
-      <c r="D15" s="611" t="n"/>
-      <c r="E15" s="611" t="n"/>
-      <c r="F15" s="611" t="n"/>
-      <c r="G15" s="611" t="n"/>
-      <c r="H15" s="611" t="n"/>
+      <c r="A15" s="655" t="n"/>
+      <c r="B15" s="655" t="n"/>
+      <c r="C15" s="655" t="n"/>
+      <c r="D15" s="655" t="n"/>
+      <c r="E15" s="655" t="n"/>
+      <c r="F15" s="655" t="n"/>
+      <c r="G15" s="655" t="n"/>
+      <c r="H15" s="655" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="611" t="n"/>
-      <c r="B16" s="611" t="n"/>
-      <c r="C16" s="611" t="n"/>
-      <c r="D16" s="611" t="n"/>
-      <c r="E16" s="611" t="n"/>
-      <c r="F16" s="611" t="n"/>
-      <c r="G16" s="611" t="n"/>
-      <c r="H16" s="611" t="n"/>
+      <c r="A16" s="655" t="n"/>
+      <c r="B16" s="655" t="n"/>
+      <c r="C16" s="655" t="n"/>
+      <c r="D16" s="655" t="n"/>
+      <c r="E16" s="655" t="n"/>
+      <c r="F16" s="655" t="n"/>
+      <c r="G16" s="655" t="n"/>
+      <c r="H16" s="655" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="611" t="n"/>
-      <c r="B17" s="611" t="n"/>
-      <c r="C17" s="611" t="n"/>
-      <c r="D17" s="611" t="n"/>
-      <c r="E17" s="611" t="n"/>
-      <c r="F17" s="611" t="n"/>
-      <c r="G17" s="611" t="n"/>
-      <c r="H17" s="611" t="n"/>
+      <c r="A17" s="655" t="n"/>
+      <c r="B17" s="655" t="n"/>
+      <c r="C17" s="655" t="n"/>
+      <c r="D17" s="655" t="n"/>
+      <c r="E17" s="655" t="n"/>
+      <c r="F17" s="655" t="n"/>
+      <c r="G17" s="655" t="n"/>
+      <c r="H17" s="655" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="611" t="n"/>
-      <c r="B18" s="611" t="n"/>
-      <c r="C18" s="611" t="n"/>
-      <c r="D18" s="611" t="n"/>
-      <c r="E18" s="611" t="n"/>
-      <c r="F18" s="611" t="n"/>
-      <c r="G18" s="611" t="n"/>
-      <c r="H18" s="611" t="n"/>
+      <c r="A18" s="655" t="n"/>
+      <c r="B18" s="655" t="n"/>
+      <c r="C18" s="655" t="n"/>
+      <c r="D18" s="655" t="n"/>
+      <c r="E18" s="655" t="n"/>
+      <c r="F18" s="655" t="n"/>
+      <c r="G18" s="655" t="n"/>
+      <c r="H18" s="655" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="611" t="n"/>
-      <c r="B19" s="611" t="n"/>
-      <c r="C19" s="611" t="n"/>
-      <c r="D19" s="611" t="n"/>
-      <c r="E19" s="611" t="n"/>
-      <c r="F19" s="611" t="n"/>
-      <c r="G19" s="611" t="n"/>
-      <c r="H19" s="611" t="n"/>
+      <c r="A19" s="655" t="n"/>
+      <c r="B19" s="655" t="n"/>
+      <c r="C19" s="655" t="n"/>
+      <c r="D19" s="655" t="n"/>
+      <c r="E19" s="655" t="n"/>
+      <c r="F19" s="655" t="n"/>
+      <c r="G19" s="655" t="n"/>
+      <c r="H19" s="655" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="611" t="n"/>
-      <c r="B20" s="611" t="n"/>
-      <c r="C20" s="611" t="n"/>
-      <c r="D20" s="611" t="n"/>
-      <c r="E20" s="611" t="n"/>
-      <c r="F20" s="611" t="n"/>
-      <c r="G20" s="611" t="n"/>
-      <c r="H20" s="611" t="n"/>
+      <c r="A20" s="655" t="n"/>
+      <c r="B20" s="655" t="n"/>
+      <c r="C20" s="655" t="n"/>
+      <c r="D20" s="655" t="n"/>
+      <c r="E20" s="655" t="n"/>
+      <c r="F20" s="655" t="n"/>
+      <c r="G20" s="655" t="n"/>
+      <c r="H20" s="655" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="611" t="n"/>
-      <c r="B21" s="611" t="n"/>
-      <c r="C21" s="611" t="n"/>
-      <c r="D21" s="611" t="n"/>
-      <c r="E21" s="611" t="n"/>
-      <c r="F21" s="611" t="n"/>
-      <c r="G21" s="611" t="n"/>
-      <c r="H21" s="611" t="n"/>
+      <c r="A21" s="655" t="n"/>
+      <c r="B21" s="655" t="n"/>
+      <c r="C21" s="655" t="n"/>
+      <c r="D21" s="655" t="n"/>
+      <c r="E21" s="655" t="n"/>
+      <c r="F21" s="655" t="n"/>
+      <c r="G21" s="655" t="n"/>
+      <c r="H21" s="655" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="611" t="n"/>
-      <c r="B22" s="611" t="n"/>
-      <c r="C22" s="611" t="n"/>
-      <c r="D22" s="611" t="n"/>
-      <c r="E22" s="611" t="n"/>
-      <c r="F22" s="611" t="n"/>
-      <c r="G22" s="611" t="n"/>
-      <c r="H22" s="611" t="n"/>
+      <c r="A22" s="655" t="n"/>
+      <c r="B22" s="655" t="n"/>
+      <c r="C22" s="655" t="n"/>
+      <c r="D22" s="655" t="n"/>
+      <c r="E22" s="655" t="n"/>
+      <c r="F22" s="655" t="n"/>
+      <c r="G22" s="655" t="n"/>
+      <c r="H22" s="655" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="611" t="n"/>
-      <c r="B23" s="611" t="n"/>
-      <c r="C23" s="611" t="n"/>
-      <c r="D23" s="611" t="n"/>
-      <c r="E23" s="611" t="n"/>
-      <c r="F23" s="611" t="n"/>
-      <c r="G23" s="611" t="n"/>
-      <c r="H23" s="611" t="n"/>
+      <c r="A23" s="655" t="n"/>
+      <c r="B23" s="655" t="n"/>
+      <c r="C23" s="655" t="n"/>
+      <c r="D23" s="655" t="n"/>
+      <c r="E23" s="655" t="n"/>
+      <c r="F23" s="655" t="n"/>
+      <c r="G23" s="655" t="n"/>
+      <c r="H23" s="655" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="611" t="n"/>
-      <c r="B24" s="611" t="n"/>
-      <c r="C24" s="611" t="n"/>
-      <c r="D24" s="611" t="n"/>
-      <c r="E24" s="611" t="n"/>
-      <c r="F24" s="611" t="n"/>
-      <c r="G24" s="611" t="n"/>
-      <c r="H24" s="611" t="n"/>
+      <c r="A24" s="655" t="n"/>
+      <c r="B24" s="655" t="n"/>
+      <c r="C24" s="655" t="n"/>
+      <c r="D24" s="655" t="n"/>
+      <c r="E24" s="655" t="n"/>
+      <c r="F24" s="655" t="n"/>
+      <c r="G24" s="655" t="n"/>
+      <c r="H24" s="655" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="611" t="n"/>
-      <c r="B25" s="611" t="n"/>
-      <c r="C25" s="611" t="n"/>
-      <c r="D25" s="611" t="n"/>
-      <c r="E25" s="611" t="n"/>
-      <c r="F25" s="611" t="n"/>
-      <c r="G25" s="611" t="n"/>
-      <c r="H25" s="611" t="n"/>
+      <c r="A25" s="655" t="n"/>
+      <c r="B25" s="655" t="n"/>
+      <c r="C25" s="655" t="n"/>
+      <c r="D25" s="655" t="n"/>
+      <c r="E25" s="655" t="n"/>
+      <c r="F25" s="655" t="n"/>
+      <c r="G25" s="655" t="n"/>
+      <c r="H25" s="655" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="611" t="n"/>
-      <c r="B26" s="611" t="n"/>
-      <c r="C26" s="611" t="n"/>
-      <c r="D26" s="611" t="n"/>
-      <c r="E26" s="611" t="n"/>
-      <c r="F26" s="611" t="n"/>
-      <c r="G26" s="611" t="n"/>
-      <c r="H26" s="611" t="n"/>
+      <c r="A26" s="655" t="n"/>
+      <c r="B26" s="655" t="n"/>
+      <c r="C26" s="655" t="n"/>
+      <c r="D26" s="655" t="n"/>
+      <c r="E26" s="655" t="n"/>
+      <c r="F26" s="655" t="n"/>
+      <c r="G26" s="655" t="n"/>
+      <c r="H26" s="655" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="611" t="n"/>
-      <c r="B27" s="611" t="n"/>
-      <c r="C27" s="611" t="n"/>
-      <c r="D27" s="611" t="n"/>
-      <c r="E27" s="611" t="n"/>
-      <c r="F27" s="611" t="n"/>
-      <c r="G27" s="611" t="n"/>
-      <c r="H27" s="611" t="n"/>
+      <c r="A27" s="655" t="n"/>
+      <c r="B27" s="655" t="n"/>
+      <c r="C27" s="655" t="n"/>
+      <c r="D27" s="655" t="n"/>
+      <c r="E27" s="655" t="n"/>
+      <c r="F27" s="655" t="n"/>
+      <c r="G27" s="655" t="n"/>
+      <c r="H27" s="655" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="611" t="n"/>
-      <c r="B28" s="611" t="n"/>
-      <c r="C28" s="611" t="n"/>
-      <c r="D28" s="611" t="n"/>
-      <c r="E28" s="611" t="n"/>
-      <c r="F28" s="611" t="n"/>
-      <c r="G28" s="611" t="n"/>
-      <c r="H28" s="611" t="n"/>
+      <c r="A28" s="655" t="n"/>
+      <c r="B28" s="655" t="n"/>
+      <c r="C28" s="655" t="n"/>
+      <c r="D28" s="655" t="n"/>
+      <c r="E28" s="655" t="n"/>
+      <c r="F28" s="655" t="n"/>
+      <c r="G28" s="655" t="n"/>
+      <c r="H28" s="655" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="611" t="n"/>
-      <c r="B29" s="611" t="n"/>
-      <c r="C29" s="611" t="n"/>
-      <c r="D29" s="611" t="n"/>
-      <c r="E29" s="611" t="n"/>
-      <c r="F29" s="611" t="n"/>
-      <c r="G29" s="611" t="n"/>
-      <c r="H29" s="611" t="n"/>
+      <c r="A29" s="655" t="n"/>
+      <c r="B29" s="655" t="n"/>
+      <c r="C29" s="655" t="n"/>
+      <c r="D29" s="655" t="n"/>
+      <c r="E29" s="655" t="n"/>
+      <c r="F29" s="655" t="n"/>
+      <c r="G29" s="655" t="n"/>
+      <c r="H29" s="655" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="611" t="n"/>
-      <c r="B30" s="611" t="n"/>
-      <c r="C30" s="611" t="n"/>
-      <c r="D30" s="611" t="n"/>
-      <c r="E30" s="611" t="n"/>
-      <c r="F30" s="611" t="n"/>
-      <c r="G30" s="611" t="n"/>
-      <c r="H30" s="611" t="n"/>
+      <c r="A30" s="655" t="n"/>
+      <c r="B30" s="655" t="n"/>
+      <c r="C30" s="655" t="n"/>
+      <c r="D30" s="655" t="n"/>
+      <c r="E30" s="655" t="n"/>
+      <c r="F30" s="655" t="n"/>
+      <c r="G30" s="655" t="n"/>
+      <c r="H30" s="655" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="611" t="n"/>
-      <c r="B31" s="611" t="n"/>
-      <c r="C31" s="611" t="n"/>
-      <c r="D31" s="611" t="n"/>
-      <c r="E31" s="611" t="n"/>
-      <c r="F31" s="611" t="n"/>
-      <c r="G31" s="611" t="n"/>
-      <c r="H31" s="611" t="n"/>
+      <c r="A31" s="655" t="n"/>
+      <c r="B31" s="655" t="n"/>
+      <c r="C31" s="655" t="n"/>
+      <c r="D31" s="655" t="n"/>
+      <c r="E31" s="655" t="n"/>
+      <c r="F31" s="655" t="n"/>
+      <c r="G31" s="655" t="n"/>
+      <c r="H31" s="655" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="611" t="n"/>
-      <c r="B32" s="611" t="n"/>
-      <c r="C32" s="611" t="n"/>
-      <c r="D32" s="611" t="n"/>
-      <c r="E32" s="611" t="n"/>
-      <c r="F32" s="611" t="n"/>
-      <c r="G32" s="611" t="n"/>
-      <c r="H32" s="611" t="n"/>
+      <c r="A32" s="655" t="n"/>
+      <c r="B32" s="655" t="n"/>
+      <c r="C32" s="655" t="n"/>
+      <c r="D32" s="655" t="n"/>
+      <c r="E32" s="655" t="n"/>
+      <c r="F32" s="655" t="n"/>
+      <c r="G32" s="655" t="n"/>
+      <c r="H32" s="655" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="611" t="n"/>
-      <c r="B33" s="611" t="n"/>
-      <c r="C33" s="611" t="n"/>
-      <c r="D33" s="611" t="n"/>
-      <c r="E33" s="611" t="n"/>
-      <c r="F33" s="611" t="n"/>
-      <c r="G33" s="611" t="n"/>
-      <c r="H33" s="611" t="n"/>
+      <c r="A33" s="655" t="n"/>
+      <c r="B33" s="655" t="n"/>
+      <c r="C33" s="655" t="n"/>
+      <c r="D33" s="655" t="n"/>
+      <c r="E33" s="655" t="n"/>
+      <c r="F33" s="655" t="n"/>
+      <c r="G33" s="655" t="n"/>
+      <c r="H33" s="655" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="611" t="n"/>
-      <c r="B34" s="611" t="n"/>
-      <c r="C34" s="611" t="n"/>
-      <c r="D34" s="611" t="n"/>
-      <c r="E34" s="611" t="n"/>
-      <c r="F34" s="611" t="n"/>
-      <c r="G34" s="611" t="n"/>
-      <c r="H34" s="611" t="n"/>
+      <c r="A34" s="655" t="n"/>
+      <c r="B34" s="655" t="n"/>
+      <c r="C34" s="655" t="n"/>
+      <c r="D34" s="655" t="n"/>
+      <c r="E34" s="655" t="n"/>
+      <c r="F34" s="655" t="n"/>
+      <c r="G34" s="655" t="n"/>
+      <c r="H34" s="655" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="611" t="n"/>
-      <c r="B35" s="611" t="n"/>
-      <c r="C35" s="611" t="n"/>
-      <c r="D35" s="611" t="n"/>
-      <c r="E35" s="611" t="n"/>
-      <c r="F35" s="611" t="n"/>
-      <c r="G35" s="611" t="n"/>
-      <c r="H35" s="611" t="n"/>
+      <c r="A35" s="655" t="n"/>
+      <c r="B35" s="655" t="n"/>
+      <c r="C35" s="655" t="n"/>
+      <c r="D35" s="655" t="n"/>
+      <c r="E35" s="655" t="n"/>
+      <c r="F35" s="655" t="n"/>
+      <c r="G35" s="655" t="n"/>
+      <c r="H35" s="655" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="611" t="n"/>
-      <c r="B36" s="611" t="n"/>
-      <c r="C36" s="611" t="n"/>
-      <c r="D36" s="611" t="n"/>
-      <c r="E36" s="611" t="n"/>
-      <c r="F36" s="611" t="n"/>
-      <c r="G36" s="611" t="n"/>
-      <c r="H36" s="611" t="n"/>
+      <c r="A36" s="655" t="n"/>
+      <c r="B36" s="655" t="n"/>
+      <c r="C36" s="655" t="n"/>
+      <c r="D36" s="655" t="n"/>
+      <c r="E36" s="655" t="n"/>
+      <c r="F36" s="655" t="n"/>
+      <c r="G36" s="655" t="n"/>
+      <c r="H36" s="655" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="611" t="n"/>
-      <c r="B37" s="611" t="n"/>
-      <c r="C37" s="611" t="n"/>
-      <c r="D37" s="611" t="n"/>
-      <c r="E37" s="611" t="n"/>
-      <c r="F37" s="611" t="n"/>
-      <c r="G37" s="611" t="n"/>
-      <c r="H37" s="611" t="n"/>
+      <c r="A37" s="655" t="n"/>
+      <c r="B37" s="655" t="n"/>
+      <c r="C37" s="655" t="n"/>
+      <c r="D37" s="655" t="n"/>
+      <c r="E37" s="655" t="n"/>
+      <c r="F37" s="655" t="n"/>
+      <c r="G37" s="655" t="n"/>
+      <c r="H37" s="655" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="611" t="n"/>
-      <c r="B38" s="611" t="n"/>
-      <c r="C38" s="611" t="n"/>
-      <c r="D38" s="611" t="n"/>
-      <c r="E38" s="611" t="n"/>
-      <c r="F38" s="611" t="n"/>
-      <c r="G38" s="611" t="n"/>
-      <c r="H38" s="611" t="n"/>
+      <c r="A38" s="655" t="n"/>
+      <c r="B38" s="655" t="n"/>
+      <c r="C38" s="655" t="n"/>
+      <c r="D38" s="655" t="n"/>
+      <c r="E38" s="655" t="n"/>
+      <c r="F38" s="655" t="n"/>
+      <c r="G38" s="655" t="n"/>
+      <c r="H38" s="655" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="611" t="n"/>
-      <c r="B39" s="611" t="n"/>
-      <c r="C39" s="611" t="n"/>
-      <c r="D39" s="611" t="n"/>
-      <c r="E39" s="611" t="n"/>
-      <c r="F39" s="611" t="n"/>
-      <c r="G39" s="611" t="n"/>
-      <c r="H39" s="611" t="n"/>
+      <c r="A39" s="655" t="n"/>
+      <c r="B39" s="655" t="n"/>
+      <c r="C39" s="655" t="n"/>
+      <c r="D39" s="655" t="n"/>
+      <c r="E39" s="655" t="n"/>
+      <c r="F39" s="655" t="n"/>
+      <c r="G39" s="655" t="n"/>
+      <c r="H39" s="655" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="611" t="n"/>
-      <c r="B40" s="611" t="n"/>
-      <c r="C40" s="611" t="n"/>
-      <c r="D40" s="611" t="n"/>
-      <c r="E40" s="611" t="n"/>
-      <c r="F40" s="611" t="n"/>
-      <c r="G40" s="611" t="n"/>
-      <c r="H40" s="611" t="n"/>
+      <c r="A40" s="655" t="n"/>
+      <c r="B40" s="655" t="n"/>
+      <c r="C40" s="655" t="n"/>
+      <c r="D40" s="655" t="n"/>
+      <c r="E40" s="655" t="n"/>
+      <c r="F40" s="655" t="n"/>
+      <c r="G40" s="655" t="n"/>
+      <c r="H40" s="655" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
     </row>
@@ -2941,504 +3073,504 @@
       <c r="J2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="612" t="inlineStr">
+      <c r="A3" s="656" t="inlineStr">
         <is>
           <t>15.07.2026</t>
         </is>
       </c>
-      <c r="B3" s="612" t="inlineStr">
+      <c r="B3" s="656" t="inlineStr">
         <is>
           <t>4039-95</t>
         </is>
       </c>
-      <c r="C3" s="612" t="inlineStr">
+      <c r="C3" s="656" t="inlineStr">
         <is>
           <t>1.0026-2X2500X1250</t>
         </is>
       </c>
-      <c r="D3" s="612" t="n">
+      <c r="D3" s="656" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="612" t="inlineStr">
+      <c r="E3" s="656" t="inlineStr">
         <is>
           <t>00:04:03</t>
         </is>
       </c>
-      <c r="F3" s="612" t="n"/>
-      <c r="G3" s="612" t="n"/>
-      <c r="H3" s="612" t="n"/>
+      <c r="F3" s="656" t="n"/>
+      <c r="G3" s="656" t="n"/>
+      <c r="H3" s="656" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="612" t="n"/>
-      <c r="B4" s="612" t="inlineStr">
+      <c r="A4" s="656" t="n"/>
+      <c r="B4" s="656" t="inlineStr">
         <is>
           <t>4039-96</t>
         </is>
       </c>
-      <c r="C4" s="612" t="inlineStr">
+      <c r="C4" s="656" t="inlineStr">
         <is>
           <t>3.3535-2X2500X1250</t>
         </is>
       </c>
-      <c r="D4" s="612" t="n">
+      <c r="D4" s="656" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="612" t="inlineStr">
+      <c r="E4" s="656" t="inlineStr">
         <is>
           <t>00:03:09</t>
         </is>
       </c>
-      <c r="F4" s="612" t="n"/>
-      <c r="G4" s="612" t="n"/>
-      <c r="H4" s="612" t="n"/>
+      <c r="F4" s="656" t="n"/>
+      <c r="G4" s="656" t="n"/>
+      <c r="H4" s="656" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="612" t="n"/>
-      <c r="B5" s="612" t="inlineStr">
+      <c r="A5" s="656" t="n"/>
+      <c r="B5" s="656" t="inlineStr">
         <is>
           <t>4039-97</t>
         </is>
       </c>
-      <c r="C5" s="612" t="inlineStr">
+      <c r="C5" s="656" t="inlineStr">
         <is>
           <t>-----</t>
         </is>
       </c>
-      <c r="D5" s="612" t="n">
+      <c r="D5" s="656" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="612" t="inlineStr">
+      <c r="E5" s="656" t="inlineStr">
         <is>
           <t>00:03:56</t>
         </is>
       </c>
-      <c r="F5" s="612" t="n"/>
-      <c r="G5" s="612" t="n"/>
-      <c r="H5" s="612" t="n"/>
+      <c r="F5" s="656" t="n"/>
+      <c r="G5" s="656" t="n"/>
+      <c r="H5" s="656" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="612" t="n"/>
-      <c r="B6" s="612" t="n"/>
-      <c r="C6" s="612" t="n"/>
-      <c r="D6" s="612" t="n"/>
-      <c r="E6" s="612" t="n"/>
-      <c r="F6" s="612" t="n"/>
-      <c r="G6" s="612" t="n"/>
-      <c r="H6" s="612" t="n"/>
+      <c r="A6" s="656" t="n"/>
+      <c r="B6" s="656" t="n"/>
+      <c r="C6" s="656" t="n"/>
+      <c r="D6" s="656" t="n"/>
+      <c r="E6" s="656" t="n"/>
+      <c r="F6" s="656" t="n"/>
+      <c r="G6" s="656" t="n"/>
+      <c r="H6" s="656" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="611" t="n"/>
-      <c r="B7" s="611" t="n"/>
-      <c r="C7" s="611" t="n"/>
-      <c r="D7" s="611" t="n"/>
-      <c r="E7" s="611" t="n"/>
-      <c r="F7" s="611" t="n"/>
-      <c r="G7" s="611" t="n"/>
-      <c r="H7" s="611" t="n"/>
+      <c r="A7" s="656" t="n"/>
+      <c r="B7" s="656" t="n"/>
+      <c r="C7" s="656" t="n"/>
+      <c r="D7" s="656" t="n"/>
+      <c r="E7" s="656" t="n"/>
+      <c r="F7" s="656" t="n"/>
+      <c r="G7" s="656" t="n"/>
+      <c r="H7" s="656" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="611" t="n"/>
-      <c r="B8" s="611" t="n"/>
-      <c r="C8" s="611" t="n"/>
-      <c r="D8" s="611" t="n"/>
-      <c r="E8" s="611" t="n"/>
-      <c r="F8" s="611" t="n"/>
-      <c r="G8" s="611" t="n"/>
-      <c r="H8" s="611" t="n"/>
+      <c r="A8" s="656" t="n"/>
+      <c r="B8" s="656" t="n"/>
+      <c r="C8" s="656" t="n"/>
+      <c r="D8" s="656" t="n"/>
+      <c r="E8" s="656" t="n"/>
+      <c r="F8" s="656" t="n"/>
+      <c r="G8" s="656" t="n"/>
+      <c r="H8" s="656" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="611" t="n"/>
-      <c r="B9" s="611" t="n"/>
-      <c r="C9" s="611" t="n"/>
-      <c r="D9" s="611" t="n"/>
-      <c r="E9" s="611" t="n"/>
-      <c r="F9" s="611" t="n"/>
-      <c r="G9" s="611" t="n"/>
-      <c r="H9" s="611" t="n"/>
+      <c r="A9" s="656" t="n"/>
+      <c r="B9" s="656" t="n"/>
+      <c r="C9" s="656" t="n"/>
+      <c r="D9" s="656" t="n"/>
+      <c r="E9" s="656" t="n"/>
+      <c r="F9" s="656" t="n"/>
+      <c r="G9" s="656" t="n"/>
+      <c r="H9" s="656" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="611" t="n"/>
-      <c r="B10" s="611" t="n"/>
-      <c r="C10" s="611" t="n"/>
-      <c r="D10" s="611" t="n"/>
-      <c r="E10" s="611" t="n"/>
-      <c r="F10" s="611" t="n"/>
-      <c r="G10" s="611" t="n"/>
-      <c r="H10" s="611" t="n"/>
+      <c r="A10" s="656" t="n"/>
+      <c r="B10" s="656" t="n"/>
+      <c r="C10" s="656" t="n"/>
+      <c r="D10" s="656" t="n"/>
+      <c r="E10" s="656" t="n"/>
+      <c r="F10" s="656" t="n"/>
+      <c r="G10" s="656" t="n"/>
+      <c r="H10" s="656" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="611" t="n"/>
-      <c r="B11" s="611" t="n"/>
-      <c r="C11" s="611" t="n"/>
-      <c r="D11" s="611" t="n"/>
-      <c r="E11" s="611" t="n"/>
-      <c r="F11" s="611" t="n"/>
-      <c r="G11" s="611" t="n"/>
-      <c r="H11" s="611" t="n"/>
+      <c r="A11" s="656" t="n"/>
+      <c r="B11" s="656" t="n"/>
+      <c r="C11" s="656" t="n"/>
+      <c r="D11" s="656" t="n"/>
+      <c r="E11" s="656" t="n"/>
+      <c r="F11" s="656" t="n"/>
+      <c r="G11" s="656" t="n"/>
+      <c r="H11" s="656" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="611" t="n"/>
-      <c r="B12" s="611" t="n"/>
-      <c r="C12" s="611" t="n"/>
-      <c r="D12" s="611" t="n"/>
-      <c r="E12" s="611" t="n"/>
-      <c r="F12" s="611" t="n"/>
-      <c r="G12" s="611" t="n"/>
-      <c r="H12" s="611" t="n"/>
+      <c r="A12" s="656" t="n"/>
+      <c r="B12" s="656" t="n"/>
+      <c r="C12" s="656" t="n"/>
+      <c r="D12" s="656" t="n"/>
+      <c r="E12" s="656" t="n"/>
+      <c r="F12" s="656" t="n"/>
+      <c r="G12" s="656" t="n"/>
+      <c r="H12" s="656" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="611" t="n"/>
-      <c r="B13" s="611" t="n"/>
-      <c r="C13" s="611" t="n"/>
-      <c r="D13" s="611" t="n"/>
-      <c r="E13" s="611" t="n"/>
-      <c r="F13" s="611" t="n"/>
-      <c r="G13" s="611" t="n"/>
-      <c r="H13" s="611" t="n"/>
+      <c r="A13" s="656" t="n"/>
+      <c r="B13" s="656" t="n"/>
+      <c r="C13" s="656" t="n"/>
+      <c r="D13" s="656" t="n"/>
+      <c r="E13" s="656" t="n"/>
+      <c r="F13" s="656" t="n"/>
+      <c r="G13" s="656" t="n"/>
+      <c r="H13" s="656" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="611" t="n"/>
-      <c r="B14" s="611" t="n"/>
-      <c r="C14" s="611" t="n"/>
-      <c r="D14" s="611" t="n"/>
-      <c r="E14" s="611" t="n"/>
-      <c r="F14" s="611" t="n"/>
-      <c r="G14" s="611" t="n"/>
-      <c r="H14" s="611" t="n"/>
+      <c r="A14" s="656" t="n"/>
+      <c r="B14" s="656" t="n"/>
+      <c r="C14" s="656" t="n"/>
+      <c r="D14" s="656" t="n"/>
+      <c r="E14" s="656" t="n"/>
+      <c r="F14" s="656" t="n"/>
+      <c r="G14" s="656" t="n"/>
+      <c r="H14" s="656" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="611" t="n"/>
-      <c r="B15" s="611" t="n"/>
-      <c r="C15" s="611" t="n"/>
-      <c r="D15" s="611" t="n"/>
-      <c r="E15" s="611" t="n"/>
-      <c r="F15" s="611" t="n"/>
-      <c r="G15" s="611" t="n"/>
-      <c r="H15" s="611" t="n"/>
+      <c r="A15" s="656" t="n"/>
+      <c r="B15" s="656" t="n"/>
+      <c r="C15" s="656" t="n"/>
+      <c r="D15" s="656" t="n"/>
+      <c r="E15" s="656" t="n"/>
+      <c r="F15" s="656" t="n"/>
+      <c r="G15" s="656" t="n"/>
+      <c r="H15" s="656" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="611" t="n"/>
-      <c r="B16" s="611" t="n"/>
-      <c r="C16" s="611" t="n"/>
-      <c r="D16" s="611" t="n"/>
-      <c r="E16" s="611" t="n"/>
-      <c r="F16" s="611" t="n"/>
-      <c r="G16" s="611" t="n"/>
-      <c r="H16" s="611" t="n"/>
+      <c r="A16" s="656" t="n"/>
+      <c r="B16" s="656" t="n"/>
+      <c r="C16" s="656" t="n"/>
+      <c r="D16" s="656" t="n"/>
+      <c r="E16" s="656" t="n"/>
+      <c r="F16" s="656" t="n"/>
+      <c r="G16" s="656" t="n"/>
+      <c r="H16" s="656" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="611" t="n"/>
-      <c r="B17" s="611" t="n"/>
-      <c r="C17" s="611" t="n"/>
-      <c r="D17" s="611" t="n"/>
-      <c r="E17" s="611" t="n"/>
-      <c r="F17" s="611" t="n"/>
-      <c r="G17" s="611" t="n"/>
-      <c r="H17" s="611" t="n"/>
+      <c r="A17" s="656" t="n"/>
+      <c r="B17" s="656" t="n"/>
+      <c r="C17" s="656" t="n"/>
+      <c r="D17" s="656" t="n"/>
+      <c r="E17" s="656" t="n"/>
+      <c r="F17" s="656" t="n"/>
+      <c r="G17" s="656" t="n"/>
+      <c r="H17" s="656" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="611" t="n"/>
-      <c r="B18" s="611" t="n"/>
-      <c r="C18" s="611" t="n"/>
-      <c r="D18" s="611" t="n"/>
-      <c r="E18" s="611" t="n"/>
-      <c r="F18" s="611" t="n"/>
-      <c r="G18" s="611" t="n"/>
-      <c r="H18" s="611" t="n"/>
+      <c r="A18" s="656" t="n"/>
+      <c r="B18" s="656" t="n"/>
+      <c r="C18" s="656" t="n"/>
+      <c r="D18" s="656" t="n"/>
+      <c r="E18" s="656" t="n"/>
+      <c r="F18" s="656" t="n"/>
+      <c r="G18" s="656" t="n"/>
+      <c r="H18" s="656" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="611" t="n"/>
-      <c r="B19" s="611" t="n"/>
-      <c r="C19" s="611" t="n"/>
-      <c r="D19" s="611" t="n"/>
-      <c r="E19" s="611" t="n"/>
-      <c r="F19" s="611" t="n"/>
-      <c r="G19" s="611" t="n"/>
-      <c r="H19" s="611" t="n"/>
+      <c r="A19" s="656" t="n"/>
+      <c r="B19" s="656" t="n"/>
+      <c r="C19" s="656" t="n"/>
+      <c r="D19" s="656" t="n"/>
+      <c r="E19" s="656" t="n"/>
+      <c r="F19" s="656" t="n"/>
+      <c r="G19" s="656" t="n"/>
+      <c r="H19" s="656" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="611" t="n"/>
-      <c r="B20" s="611" t="n"/>
-      <c r="C20" s="611" t="n"/>
-      <c r="D20" s="611" t="n"/>
-      <c r="E20" s="611" t="n"/>
-      <c r="F20" s="611" t="n"/>
-      <c r="G20" s="611" t="n"/>
-      <c r="H20" s="611" t="n"/>
+      <c r="A20" s="656" t="n"/>
+      <c r="B20" s="656" t="n"/>
+      <c r="C20" s="656" t="n"/>
+      <c r="D20" s="656" t="n"/>
+      <c r="E20" s="656" t="n"/>
+      <c r="F20" s="656" t="n"/>
+      <c r="G20" s="656" t="n"/>
+      <c r="H20" s="656" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="611" t="n"/>
-      <c r="B21" s="611" t="n"/>
-      <c r="C21" s="611" t="n"/>
-      <c r="D21" s="611" t="n"/>
-      <c r="E21" s="611" t="n"/>
-      <c r="F21" s="611" t="n"/>
-      <c r="G21" s="611" t="n"/>
-      <c r="H21" s="611" t="n"/>
+      <c r="A21" s="656" t="n"/>
+      <c r="B21" s="656" t="n"/>
+      <c r="C21" s="656" t="n"/>
+      <c r="D21" s="656" t="n"/>
+      <c r="E21" s="656" t="n"/>
+      <c r="F21" s="656" t="n"/>
+      <c r="G21" s="656" t="n"/>
+      <c r="H21" s="656" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="611" t="n"/>
-      <c r="B22" s="611" t="n"/>
-      <c r="C22" s="611" t="n"/>
-      <c r="D22" s="611" t="n"/>
-      <c r="E22" s="611" t="n"/>
-      <c r="F22" s="611" t="n"/>
-      <c r="G22" s="611" t="n"/>
-      <c r="H22" s="611" t="n"/>
+      <c r="A22" s="656" t="n"/>
+      <c r="B22" s="656" t="n"/>
+      <c r="C22" s="656" t="n"/>
+      <c r="D22" s="656" t="n"/>
+      <c r="E22" s="656" t="n"/>
+      <c r="F22" s="656" t="n"/>
+      <c r="G22" s="656" t="n"/>
+      <c r="H22" s="656" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="611" t="n"/>
-      <c r="B23" s="611" t="n"/>
-      <c r="C23" s="611" t="n"/>
-      <c r="D23" s="611" t="n"/>
-      <c r="E23" s="611" t="n"/>
-      <c r="F23" s="611" t="n"/>
-      <c r="G23" s="611" t="n"/>
-      <c r="H23" s="611" t="n"/>
+      <c r="A23" s="656" t="n"/>
+      <c r="B23" s="656" t="n"/>
+      <c r="C23" s="656" t="n"/>
+      <c r="D23" s="656" t="n"/>
+      <c r="E23" s="656" t="n"/>
+      <c r="F23" s="656" t="n"/>
+      <c r="G23" s="656" t="n"/>
+      <c r="H23" s="656" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="611" t="n"/>
-      <c r="B24" s="611" t="n"/>
-      <c r="C24" s="611" t="n"/>
-      <c r="D24" s="611" t="n"/>
-      <c r="E24" s="611" t="n"/>
-      <c r="F24" s="611" t="n"/>
-      <c r="G24" s="611" t="n"/>
-      <c r="H24" s="611" t="n"/>
+      <c r="A24" s="656" t="n"/>
+      <c r="B24" s="656" t="n"/>
+      <c r="C24" s="656" t="n"/>
+      <c r="D24" s="656" t="n"/>
+      <c r="E24" s="656" t="n"/>
+      <c r="F24" s="656" t="n"/>
+      <c r="G24" s="656" t="n"/>
+      <c r="H24" s="656" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="611" t="n"/>
-      <c r="B25" s="611" t="n"/>
-      <c r="C25" s="611" t="n"/>
-      <c r="D25" s="611" t="n"/>
-      <c r="E25" s="611" t="n"/>
-      <c r="F25" s="611" t="n"/>
-      <c r="G25" s="611" t="n"/>
-      <c r="H25" s="611" t="n"/>
+      <c r="A25" s="656" t="n"/>
+      <c r="B25" s="656" t="n"/>
+      <c r="C25" s="656" t="n"/>
+      <c r="D25" s="656" t="n"/>
+      <c r="E25" s="656" t="n"/>
+      <c r="F25" s="656" t="n"/>
+      <c r="G25" s="656" t="n"/>
+      <c r="H25" s="656" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="611" t="n"/>
-      <c r="B26" s="611" t="n"/>
-      <c r="C26" s="611" t="n"/>
-      <c r="D26" s="611" t="n"/>
-      <c r="E26" s="611" t="n"/>
-      <c r="F26" s="611" t="n"/>
-      <c r="G26" s="611" t="n"/>
-      <c r="H26" s="611" t="n"/>
+      <c r="A26" s="656" t="n"/>
+      <c r="B26" s="656" t="n"/>
+      <c r="C26" s="656" t="n"/>
+      <c r="D26" s="656" t="n"/>
+      <c r="E26" s="656" t="n"/>
+      <c r="F26" s="656" t="n"/>
+      <c r="G26" s="656" t="n"/>
+      <c r="H26" s="656" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="611" t="n"/>
-      <c r="B27" s="611" t="n"/>
-      <c r="C27" s="611" t="n"/>
-      <c r="D27" s="611" t="n"/>
-      <c r="E27" s="611" t="n"/>
-      <c r="F27" s="611" t="n"/>
-      <c r="G27" s="611" t="n"/>
-      <c r="H27" s="611" t="n"/>
+      <c r="A27" s="656" t="n"/>
+      <c r="B27" s="656" t="n"/>
+      <c r="C27" s="656" t="n"/>
+      <c r="D27" s="656" t="n"/>
+      <c r="E27" s="656" t="n"/>
+      <c r="F27" s="656" t="n"/>
+      <c r="G27" s="656" t="n"/>
+      <c r="H27" s="656" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="611" t="n"/>
-      <c r="B28" s="611" t="n"/>
-      <c r="C28" s="611" t="n"/>
-      <c r="D28" s="611" t="n"/>
-      <c r="E28" s="611" t="n"/>
-      <c r="F28" s="611" t="n"/>
-      <c r="G28" s="611" t="n"/>
-      <c r="H28" s="611" t="n"/>
+      <c r="A28" s="656" t="n"/>
+      <c r="B28" s="656" t="n"/>
+      <c r="C28" s="656" t="n"/>
+      <c r="D28" s="656" t="n"/>
+      <c r="E28" s="656" t="n"/>
+      <c r="F28" s="656" t="n"/>
+      <c r="G28" s="656" t="n"/>
+      <c r="H28" s="656" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="611" t="n"/>
-      <c r="B29" s="611" t="n"/>
-      <c r="C29" s="611" t="n"/>
-      <c r="D29" s="611" t="n"/>
-      <c r="E29" s="611" t="n"/>
-      <c r="F29" s="611" t="n"/>
-      <c r="G29" s="611" t="n"/>
-      <c r="H29" s="611" t="n"/>
+      <c r="A29" s="656" t="n"/>
+      <c r="B29" s="656" t="n"/>
+      <c r="C29" s="656" t="n"/>
+      <c r="D29" s="656" t="n"/>
+      <c r="E29" s="656" t="n"/>
+      <c r="F29" s="656" t="n"/>
+      <c r="G29" s="656" t="n"/>
+      <c r="H29" s="656" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="611" t="n"/>
-      <c r="B30" s="611" t="n"/>
-      <c r="C30" s="611" t="n"/>
-      <c r="D30" s="611" t="n"/>
-      <c r="E30" s="611" t="n"/>
-      <c r="F30" s="611" t="n"/>
-      <c r="G30" s="611" t="n"/>
-      <c r="H30" s="611" t="n"/>
+      <c r="A30" s="656" t="n"/>
+      <c r="B30" s="656" t="n"/>
+      <c r="C30" s="656" t="n"/>
+      <c r="D30" s="656" t="n"/>
+      <c r="E30" s="656" t="n"/>
+      <c r="F30" s="656" t="n"/>
+      <c r="G30" s="656" t="n"/>
+      <c r="H30" s="656" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="611" t="n"/>
-      <c r="B31" s="611" t="n"/>
-      <c r="C31" s="611" t="n"/>
-      <c r="D31" s="611" t="n"/>
-      <c r="E31" s="611" t="n"/>
-      <c r="F31" s="611" t="n"/>
-      <c r="G31" s="611" t="n"/>
-      <c r="H31" s="611" t="n"/>
+      <c r="A31" s="656" t="n"/>
+      <c r="B31" s="656" t="n"/>
+      <c r="C31" s="656" t="n"/>
+      <c r="D31" s="656" t="n"/>
+      <c r="E31" s="656" t="n"/>
+      <c r="F31" s="656" t="n"/>
+      <c r="G31" s="656" t="n"/>
+      <c r="H31" s="656" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="611" t="n"/>
-      <c r="B32" s="611" t="n"/>
-      <c r="C32" s="611" t="n"/>
-      <c r="D32" s="611" t="n"/>
-      <c r="E32" s="611" t="n"/>
-      <c r="F32" s="611" t="n"/>
-      <c r="G32" s="611" t="n"/>
-      <c r="H32" s="611" t="n"/>
+      <c r="A32" s="656" t="n"/>
+      <c r="B32" s="656" t="n"/>
+      <c r="C32" s="656" t="n"/>
+      <c r="D32" s="656" t="n"/>
+      <c r="E32" s="656" t="n"/>
+      <c r="F32" s="656" t="n"/>
+      <c r="G32" s="656" t="n"/>
+      <c r="H32" s="656" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="611" t="n"/>
-      <c r="B33" s="611" t="n"/>
-      <c r="C33" s="611" t="n"/>
-      <c r="D33" s="611" t="n"/>
-      <c r="E33" s="611" t="n"/>
-      <c r="F33" s="611" t="n"/>
-      <c r="G33" s="611" t="n"/>
-      <c r="H33" s="611" t="n"/>
+      <c r="A33" s="656" t="n"/>
+      <c r="B33" s="656" t="n"/>
+      <c r="C33" s="656" t="n"/>
+      <c r="D33" s="656" t="n"/>
+      <c r="E33" s="656" t="n"/>
+      <c r="F33" s="656" t="n"/>
+      <c r="G33" s="656" t="n"/>
+      <c r="H33" s="656" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="611" t="n"/>
-      <c r="B34" s="611" t="n"/>
-      <c r="C34" s="611" t="n"/>
-      <c r="D34" s="611" t="n"/>
-      <c r="E34" s="611" t="n"/>
-      <c r="F34" s="611" t="n"/>
-      <c r="G34" s="611" t="n"/>
-      <c r="H34" s="611" t="n"/>
+      <c r="A34" s="656" t="n"/>
+      <c r="B34" s="656" t="n"/>
+      <c r="C34" s="656" t="n"/>
+      <c r="D34" s="656" t="n"/>
+      <c r="E34" s="656" t="n"/>
+      <c r="F34" s="656" t="n"/>
+      <c r="G34" s="656" t="n"/>
+      <c r="H34" s="656" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="611" t="n"/>
-      <c r="B35" s="611" t="n"/>
-      <c r="C35" s="611" t="n"/>
-      <c r="D35" s="611" t="n"/>
-      <c r="E35" s="611" t="n"/>
-      <c r="F35" s="611" t="n"/>
-      <c r="G35" s="611" t="n"/>
-      <c r="H35" s="611" t="n"/>
+      <c r="A35" s="656" t="n"/>
+      <c r="B35" s="656" t="n"/>
+      <c r="C35" s="656" t="n"/>
+      <c r="D35" s="656" t="n"/>
+      <c r="E35" s="656" t="n"/>
+      <c r="F35" s="656" t="n"/>
+      <c r="G35" s="656" t="n"/>
+      <c r="H35" s="656" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="611" t="n"/>
-      <c r="B36" s="611" t="n"/>
-      <c r="C36" s="611" t="n"/>
-      <c r="D36" s="611" t="n"/>
-      <c r="E36" s="611" t="n"/>
-      <c r="F36" s="611" t="n"/>
-      <c r="G36" s="611" t="n"/>
-      <c r="H36" s="611" t="n"/>
+      <c r="A36" s="656" t="n"/>
+      <c r="B36" s="656" t="n"/>
+      <c r="C36" s="656" t="n"/>
+      <c r="D36" s="656" t="n"/>
+      <c r="E36" s="656" t="n"/>
+      <c r="F36" s="656" t="n"/>
+      <c r="G36" s="656" t="n"/>
+      <c r="H36" s="656" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="611" t="n"/>
-      <c r="B37" s="611" t="n"/>
-      <c r="C37" s="611" t="n"/>
-      <c r="D37" s="611" t="n"/>
-      <c r="E37" s="611" t="n"/>
-      <c r="F37" s="611" t="n"/>
-      <c r="G37" s="611" t="n"/>
-      <c r="H37" s="611" t="n"/>
+      <c r="A37" s="656" t="n"/>
+      <c r="B37" s="656" t="n"/>
+      <c r="C37" s="656" t="n"/>
+      <c r="D37" s="656" t="n"/>
+      <c r="E37" s="656" t="n"/>
+      <c r="F37" s="656" t="n"/>
+      <c r="G37" s="656" t="n"/>
+      <c r="H37" s="656" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="611" t="n"/>
-      <c r="B38" s="611" t="n"/>
-      <c r="C38" s="611" t="n"/>
-      <c r="D38" s="611" t="n"/>
-      <c r="E38" s="611" t="n"/>
-      <c r="F38" s="611" t="n"/>
-      <c r="G38" s="611" t="n"/>
-      <c r="H38" s="611" t="n"/>
+      <c r="A38" s="656" t="n"/>
+      <c r="B38" s="656" t="n"/>
+      <c r="C38" s="656" t="n"/>
+      <c r="D38" s="656" t="n"/>
+      <c r="E38" s="656" t="n"/>
+      <c r="F38" s="656" t="n"/>
+      <c r="G38" s="656" t="n"/>
+      <c r="H38" s="656" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="611" t="n"/>
-      <c r="B39" s="611" t="n"/>
-      <c r="C39" s="611" t="n"/>
-      <c r="D39" s="611" t="n"/>
-      <c r="E39" s="611" t="n"/>
-      <c r="F39" s="611" t="n"/>
-      <c r="G39" s="611" t="n"/>
-      <c r="H39" s="611" t="n"/>
+      <c r="A39" s="656" t="n"/>
+      <c r="B39" s="656" t="n"/>
+      <c r="C39" s="656" t="n"/>
+      <c r="D39" s="656" t="n"/>
+      <c r="E39" s="656" t="n"/>
+      <c r="F39" s="656" t="n"/>
+      <c r="G39" s="656" t="n"/>
+      <c r="H39" s="656" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="611" t="n"/>
-      <c r="B40" s="611" t="n"/>
-      <c r="C40" s="611" t="n"/>
-      <c r="D40" s="611" t="n"/>
-      <c r="E40" s="611" t="n"/>
-      <c r="F40" s="611" t="n"/>
-      <c r="G40" s="611" t="n"/>
-      <c r="H40" s="611" t="n"/>
+      <c r="A40" s="656" t="n"/>
+      <c r="B40" s="656" t="n"/>
+      <c r="C40" s="656" t="n"/>
+      <c r="D40" s="656" t="n"/>
+      <c r="E40" s="656" t="n"/>
+      <c r="F40" s="656" t="n"/>
+      <c r="G40" s="656" t="n"/>
+      <c r="H40" s="656" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
     </row>

</xml_diff>

<commit_message>
feat: img preview for leftover parts
</commit_message>
<xml_diff>
--- a/users/uzuran/burn_table.xlsx
+++ b/users/uzuran/burn_table.xlsx
@@ -67,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="657">
+  <cellXfs count="667">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1760,6 +1760,36 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2470,532 +2500,532 @@
       <c r="J2" s="3" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="655" t="inlineStr">
+      <c r="A3" s="665" t="inlineStr">
         <is>
           <t>14.07.2026</t>
         </is>
       </c>
-      <c r="B3" s="655" t="inlineStr">
+      <c r="B3" s="665" t="inlineStr">
         <is>
           <t>4039-95</t>
         </is>
       </c>
-      <c r="C3" s="655" t="inlineStr">
+      <c r="C3" s="665" t="inlineStr">
         <is>
           <t>1.0026-2X2500X1250</t>
         </is>
       </c>
-      <c r="D3" s="655" t="n">
+      <c r="D3" s="665" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="655" t="inlineStr">
+      <c r="E3" s="665" t="inlineStr">
         <is>
           <t>00:04:03</t>
         </is>
       </c>
-      <c r="F3" s="655" t="n"/>
-      <c r="G3" s="655" t="n"/>
-      <c r="H3" s="655" t="n"/>
+      <c r="F3" s="665" t="n"/>
+      <c r="G3" s="665" t="n"/>
+      <c r="H3" s="665" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="655" t="n"/>
-      <c r="B4" s="655" t="inlineStr">
+      <c r="A4" s="665" t="n"/>
+      <c r="B4" s="665" t="inlineStr">
         <is>
           <t>4039-96</t>
         </is>
       </c>
-      <c r="C4" s="655" t="inlineStr">
+      <c r="C4" s="665" t="inlineStr">
         <is>
           <t>3.3535-2X2500X1250</t>
         </is>
       </c>
-      <c r="D4" s="655" t="n">
+      <c r="D4" s="665" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="655" t="inlineStr">
+      <c r="E4" s="665" t="inlineStr">
         <is>
           <t>00:03:09</t>
         </is>
       </c>
-      <c r="F4" s="655" t="n"/>
-      <c r="G4" s="655" t="n"/>
-      <c r="H4" s="655" t="n"/>
+      <c r="F4" s="665" t="n"/>
+      <c r="G4" s="665" t="n"/>
+      <c r="H4" s="665" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="655" t="n"/>
-      <c r="B5" s="655" t="inlineStr">
+      <c r="A5" s="665" t="n"/>
+      <c r="B5" s="665" t="inlineStr">
         <is>
           <t>4039-97</t>
         </is>
       </c>
-      <c r="C5" s="655" t="inlineStr">
+      <c r="C5" s="665" t="inlineStr">
         <is>
           <t>-----</t>
         </is>
       </c>
-      <c r="D5" s="655" t="n">
+      <c r="D5" s="665" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="655" t="inlineStr">
+      <c r="E5" s="665" t="inlineStr">
         <is>
           <t>00:03:56</t>
         </is>
       </c>
-      <c r="F5" s="655" t="n"/>
-      <c r="G5" s="655" t="n"/>
-      <c r="H5" s="655" t="n"/>
+      <c r="F5" s="665" t="n"/>
+      <c r="G5" s="665" t="n"/>
+      <c r="H5" s="665" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="655" t="n"/>
-      <c r="B6" s="655" t="inlineStr">
+      <c r="A6" s="665" t="n"/>
+      <c r="B6" s="665" t="inlineStr">
         <is>
           <t>4039-98</t>
         </is>
       </c>
-      <c r="C6" s="655" t="inlineStr">
+      <c r="C6" s="665" t="inlineStr">
         <is>
           <t>-----</t>
         </is>
       </c>
-      <c r="D6" s="655" t="n">
+      <c r="D6" s="665" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="655" t="inlineStr">
+      <c r="E6" s="665" t="inlineStr">
         <is>
           <t>00:03:02</t>
         </is>
       </c>
-      <c r="F6" s="655" t="n"/>
-      <c r="G6" s="655" t="n"/>
-      <c r="H6" s="655" t="n"/>
+      <c r="F6" s="665" t="n"/>
+      <c r="G6" s="665" t="n"/>
+      <c r="H6" s="665" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="655" t="n"/>
-      <c r="B7" s="655" t="inlineStr">
+      <c r="A7" s="665" t="n"/>
+      <c r="B7" s="665" t="inlineStr">
         <is>
           <t>4039-99</t>
         </is>
       </c>
-      <c r="C7" s="655" t="inlineStr">
+      <c r="C7" s="665" t="inlineStr">
         <is>
           <t>3.3535-2X3000X1500</t>
         </is>
       </c>
-      <c r="D7" s="655" t="n">
+      <c r="D7" s="665" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="655" t="inlineStr">
+      <c r="E7" s="665" t="inlineStr">
         <is>
           <t>00:02:44</t>
         </is>
       </c>
-      <c r="F7" s="655" t="n"/>
-      <c r="G7" s="655" t="n"/>
-      <c r="H7" s="655" t="n"/>
+      <c r="F7" s="665" t="n"/>
+      <c r="G7" s="665" t="n"/>
+      <c r="H7" s="665" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="655" t="n"/>
-      <c r="B8" s="655" t="n"/>
-      <c r="C8" s="655" t="n"/>
-      <c r="D8" s="655" t="n"/>
-      <c r="E8" s="655" t="n"/>
-      <c r="F8" s="655" t="n"/>
-      <c r="G8" s="655" t="n"/>
-      <c r="H8" s="655" t="n"/>
+      <c r="A8" s="665" t="n"/>
+      <c r="B8" s="665" t="n"/>
+      <c r="C8" s="665" t="n"/>
+      <c r="D8" s="665" t="n"/>
+      <c r="E8" s="665" t="n"/>
+      <c r="F8" s="665" t="n"/>
+      <c r="G8" s="665" t="n"/>
+      <c r="H8" s="665" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="655" t="n"/>
-      <c r="B9" s="655" t="n"/>
-      <c r="C9" s="655" t="n"/>
-      <c r="D9" s="655" t="n"/>
-      <c r="E9" s="655" t="n"/>
-      <c r="F9" s="655" t="n"/>
-      <c r="G9" s="655" t="n"/>
-      <c r="H9" s="655" t="n"/>
+      <c r="A9" s="665" t="n"/>
+      <c r="B9" s="665" t="n"/>
+      <c r="C9" s="665" t="n"/>
+      <c r="D9" s="665" t="n"/>
+      <c r="E9" s="665" t="n"/>
+      <c r="F9" s="665" t="n"/>
+      <c r="G9" s="665" t="n"/>
+      <c r="H9" s="665" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="655" t="n"/>
-      <c r="B10" s="655" t="n"/>
-      <c r="C10" s="655" t="n"/>
-      <c r="D10" s="655" t="n"/>
-      <c r="E10" s="655" t="n"/>
-      <c r="F10" s="655" t="n"/>
-      <c r="G10" s="655" t="n"/>
-      <c r="H10" s="655" t="n"/>
+      <c r="A10" s="665" t="n"/>
+      <c r="B10" s="665" t="n"/>
+      <c r="C10" s="665" t="n"/>
+      <c r="D10" s="665" t="n"/>
+      <c r="E10" s="665" t="n"/>
+      <c r="F10" s="665" t="n"/>
+      <c r="G10" s="665" t="n"/>
+      <c r="H10" s="665" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="655" t="n"/>
-      <c r="B11" s="655" t="n"/>
-      <c r="C11" s="655" t="n"/>
-      <c r="D11" s="655" t="n"/>
-      <c r="E11" s="655" t="n"/>
-      <c r="F11" s="655" t="n"/>
-      <c r="G11" s="655" t="n"/>
-      <c r="H11" s="655" t="n"/>
+      <c r="A11" s="665" t="n"/>
+      <c r="B11" s="665" t="n"/>
+      <c r="C11" s="665" t="n"/>
+      <c r="D11" s="665" t="n"/>
+      <c r="E11" s="665" t="n"/>
+      <c r="F11" s="665" t="n"/>
+      <c r="G11" s="665" t="n"/>
+      <c r="H11" s="665" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="655" t="n"/>
-      <c r="B12" s="655" t="n"/>
-      <c r="C12" s="655" t="n"/>
-      <c r="D12" s="655" t="n"/>
-      <c r="E12" s="655" t="n"/>
-      <c r="F12" s="655" t="n"/>
-      <c r="G12" s="655" t="n"/>
-      <c r="H12" s="655" t="n"/>
+      <c r="A12" s="665" t="n"/>
+      <c r="B12" s="665" t="n"/>
+      <c r="C12" s="665" t="n"/>
+      <c r="D12" s="665" t="n"/>
+      <c r="E12" s="665" t="n"/>
+      <c r="F12" s="665" t="n"/>
+      <c r="G12" s="665" t="n"/>
+      <c r="H12" s="665" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="655" t="n"/>
-      <c r="B13" s="655" t="n"/>
-      <c r="C13" s="655" t="n"/>
-      <c r="D13" s="655" t="n"/>
-      <c r="E13" s="655" t="n"/>
-      <c r="F13" s="655" t="n"/>
-      <c r="G13" s="655" t="n"/>
-      <c r="H13" s="655" t="n"/>
+      <c r="A13" s="665" t="n"/>
+      <c r="B13" s="665" t="n"/>
+      <c r="C13" s="665" t="n"/>
+      <c r="D13" s="665" t="n"/>
+      <c r="E13" s="665" t="n"/>
+      <c r="F13" s="665" t="n"/>
+      <c r="G13" s="665" t="n"/>
+      <c r="H13" s="665" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="655" t="n"/>
-      <c r="B14" s="655" t="n"/>
-      <c r="C14" s="655" t="n"/>
-      <c r="D14" s="655" t="n"/>
-      <c r="E14" s="655" t="n"/>
-      <c r="F14" s="655" t="n"/>
-      <c r="G14" s="655" t="n"/>
-      <c r="H14" s="655" t="n"/>
+      <c r="A14" s="665" t="n"/>
+      <c r="B14" s="665" t="n"/>
+      <c r="C14" s="665" t="n"/>
+      <c r="D14" s="665" t="n"/>
+      <c r="E14" s="665" t="n"/>
+      <c r="F14" s="665" t="n"/>
+      <c r="G14" s="665" t="n"/>
+      <c r="H14" s="665" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="655" t="n"/>
-      <c r="B15" s="655" t="n"/>
-      <c r="C15" s="655" t="n"/>
-      <c r="D15" s="655" t="n"/>
-      <c r="E15" s="655" t="n"/>
-      <c r="F15" s="655" t="n"/>
-      <c r="G15" s="655" t="n"/>
-      <c r="H15" s="655" t="n"/>
+      <c r="A15" s="665" t="n"/>
+      <c r="B15" s="665" t="n"/>
+      <c r="C15" s="665" t="n"/>
+      <c r="D15" s="665" t="n"/>
+      <c r="E15" s="665" t="n"/>
+      <c r="F15" s="665" t="n"/>
+      <c r="G15" s="665" t="n"/>
+      <c r="H15" s="665" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="655" t="n"/>
-      <c r="B16" s="655" t="n"/>
-      <c r="C16" s="655" t="n"/>
-      <c r="D16" s="655" t="n"/>
-      <c r="E16" s="655" t="n"/>
-      <c r="F16" s="655" t="n"/>
-      <c r="G16" s="655" t="n"/>
-      <c r="H16" s="655" t="n"/>
+      <c r="A16" s="665" t="n"/>
+      <c r="B16" s="665" t="n"/>
+      <c r="C16" s="665" t="n"/>
+      <c r="D16" s="665" t="n"/>
+      <c r="E16" s="665" t="n"/>
+      <c r="F16" s="665" t="n"/>
+      <c r="G16" s="665" t="n"/>
+      <c r="H16" s="665" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="655" t="n"/>
-      <c r="B17" s="655" t="n"/>
-      <c r="C17" s="655" t="n"/>
-      <c r="D17" s="655" t="n"/>
-      <c r="E17" s="655" t="n"/>
-      <c r="F17" s="655" t="n"/>
-      <c r="G17" s="655" t="n"/>
-      <c r="H17" s="655" t="n"/>
+      <c r="A17" s="665" t="n"/>
+      <c r="B17" s="665" t="n"/>
+      <c r="C17" s="665" t="n"/>
+      <c r="D17" s="665" t="n"/>
+      <c r="E17" s="665" t="n"/>
+      <c r="F17" s="665" t="n"/>
+      <c r="G17" s="665" t="n"/>
+      <c r="H17" s="665" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="655" t="n"/>
-      <c r="B18" s="655" t="n"/>
-      <c r="C18" s="655" t="n"/>
-      <c r="D18" s="655" t="n"/>
-      <c r="E18" s="655" t="n"/>
-      <c r="F18" s="655" t="n"/>
-      <c r="G18" s="655" t="n"/>
-      <c r="H18" s="655" t="n"/>
+      <c r="A18" s="665" t="n"/>
+      <c r="B18" s="665" t="n"/>
+      <c r="C18" s="665" t="n"/>
+      <c r="D18" s="665" t="n"/>
+      <c r="E18" s="665" t="n"/>
+      <c r="F18" s="665" t="n"/>
+      <c r="G18" s="665" t="n"/>
+      <c r="H18" s="665" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="655" t="n"/>
-      <c r="B19" s="655" t="n"/>
-      <c r="C19" s="655" t="n"/>
-      <c r="D19" s="655" t="n"/>
-      <c r="E19" s="655" t="n"/>
-      <c r="F19" s="655" t="n"/>
-      <c r="G19" s="655" t="n"/>
-      <c r="H19" s="655" t="n"/>
+      <c r="A19" s="665" t="n"/>
+      <c r="B19" s="665" t="n"/>
+      <c r="C19" s="665" t="n"/>
+      <c r="D19" s="665" t="n"/>
+      <c r="E19" s="665" t="n"/>
+      <c r="F19" s="665" t="n"/>
+      <c r="G19" s="665" t="n"/>
+      <c r="H19" s="665" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="655" t="n"/>
-      <c r="B20" s="655" t="n"/>
-      <c r="C20" s="655" t="n"/>
-      <c r="D20" s="655" t="n"/>
-      <c r="E20" s="655" t="n"/>
-      <c r="F20" s="655" t="n"/>
-      <c r="G20" s="655" t="n"/>
-      <c r="H20" s="655" t="n"/>
+      <c r="A20" s="665" t="n"/>
+      <c r="B20" s="665" t="n"/>
+      <c r="C20" s="665" t="n"/>
+      <c r="D20" s="665" t="n"/>
+      <c r="E20" s="665" t="n"/>
+      <c r="F20" s="665" t="n"/>
+      <c r="G20" s="665" t="n"/>
+      <c r="H20" s="665" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="655" t="n"/>
-      <c r="B21" s="655" t="n"/>
-      <c r="C21" s="655" t="n"/>
-      <c r="D21" s="655" t="n"/>
-      <c r="E21" s="655" t="n"/>
-      <c r="F21" s="655" t="n"/>
-      <c r="G21" s="655" t="n"/>
-      <c r="H21" s="655" t="n"/>
+      <c r="A21" s="665" t="n"/>
+      <c r="B21" s="665" t="n"/>
+      <c r="C21" s="665" t="n"/>
+      <c r="D21" s="665" t="n"/>
+      <c r="E21" s="665" t="n"/>
+      <c r="F21" s="665" t="n"/>
+      <c r="G21" s="665" t="n"/>
+      <c r="H21" s="665" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="655" t="n"/>
-      <c r="B22" s="655" t="n"/>
-      <c r="C22" s="655" t="n"/>
-      <c r="D22" s="655" t="n"/>
-      <c r="E22" s="655" t="n"/>
-      <c r="F22" s="655" t="n"/>
-      <c r="G22" s="655" t="n"/>
-      <c r="H22" s="655" t="n"/>
+      <c r="A22" s="665" t="n"/>
+      <c r="B22" s="665" t="n"/>
+      <c r="C22" s="665" t="n"/>
+      <c r="D22" s="665" t="n"/>
+      <c r="E22" s="665" t="n"/>
+      <c r="F22" s="665" t="n"/>
+      <c r="G22" s="665" t="n"/>
+      <c r="H22" s="665" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="655" t="n"/>
-      <c r="B23" s="655" t="n"/>
-      <c r="C23" s="655" t="n"/>
-      <c r="D23" s="655" t="n"/>
-      <c r="E23" s="655" t="n"/>
-      <c r="F23" s="655" t="n"/>
-      <c r="G23" s="655" t="n"/>
-      <c r="H23" s="655" t="n"/>
+      <c r="A23" s="665" t="n"/>
+      <c r="B23" s="665" t="n"/>
+      <c r="C23" s="665" t="n"/>
+      <c r="D23" s="665" t="n"/>
+      <c r="E23" s="665" t="n"/>
+      <c r="F23" s="665" t="n"/>
+      <c r="G23" s="665" t="n"/>
+      <c r="H23" s="665" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="655" t="n"/>
-      <c r="B24" s="655" t="n"/>
-      <c r="C24" s="655" t="n"/>
-      <c r="D24" s="655" t="n"/>
-      <c r="E24" s="655" t="n"/>
-      <c r="F24" s="655" t="n"/>
-      <c r="G24" s="655" t="n"/>
-      <c r="H24" s="655" t="n"/>
+      <c r="A24" s="665" t="n"/>
+      <c r="B24" s="665" t="n"/>
+      <c r="C24" s="665" t="n"/>
+      <c r="D24" s="665" t="n"/>
+      <c r="E24" s="665" t="n"/>
+      <c r="F24" s="665" t="n"/>
+      <c r="G24" s="665" t="n"/>
+      <c r="H24" s="665" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="655" t="n"/>
-      <c r="B25" s="655" t="n"/>
-      <c r="C25" s="655" t="n"/>
-      <c r="D25" s="655" t="n"/>
-      <c r="E25" s="655" t="n"/>
-      <c r="F25" s="655" t="n"/>
-      <c r="G25" s="655" t="n"/>
-      <c r="H25" s="655" t="n"/>
+      <c r="A25" s="665" t="n"/>
+      <c r="B25" s="665" t="n"/>
+      <c r="C25" s="665" t="n"/>
+      <c r="D25" s="665" t="n"/>
+      <c r="E25" s="665" t="n"/>
+      <c r="F25" s="665" t="n"/>
+      <c r="G25" s="665" t="n"/>
+      <c r="H25" s="665" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="655" t="n"/>
-      <c r="B26" s="655" t="n"/>
-      <c r="C26" s="655" t="n"/>
-      <c r="D26" s="655" t="n"/>
-      <c r="E26" s="655" t="n"/>
-      <c r="F26" s="655" t="n"/>
-      <c r="G26" s="655" t="n"/>
-      <c r="H26" s="655" t="n"/>
+      <c r="A26" s="665" t="n"/>
+      <c r="B26" s="665" t="n"/>
+      <c r="C26" s="665" t="n"/>
+      <c r="D26" s="665" t="n"/>
+      <c r="E26" s="665" t="n"/>
+      <c r="F26" s="665" t="n"/>
+      <c r="G26" s="665" t="n"/>
+      <c r="H26" s="665" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="655" t="n"/>
-      <c r="B27" s="655" t="n"/>
-      <c r="C27" s="655" t="n"/>
-      <c r="D27" s="655" t="n"/>
-      <c r="E27" s="655" t="n"/>
-      <c r="F27" s="655" t="n"/>
-      <c r="G27" s="655" t="n"/>
-      <c r="H27" s="655" t="n"/>
+      <c r="A27" s="665" t="n"/>
+      <c r="B27" s="665" t="n"/>
+      <c r="C27" s="665" t="n"/>
+      <c r="D27" s="665" t="n"/>
+      <c r="E27" s="665" t="n"/>
+      <c r="F27" s="665" t="n"/>
+      <c r="G27" s="665" t="n"/>
+      <c r="H27" s="665" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="655" t="n"/>
-      <c r="B28" s="655" t="n"/>
-      <c r="C28" s="655" t="n"/>
-      <c r="D28" s="655" t="n"/>
-      <c r="E28" s="655" t="n"/>
-      <c r="F28" s="655" t="n"/>
-      <c r="G28" s="655" t="n"/>
-      <c r="H28" s="655" t="n"/>
+      <c r="A28" s="665" t="n"/>
+      <c r="B28" s="665" t="n"/>
+      <c r="C28" s="665" t="n"/>
+      <c r="D28" s="665" t="n"/>
+      <c r="E28" s="665" t="n"/>
+      <c r="F28" s="665" t="n"/>
+      <c r="G28" s="665" t="n"/>
+      <c r="H28" s="665" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="655" t="n"/>
-      <c r="B29" s="655" t="n"/>
-      <c r="C29" s="655" t="n"/>
-      <c r="D29" s="655" t="n"/>
-      <c r="E29" s="655" t="n"/>
-      <c r="F29" s="655" t="n"/>
-      <c r="G29" s="655" t="n"/>
-      <c r="H29" s="655" t="n"/>
+      <c r="A29" s="665" t="n"/>
+      <c r="B29" s="665" t="n"/>
+      <c r="C29" s="665" t="n"/>
+      <c r="D29" s="665" t="n"/>
+      <c r="E29" s="665" t="n"/>
+      <c r="F29" s="665" t="n"/>
+      <c r="G29" s="665" t="n"/>
+      <c r="H29" s="665" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="655" t="n"/>
-      <c r="B30" s="655" t="n"/>
-      <c r="C30" s="655" t="n"/>
-      <c r="D30" s="655" t="n"/>
-      <c r="E30" s="655" t="n"/>
-      <c r="F30" s="655" t="n"/>
-      <c r="G30" s="655" t="n"/>
-      <c r="H30" s="655" t="n"/>
+      <c r="A30" s="665" t="n"/>
+      <c r="B30" s="665" t="n"/>
+      <c r="C30" s="665" t="n"/>
+      <c r="D30" s="665" t="n"/>
+      <c r="E30" s="665" t="n"/>
+      <c r="F30" s="665" t="n"/>
+      <c r="G30" s="665" t="n"/>
+      <c r="H30" s="665" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="655" t="n"/>
-      <c r="B31" s="655" t="n"/>
-      <c r="C31" s="655" t="n"/>
-      <c r="D31" s="655" t="n"/>
-      <c r="E31" s="655" t="n"/>
-      <c r="F31" s="655" t="n"/>
-      <c r="G31" s="655" t="n"/>
-      <c r="H31" s="655" t="n"/>
+      <c r="A31" s="665" t="n"/>
+      <c r="B31" s="665" t="n"/>
+      <c r="C31" s="665" t="n"/>
+      <c r="D31" s="665" t="n"/>
+      <c r="E31" s="665" t="n"/>
+      <c r="F31" s="665" t="n"/>
+      <c r="G31" s="665" t="n"/>
+      <c r="H31" s="665" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="655" t="n"/>
-      <c r="B32" s="655" t="n"/>
-      <c r="C32" s="655" t="n"/>
-      <c r="D32" s="655" t="n"/>
-      <c r="E32" s="655" t="n"/>
-      <c r="F32" s="655" t="n"/>
-      <c r="G32" s="655" t="n"/>
-      <c r="H32" s="655" t="n"/>
+      <c r="A32" s="665" t="n"/>
+      <c r="B32" s="665" t="n"/>
+      <c r="C32" s="665" t="n"/>
+      <c r="D32" s="665" t="n"/>
+      <c r="E32" s="665" t="n"/>
+      <c r="F32" s="665" t="n"/>
+      <c r="G32" s="665" t="n"/>
+      <c r="H32" s="665" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="655" t="n"/>
-      <c r="B33" s="655" t="n"/>
-      <c r="C33" s="655" t="n"/>
-      <c r="D33" s="655" t="n"/>
-      <c r="E33" s="655" t="n"/>
-      <c r="F33" s="655" t="n"/>
-      <c r="G33" s="655" t="n"/>
-      <c r="H33" s="655" t="n"/>
+      <c r="A33" s="665" t="n"/>
+      <c r="B33" s="665" t="n"/>
+      <c r="C33" s="665" t="n"/>
+      <c r="D33" s="665" t="n"/>
+      <c r="E33" s="665" t="n"/>
+      <c r="F33" s="665" t="n"/>
+      <c r="G33" s="665" t="n"/>
+      <c r="H33" s="665" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="655" t="n"/>
-      <c r="B34" s="655" t="n"/>
-      <c r="C34" s="655" t="n"/>
-      <c r="D34" s="655" t="n"/>
-      <c r="E34" s="655" t="n"/>
-      <c r="F34" s="655" t="n"/>
-      <c r="G34" s="655" t="n"/>
-      <c r="H34" s="655" t="n"/>
+      <c r="A34" s="665" t="n"/>
+      <c r="B34" s="665" t="n"/>
+      <c r="C34" s="665" t="n"/>
+      <c r="D34" s="665" t="n"/>
+      <c r="E34" s="665" t="n"/>
+      <c r="F34" s="665" t="n"/>
+      <c r="G34" s="665" t="n"/>
+      <c r="H34" s="665" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="655" t="n"/>
-      <c r="B35" s="655" t="n"/>
-      <c r="C35" s="655" t="n"/>
-      <c r="D35" s="655" t="n"/>
-      <c r="E35" s="655" t="n"/>
-      <c r="F35" s="655" t="n"/>
-      <c r="G35" s="655" t="n"/>
-      <c r="H35" s="655" t="n"/>
+      <c r="A35" s="665" t="n"/>
+      <c r="B35" s="665" t="n"/>
+      <c r="C35" s="665" t="n"/>
+      <c r="D35" s="665" t="n"/>
+      <c r="E35" s="665" t="n"/>
+      <c r="F35" s="665" t="n"/>
+      <c r="G35" s="665" t="n"/>
+      <c r="H35" s="665" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="655" t="n"/>
-      <c r="B36" s="655" t="n"/>
-      <c r="C36" s="655" t="n"/>
-      <c r="D36" s="655" t="n"/>
-      <c r="E36" s="655" t="n"/>
-      <c r="F36" s="655" t="n"/>
-      <c r="G36" s="655" t="n"/>
-      <c r="H36" s="655" t="n"/>
+      <c r="A36" s="665" t="n"/>
+      <c r="B36" s="665" t="n"/>
+      <c r="C36" s="665" t="n"/>
+      <c r="D36" s="665" t="n"/>
+      <c r="E36" s="665" t="n"/>
+      <c r="F36" s="665" t="n"/>
+      <c r="G36" s="665" t="n"/>
+      <c r="H36" s="665" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="655" t="n"/>
-      <c r="B37" s="655" t="n"/>
-      <c r="C37" s="655" t="n"/>
-      <c r="D37" s="655" t="n"/>
-      <c r="E37" s="655" t="n"/>
-      <c r="F37" s="655" t="n"/>
-      <c r="G37" s="655" t="n"/>
-      <c r="H37" s="655" t="n"/>
+      <c r="A37" s="665" t="n"/>
+      <c r="B37" s="665" t="n"/>
+      <c r="C37" s="665" t="n"/>
+      <c r="D37" s="665" t="n"/>
+      <c r="E37" s="665" t="n"/>
+      <c r="F37" s="665" t="n"/>
+      <c r="G37" s="665" t="n"/>
+      <c r="H37" s="665" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="655" t="n"/>
-      <c r="B38" s="655" t="n"/>
-      <c r="C38" s="655" t="n"/>
-      <c r="D38" s="655" t="n"/>
-      <c r="E38" s="655" t="n"/>
-      <c r="F38" s="655" t="n"/>
-      <c r="G38" s="655" t="n"/>
-      <c r="H38" s="655" t="n"/>
+      <c r="A38" s="665" t="n"/>
+      <c r="B38" s="665" t="n"/>
+      <c r="C38" s="665" t="n"/>
+      <c r="D38" s="665" t="n"/>
+      <c r="E38" s="665" t="n"/>
+      <c r="F38" s="665" t="n"/>
+      <c r="G38" s="665" t="n"/>
+      <c r="H38" s="665" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="655" t="n"/>
-      <c r="B39" s="655" t="n"/>
-      <c r="C39" s="655" t="n"/>
-      <c r="D39" s="655" t="n"/>
-      <c r="E39" s="655" t="n"/>
-      <c r="F39" s="655" t="n"/>
-      <c r="G39" s="655" t="n"/>
-      <c r="H39" s="655" t="n"/>
+      <c r="A39" s="665" t="n"/>
+      <c r="B39" s="665" t="n"/>
+      <c r="C39" s="665" t="n"/>
+      <c r="D39" s="665" t="n"/>
+      <c r="E39" s="665" t="n"/>
+      <c r="F39" s="665" t="n"/>
+      <c r="G39" s="665" t="n"/>
+      <c r="H39" s="665" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="655" t="n"/>
-      <c r="B40" s="655" t="n"/>
-      <c r="C40" s="655" t="n"/>
-      <c r="D40" s="655" t="n"/>
-      <c r="E40" s="655" t="n"/>
-      <c r="F40" s="655" t="n"/>
-      <c r="G40" s="655" t="n"/>
-      <c r="H40" s="655" t="n"/>
+      <c r="A40" s="665" t="n"/>
+      <c r="B40" s="665" t="n"/>
+      <c r="C40" s="665" t="n"/>
+      <c r="D40" s="665" t="n"/>
+      <c r="E40" s="665" t="n"/>
+      <c r="F40" s="665" t="n"/>
+      <c r="G40" s="665" t="n"/>
+      <c r="H40" s="665" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
     </row>
@@ -3073,504 +3103,504 @@
       <c r="J2" s="3" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="656" t="inlineStr">
+      <c r="A3" s="666" t="inlineStr">
         <is>
           <t>15.07.2026</t>
         </is>
       </c>
-      <c r="B3" s="656" t="inlineStr">
+      <c r="B3" s="666" t="inlineStr">
         <is>
           <t>4039-95</t>
         </is>
       </c>
-      <c r="C3" s="656" t="inlineStr">
+      <c r="C3" s="666" t="inlineStr">
         <is>
           <t>1.0026-2X2500X1250</t>
         </is>
       </c>
-      <c r="D3" s="656" t="n">
+      <c r="D3" s="666" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="656" t="inlineStr">
+      <c r="E3" s="666" t="inlineStr">
         <is>
           <t>00:04:03</t>
         </is>
       </c>
-      <c r="F3" s="656" t="n"/>
-      <c r="G3" s="656" t="n"/>
-      <c r="H3" s="656" t="n"/>
+      <c r="F3" s="666" t="n"/>
+      <c r="G3" s="666" t="n"/>
+      <c r="H3" s="666" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="656" t="n"/>
-      <c r="B4" s="656" t="inlineStr">
+      <c r="A4" s="666" t="n"/>
+      <c r="B4" s="666" t="inlineStr">
         <is>
           <t>4039-96</t>
         </is>
       </c>
-      <c r="C4" s="656" t="inlineStr">
+      <c r="C4" s="666" t="inlineStr">
         <is>
           <t>3.3535-2X2500X1250</t>
         </is>
       </c>
-      <c r="D4" s="656" t="n">
+      <c r="D4" s="666" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="656" t="inlineStr">
+      <c r="E4" s="666" t="inlineStr">
         <is>
           <t>00:03:09</t>
         </is>
       </c>
-      <c r="F4" s="656" t="n"/>
-      <c r="G4" s="656" t="n"/>
-      <c r="H4" s="656" t="n"/>
+      <c r="F4" s="666" t="n"/>
+      <c r="G4" s="666" t="n"/>
+      <c r="H4" s="666" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="656" t="n"/>
-      <c r="B5" s="656" t="inlineStr">
+      <c r="A5" s="666" t="n"/>
+      <c r="B5" s="666" t="inlineStr">
         <is>
           <t>4039-97</t>
         </is>
       </c>
-      <c r="C5" s="656" t="inlineStr">
+      <c r="C5" s="666" t="inlineStr">
         <is>
           <t>-----</t>
         </is>
       </c>
-      <c r="D5" s="656" t="n">
+      <c r="D5" s="666" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="656" t="inlineStr">
+      <c r="E5" s="666" t="inlineStr">
         <is>
           <t>00:03:56</t>
         </is>
       </c>
-      <c r="F5" s="656" t="n"/>
-      <c r="G5" s="656" t="n"/>
-      <c r="H5" s="656" t="n"/>
+      <c r="F5" s="666" t="n"/>
+      <c r="G5" s="666" t="n"/>
+      <c r="H5" s="666" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="656" t="n"/>
-      <c r="B6" s="656" t="n"/>
-      <c r="C6" s="656" t="n"/>
-      <c r="D6" s="656" t="n"/>
-      <c r="E6" s="656" t="n"/>
-      <c r="F6" s="656" t="n"/>
-      <c r="G6" s="656" t="n"/>
-      <c r="H6" s="656" t="n"/>
+      <c r="A6" s="666" t="n"/>
+      <c r="B6" s="666" t="n"/>
+      <c r="C6" s="666" t="n"/>
+      <c r="D6" s="666" t="n"/>
+      <c r="E6" s="666" t="n"/>
+      <c r="F6" s="666" t="n"/>
+      <c r="G6" s="666" t="n"/>
+      <c r="H6" s="666" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="656" t="n"/>
-      <c r="B7" s="656" t="n"/>
-      <c r="C7" s="656" t="n"/>
-      <c r="D7" s="656" t="n"/>
-      <c r="E7" s="656" t="n"/>
-      <c r="F7" s="656" t="n"/>
-      <c r="G7" s="656" t="n"/>
-      <c r="H7" s="656" t="n"/>
+      <c r="A7" s="666" t="n"/>
+      <c r="B7" s="666" t="n"/>
+      <c r="C7" s="666" t="n"/>
+      <c r="D7" s="666" t="n"/>
+      <c r="E7" s="666" t="n"/>
+      <c r="F7" s="666" t="n"/>
+      <c r="G7" s="666" t="n"/>
+      <c r="H7" s="666" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="656" t="n"/>
-      <c r="B8" s="656" t="n"/>
-      <c r="C8" s="656" t="n"/>
-      <c r="D8" s="656" t="n"/>
-      <c r="E8" s="656" t="n"/>
-      <c r="F8" s="656" t="n"/>
-      <c r="G8" s="656" t="n"/>
-      <c r="H8" s="656" t="n"/>
+      <c r="A8" s="666" t="n"/>
+      <c r="B8" s="666" t="n"/>
+      <c r="C8" s="666" t="n"/>
+      <c r="D8" s="666" t="n"/>
+      <c r="E8" s="666" t="n"/>
+      <c r="F8" s="666" t="n"/>
+      <c r="G8" s="666" t="n"/>
+      <c r="H8" s="666" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="656" t="n"/>
-      <c r="B9" s="656" t="n"/>
-      <c r="C9" s="656" t="n"/>
-      <c r="D9" s="656" t="n"/>
-      <c r="E9" s="656" t="n"/>
-      <c r="F9" s="656" t="n"/>
-      <c r="G9" s="656" t="n"/>
-      <c r="H9" s="656" t="n"/>
+      <c r="A9" s="666" t="n"/>
+      <c r="B9" s="666" t="n"/>
+      <c r="C9" s="666" t="n"/>
+      <c r="D9" s="666" t="n"/>
+      <c r="E9" s="666" t="n"/>
+      <c r="F9" s="666" t="n"/>
+      <c r="G9" s="666" t="n"/>
+      <c r="H9" s="666" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="656" t="n"/>
-      <c r="B10" s="656" t="n"/>
-      <c r="C10" s="656" t="n"/>
-      <c r="D10" s="656" t="n"/>
-      <c r="E10" s="656" t="n"/>
-      <c r="F10" s="656" t="n"/>
-      <c r="G10" s="656" t="n"/>
-      <c r="H10" s="656" t="n"/>
+      <c r="A10" s="666" t="n"/>
+      <c r="B10" s="666" t="n"/>
+      <c r="C10" s="666" t="n"/>
+      <c r="D10" s="666" t="n"/>
+      <c r="E10" s="666" t="n"/>
+      <c r="F10" s="666" t="n"/>
+      <c r="G10" s="666" t="n"/>
+      <c r="H10" s="666" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="656" t="n"/>
-      <c r="B11" s="656" t="n"/>
-      <c r="C11" s="656" t="n"/>
-      <c r="D11" s="656" t="n"/>
-      <c r="E11" s="656" t="n"/>
-      <c r="F11" s="656" t="n"/>
-      <c r="G11" s="656" t="n"/>
-      <c r="H11" s="656" t="n"/>
+      <c r="A11" s="666" t="n"/>
+      <c r="B11" s="666" t="n"/>
+      <c r="C11" s="666" t="n"/>
+      <c r="D11" s="666" t="n"/>
+      <c r="E11" s="666" t="n"/>
+      <c r="F11" s="666" t="n"/>
+      <c r="G11" s="666" t="n"/>
+      <c r="H11" s="666" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="656" t="n"/>
-      <c r="B12" s="656" t="n"/>
-      <c r="C12" s="656" t="n"/>
-      <c r="D12" s="656" t="n"/>
-      <c r="E12" s="656" t="n"/>
-      <c r="F12" s="656" t="n"/>
-      <c r="G12" s="656" t="n"/>
-      <c r="H12" s="656" t="n"/>
+      <c r="A12" s="666" t="n"/>
+      <c r="B12" s="666" t="n"/>
+      <c r="C12" s="666" t="n"/>
+      <c r="D12" s="666" t="n"/>
+      <c r="E12" s="666" t="n"/>
+      <c r="F12" s="666" t="n"/>
+      <c r="G12" s="666" t="n"/>
+      <c r="H12" s="666" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="656" t="n"/>
-      <c r="B13" s="656" t="n"/>
-      <c r="C13" s="656" t="n"/>
-      <c r="D13" s="656" t="n"/>
-      <c r="E13" s="656" t="n"/>
-      <c r="F13" s="656" t="n"/>
-      <c r="G13" s="656" t="n"/>
-      <c r="H13" s="656" t="n"/>
+      <c r="A13" s="666" t="n"/>
+      <c r="B13" s="666" t="n"/>
+      <c r="C13" s="666" t="n"/>
+      <c r="D13" s="666" t="n"/>
+      <c r="E13" s="666" t="n"/>
+      <c r="F13" s="666" t="n"/>
+      <c r="G13" s="666" t="n"/>
+      <c r="H13" s="666" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="656" t="n"/>
-      <c r="B14" s="656" t="n"/>
-      <c r="C14" s="656" t="n"/>
-      <c r="D14" s="656" t="n"/>
-      <c r="E14" s="656" t="n"/>
-      <c r="F14" s="656" t="n"/>
-      <c r="G14" s="656" t="n"/>
-      <c r="H14" s="656" t="n"/>
+      <c r="A14" s="666" t="n"/>
+      <c r="B14" s="666" t="n"/>
+      <c r="C14" s="666" t="n"/>
+      <c r="D14" s="666" t="n"/>
+      <c r="E14" s="666" t="n"/>
+      <c r="F14" s="666" t="n"/>
+      <c r="G14" s="666" t="n"/>
+      <c r="H14" s="666" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="656" t="n"/>
-      <c r="B15" s="656" t="n"/>
-      <c r="C15" s="656" t="n"/>
-      <c r="D15" s="656" t="n"/>
-      <c r="E15" s="656" t="n"/>
-      <c r="F15" s="656" t="n"/>
-      <c r="G15" s="656" t="n"/>
-      <c r="H15" s="656" t="n"/>
+      <c r="A15" s="666" t="n"/>
+      <c r="B15" s="666" t="n"/>
+      <c r="C15" s="666" t="n"/>
+      <c r="D15" s="666" t="n"/>
+      <c r="E15" s="666" t="n"/>
+      <c r="F15" s="666" t="n"/>
+      <c r="G15" s="666" t="n"/>
+      <c r="H15" s="666" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="656" t="n"/>
-      <c r="B16" s="656" t="n"/>
-      <c r="C16" s="656" t="n"/>
-      <c r="D16" s="656" t="n"/>
-      <c r="E16" s="656" t="n"/>
-      <c r="F16" s="656" t="n"/>
-      <c r="G16" s="656" t="n"/>
-      <c r="H16" s="656" t="n"/>
+      <c r="A16" s="666" t="n"/>
+      <c r="B16" s="666" t="n"/>
+      <c r="C16" s="666" t="n"/>
+      <c r="D16" s="666" t="n"/>
+      <c r="E16" s="666" t="n"/>
+      <c r="F16" s="666" t="n"/>
+      <c r="G16" s="666" t="n"/>
+      <c r="H16" s="666" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="656" t="n"/>
-      <c r="B17" s="656" t="n"/>
-      <c r="C17" s="656" t="n"/>
-      <c r="D17" s="656" t="n"/>
-      <c r="E17" s="656" t="n"/>
-      <c r="F17" s="656" t="n"/>
-      <c r="G17" s="656" t="n"/>
-      <c r="H17" s="656" t="n"/>
+      <c r="A17" s="666" t="n"/>
+      <c r="B17" s="666" t="n"/>
+      <c r="C17" s="666" t="n"/>
+      <c r="D17" s="666" t="n"/>
+      <c r="E17" s="666" t="n"/>
+      <c r="F17" s="666" t="n"/>
+      <c r="G17" s="666" t="n"/>
+      <c r="H17" s="666" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="656" t="n"/>
-      <c r="B18" s="656" t="n"/>
-      <c r="C18" s="656" t="n"/>
-      <c r="D18" s="656" t="n"/>
-      <c r="E18" s="656" t="n"/>
-      <c r="F18" s="656" t="n"/>
-      <c r="G18" s="656" t="n"/>
-      <c r="H18" s="656" t="n"/>
+      <c r="A18" s="666" t="n"/>
+      <c r="B18" s="666" t="n"/>
+      <c r="C18" s="666" t="n"/>
+      <c r="D18" s="666" t="n"/>
+      <c r="E18" s="666" t="n"/>
+      <c r="F18" s="666" t="n"/>
+      <c r="G18" s="666" t="n"/>
+      <c r="H18" s="666" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="656" t="n"/>
-      <c r="B19" s="656" t="n"/>
-      <c r="C19" s="656" t="n"/>
-      <c r="D19" s="656" t="n"/>
-      <c r="E19" s="656" t="n"/>
-      <c r="F19" s="656" t="n"/>
-      <c r="G19" s="656" t="n"/>
-      <c r="H19" s="656" t="n"/>
+      <c r="A19" s="666" t="n"/>
+      <c r="B19" s="666" t="n"/>
+      <c r="C19" s="666" t="n"/>
+      <c r="D19" s="666" t="n"/>
+      <c r="E19" s="666" t="n"/>
+      <c r="F19" s="666" t="n"/>
+      <c r="G19" s="666" t="n"/>
+      <c r="H19" s="666" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="656" t="n"/>
-      <c r="B20" s="656" t="n"/>
-      <c r="C20" s="656" t="n"/>
-      <c r="D20" s="656" t="n"/>
-      <c r="E20" s="656" t="n"/>
-      <c r="F20" s="656" t="n"/>
-      <c r="G20" s="656" t="n"/>
-      <c r="H20" s="656" t="n"/>
+      <c r="A20" s="666" t="n"/>
+      <c r="B20" s="666" t="n"/>
+      <c r="C20" s="666" t="n"/>
+      <c r="D20" s="666" t="n"/>
+      <c r="E20" s="666" t="n"/>
+      <c r="F20" s="666" t="n"/>
+      <c r="G20" s="666" t="n"/>
+      <c r="H20" s="666" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="656" t="n"/>
-      <c r="B21" s="656" t="n"/>
-      <c r="C21" s="656" t="n"/>
-      <c r="D21" s="656" t="n"/>
-      <c r="E21" s="656" t="n"/>
-      <c r="F21" s="656" t="n"/>
-      <c r="G21" s="656" t="n"/>
-      <c r="H21" s="656" t="n"/>
+      <c r="A21" s="666" t="n"/>
+      <c r="B21" s="666" t="n"/>
+      <c r="C21" s="666" t="n"/>
+      <c r="D21" s="666" t="n"/>
+      <c r="E21" s="666" t="n"/>
+      <c r="F21" s="666" t="n"/>
+      <c r="G21" s="666" t="n"/>
+      <c r="H21" s="666" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="656" t="n"/>
-      <c r="B22" s="656" t="n"/>
-      <c r="C22" s="656" t="n"/>
-      <c r="D22" s="656" t="n"/>
-      <c r="E22" s="656" t="n"/>
-      <c r="F22" s="656" t="n"/>
-      <c r="G22" s="656" t="n"/>
-      <c r="H22" s="656" t="n"/>
+      <c r="A22" s="666" t="n"/>
+      <c r="B22" s="666" t="n"/>
+      <c r="C22" s="666" t="n"/>
+      <c r="D22" s="666" t="n"/>
+      <c r="E22" s="666" t="n"/>
+      <c r="F22" s="666" t="n"/>
+      <c r="G22" s="666" t="n"/>
+      <c r="H22" s="666" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="656" t="n"/>
-      <c r="B23" s="656" t="n"/>
-      <c r="C23" s="656" t="n"/>
-      <c r="D23" s="656" t="n"/>
-      <c r="E23" s="656" t="n"/>
-      <c r="F23" s="656" t="n"/>
-      <c r="G23" s="656" t="n"/>
-      <c r="H23" s="656" t="n"/>
+      <c r="A23" s="666" t="n"/>
+      <c r="B23" s="666" t="n"/>
+      <c r="C23" s="666" t="n"/>
+      <c r="D23" s="666" t="n"/>
+      <c r="E23" s="666" t="n"/>
+      <c r="F23" s="666" t="n"/>
+      <c r="G23" s="666" t="n"/>
+      <c r="H23" s="666" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="656" t="n"/>
-      <c r="B24" s="656" t="n"/>
-      <c r="C24" s="656" t="n"/>
-      <c r="D24" s="656" t="n"/>
-      <c r="E24" s="656" t="n"/>
-      <c r="F24" s="656" t="n"/>
-      <c r="G24" s="656" t="n"/>
-      <c r="H24" s="656" t="n"/>
+      <c r="A24" s="666" t="n"/>
+      <c r="B24" s="666" t="n"/>
+      <c r="C24" s="666" t="n"/>
+      <c r="D24" s="666" t="n"/>
+      <c r="E24" s="666" t="n"/>
+      <c r="F24" s="666" t="n"/>
+      <c r="G24" s="666" t="n"/>
+      <c r="H24" s="666" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="656" t="n"/>
-      <c r="B25" s="656" t="n"/>
-      <c r="C25" s="656" t="n"/>
-      <c r="D25" s="656" t="n"/>
-      <c r="E25" s="656" t="n"/>
-      <c r="F25" s="656" t="n"/>
-      <c r="G25" s="656" t="n"/>
-      <c r="H25" s="656" t="n"/>
+      <c r="A25" s="666" t="n"/>
+      <c r="B25" s="666" t="n"/>
+      <c r="C25" s="666" t="n"/>
+      <c r="D25" s="666" t="n"/>
+      <c r="E25" s="666" t="n"/>
+      <c r="F25" s="666" t="n"/>
+      <c r="G25" s="666" t="n"/>
+      <c r="H25" s="666" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="656" t="n"/>
-      <c r="B26" s="656" t="n"/>
-      <c r="C26" s="656" t="n"/>
-      <c r="D26" s="656" t="n"/>
-      <c r="E26" s="656" t="n"/>
-      <c r="F26" s="656" t="n"/>
-      <c r="G26" s="656" t="n"/>
-      <c r="H26" s="656" t="n"/>
+      <c r="A26" s="666" t="n"/>
+      <c r="B26" s="666" t="n"/>
+      <c r="C26" s="666" t="n"/>
+      <c r="D26" s="666" t="n"/>
+      <c r="E26" s="666" t="n"/>
+      <c r="F26" s="666" t="n"/>
+      <c r="G26" s="666" t="n"/>
+      <c r="H26" s="666" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="656" t="n"/>
-      <c r="B27" s="656" t="n"/>
-      <c r="C27" s="656" t="n"/>
-      <c r="D27" s="656" t="n"/>
-      <c r="E27" s="656" t="n"/>
-      <c r="F27" s="656" t="n"/>
-      <c r="G27" s="656" t="n"/>
-      <c r="H27" s="656" t="n"/>
+      <c r="A27" s="666" t="n"/>
+      <c r="B27" s="666" t="n"/>
+      <c r="C27" s="666" t="n"/>
+      <c r="D27" s="666" t="n"/>
+      <c r="E27" s="666" t="n"/>
+      <c r="F27" s="666" t="n"/>
+      <c r="G27" s="666" t="n"/>
+      <c r="H27" s="666" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="656" t="n"/>
-      <c r="B28" s="656" t="n"/>
-      <c r="C28" s="656" t="n"/>
-      <c r="D28" s="656" t="n"/>
-      <c r="E28" s="656" t="n"/>
-      <c r="F28" s="656" t="n"/>
-      <c r="G28" s="656" t="n"/>
-      <c r="H28" s="656" t="n"/>
+      <c r="A28" s="666" t="n"/>
+      <c r="B28" s="666" t="n"/>
+      <c r="C28" s="666" t="n"/>
+      <c r="D28" s="666" t="n"/>
+      <c r="E28" s="666" t="n"/>
+      <c r="F28" s="666" t="n"/>
+      <c r="G28" s="666" t="n"/>
+      <c r="H28" s="666" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="656" t="n"/>
-      <c r="B29" s="656" t="n"/>
-      <c r="C29" s="656" t="n"/>
-      <c r="D29" s="656" t="n"/>
-      <c r="E29" s="656" t="n"/>
-      <c r="F29" s="656" t="n"/>
-      <c r="G29" s="656" t="n"/>
-      <c r="H29" s="656" t="n"/>
+      <c r="A29" s="666" t="n"/>
+      <c r="B29" s="666" t="n"/>
+      <c r="C29" s="666" t="n"/>
+      <c r="D29" s="666" t="n"/>
+      <c r="E29" s="666" t="n"/>
+      <c r="F29" s="666" t="n"/>
+      <c r="G29" s="666" t="n"/>
+      <c r="H29" s="666" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="656" t="n"/>
-      <c r="B30" s="656" t="n"/>
-      <c r="C30" s="656" t="n"/>
-      <c r="D30" s="656" t="n"/>
-      <c r="E30" s="656" t="n"/>
-      <c r="F30" s="656" t="n"/>
-      <c r="G30" s="656" t="n"/>
-      <c r="H30" s="656" t="n"/>
+      <c r="A30" s="666" t="n"/>
+      <c r="B30" s="666" t="n"/>
+      <c r="C30" s="666" t="n"/>
+      <c r="D30" s="666" t="n"/>
+      <c r="E30" s="666" t="n"/>
+      <c r="F30" s="666" t="n"/>
+      <c r="G30" s="666" t="n"/>
+      <c r="H30" s="666" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="656" t="n"/>
-      <c r="B31" s="656" t="n"/>
-      <c r="C31" s="656" t="n"/>
-      <c r="D31" s="656" t="n"/>
-      <c r="E31" s="656" t="n"/>
-      <c r="F31" s="656" t="n"/>
-      <c r="G31" s="656" t="n"/>
-      <c r="H31" s="656" t="n"/>
+      <c r="A31" s="666" t="n"/>
+      <c r="B31" s="666" t="n"/>
+      <c r="C31" s="666" t="n"/>
+      <c r="D31" s="666" t="n"/>
+      <c r="E31" s="666" t="n"/>
+      <c r="F31" s="666" t="n"/>
+      <c r="G31" s="666" t="n"/>
+      <c r="H31" s="666" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="656" t="n"/>
-      <c r="B32" s="656" t="n"/>
-      <c r="C32" s="656" t="n"/>
-      <c r="D32" s="656" t="n"/>
-      <c r="E32" s="656" t="n"/>
-      <c r="F32" s="656" t="n"/>
-      <c r="G32" s="656" t="n"/>
-      <c r="H32" s="656" t="n"/>
+      <c r="A32" s="666" t="n"/>
+      <c r="B32" s="666" t="n"/>
+      <c r="C32" s="666" t="n"/>
+      <c r="D32" s="666" t="n"/>
+      <c r="E32" s="666" t="n"/>
+      <c r="F32" s="666" t="n"/>
+      <c r="G32" s="666" t="n"/>
+      <c r="H32" s="666" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="656" t="n"/>
-      <c r="B33" s="656" t="n"/>
-      <c r="C33" s="656" t="n"/>
-      <c r="D33" s="656" t="n"/>
-      <c r="E33" s="656" t="n"/>
-      <c r="F33" s="656" t="n"/>
-      <c r="G33" s="656" t="n"/>
-      <c r="H33" s="656" t="n"/>
+      <c r="A33" s="666" t="n"/>
+      <c r="B33" s="666" t="n"/>
+      <c r="C33" s="666" t="n"/>
+      <c r="D33" s="666" t="n"/>
+      <c r="E33" s="666" t="n"/>
+      <c r="F33" s="666" t="n"/>
+      <c r="G33" s="666" t="n"/>
+      <c r="H33" s="666" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="656" t="n"/>
-      <c r="B34" s="656" t="n"/>
-      <c r="C34" s="656" t="n"/>
-      <c r="D34" s="656" t="n"/>
-      <c r="E34" s="656" t="n"/>
-      <c r="F34" s="656" t="n"/>
-      <c r="G34" s="656" t="n"/>
-      <c r="H34" s="656" t="n"/>
+      <c r="A34" s="666" t="n"/>
+      <c r="B34" s="666" t="n"/>
+      <c r="C34" s="666" t="n"/>
+      <c r="D34" s="666" t="n"/>
+      <c r="E34" s="666" t="n"/>
+      <c r="F34" s="666" t="n"/>
+      <c r="G34" s="666" t="n"/>
+      <c r="H34" s="666" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="656" t="n"/>
-      <c r="B35" s="656" t="n"/>
-      <c r="C35" s="656" t="n"/>
-      <c r="D35" s="656" t="n"/>
-      <c r="E35" s="656" t="n"/>
-      <c r="F35" s="656" t="n"/>
-      <c r="G35" s="656" t="n"/>
-      <c r="H35" s="656" t="n"/>
+      <c r="A35" s="666" t="n"/>
+      <c r="B35" s="666" t="n"/>
+      <c r="C35" s="666" t="n"/>
+      <c r="D35" s="666" t="n"/>
+      <c r="E35" s="666" t="n"/>
+      <c r="F35" s="666" t="n"/>
+      <c r="G35" s="666" t="n"/>
+      <c r="H35" s="666" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="656" t="n"/>
-      <c r="B36" s="656" t="n"/>
-      <c r="C36" s="656" t="n"/>
-      <c r="D36" s="656" t="n"/>
-      <c r="E36" s="656" t="n"/>
-      <c r="F36" s="656" t="n"/>
-      <c r="G36" s="656" t="n"/>
-      <c r="H36" s="656" t="n"/>
+      <c r="A36" s="666" t="n"/>
+      <c r="B36" s="666" t="n"/>
+      <c r="C36" s="666" t="n"/>
+      <c r="D36" s="666" t="n"/>
+      <c r="E36" s="666" t="n"/>
+      <c r="F36" s="666" t="n"/>
+      <c r="G36" s="666" t="n"/>
+      <c r="H36" s="666" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="656" t="n"/>
-      <c r="B37" s="656" t="n"/>
-      <c r="C37" s="656" t="n"/>
-      <c r="D37" s="656" t="n"/>
-      <c r="E37" s="656" t="n"/>
-      <c r="F37" s="656" t="n"/>
-      <c r="G37" s="656" t="n"/>
-      <c r="H37" s="656" t="n"/>
+      <c r="A37" s="666" t="n"/>
+      <c r="B37" s="666" t="n"/>
+      <c r="C37" s="666" t="n"/>
+      <c r="D37" s="666" t="n"/>
+      <c r="E37" s="666" t="n"/>
+      <c r="F37" s="666" t="n"/>
+      <c r="G37" s="666" t="n"/>
+      <c r="H37" s="666" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="656" t="n"/>
-      <c r="B38" s="656" t="n"/>
-      <c r="C38" s="656" t="n"/>
-      <c r="D38" s="656" t="n"/>
-      <c r="E38" s="656" t="n"/>
-      <c r="F38" s="656" t="n"/>
-      <c r="G38" s="656" t="n"/>
-      <c r="H38" s="656" t="n"/>
+      <c r="A38" s="666" t="n"/>
+      <c r="B38" s="666" t="n"/>
+      <c r="C38" s="666" t="n"/>
+      <c r="D38" s="666" t="n"/>
+      <c r="E38" s="666" t="n"/>
+      <c r="F38" s="666" t="n"/>
+      <c r="G38" s="666" t="n"/>
+      <c r="H38" s="666" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="656" t="n"/>
-      <c r="B39" s="656" t="n"/>
-      <c r="C39" s="656" t="n"/>
-      <c r="D39" s="656" t="n"/>
-      <c r="E39" s="656" t="n"/>
-      <c r="F39" s="656" t="n"/>
-      <c r="G39" s="656" t="n"/>
-      <c r="H39" s="656" t="n"/>
+      <c r="A39" s="666" t="n"/>
+      <c r="B39" s="666" t="n"/>
+      <c r="C39" s="666" t="n"/>
+      <c r="D39" s="666" t="n"/>
+      <c r="E39" s="666" t="n"/>
+      <c r="F39" s="666" t="n"/>
+      <c r="G39" s="666" t="n"/>
+      <c r="H39" s="666" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="656" t="n"/>
-      <c r="B40" s="656" t="n"/>
-      <c r="C40" s="656" t="n"/>
-      <c r="D40" s="656" t="n"/>
-      <c r="E40" s="656" t="n"/>
-      <c r="F40" s="656" t="n"/>
-      <c r="G40" s="656" t="n"/>
-      <c r="H40" s="656" t="n"/>
+      <c r="A40" s="666" t="n"/>
+      <c r="B40" s="666" t="n"/>
+      <c r="C40" s="666" t="n"/>
+      <c r="D40" s="666" t="n"/>
+      <c r="E40" s="666" t="n"/>
+      <c r="F40" s="666" t="n"/>
+      <c r="G40" s="666" t="n"/>
+      <c r="H40" s="666" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
     </row>

</xml_diff>

<commit_message>
fix: time, readme file
</commit_message>
<xml_diff>
--- a/users/uzuran/burn_table.xlsx
+++ b/users/uzuran/burn_table.xlsx
@@ -67,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="667">
+  <cellXfs count="676">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1760,6 +1760,33 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -2487,7 +2514,7 @@
       <c r="I1" s="3" t="n"/>
       <c r="J1" s="3" t="n"/>
     </row>
-    <row r="2" ht="18" customHeight="1">
+    <row r="2" ht="12.00188976377953" customHeight="1">
       <c r="A2" s="565" t="n"/>
       <c r="B2" s="565" t="n"/>
       <c r="C2" s="565" t="n"/>
@@ -2499,539 +2526,1001 @@
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
     </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="665" t="inlineStr">
-        <is>
-          <t>14.07.2026</t>
-        </is>
-      </c>
-      <c r="B3" s="665" t="inlineStr">
-        <is>
-          <t>4039-95</t>
-        </is>
-      </c>
-      <c r="C3" s="665" t="inlineStr">
-        <is>
-          <t>1.0026-2X2500X1250</t>
-        </is>
-      </c>
-      <c r="D3" s="665" t="n">
+    <row r="3" ht="12.00188976377953" customHeight="1">
+      <c r="A3" s="674" t="inlineStr">
+        <is>
+          <t>17.07.2026</t>
+        </is>
+      </c>
+      <c r="B3" s="674" t="inlineStr">
+        <is>
+          <t>4040-01</t>
+        </is>
+      </c>
+      <c r="C3" s="674" t="inlineStr">
+        <is>
+          <t>1.0037-5X3000X1500</t>
+        </is>
+      </c>
+      <c r="D3" s="674" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="665" t="inlineStr">
-        <is>
-          <t>00:04:03</t>
-        </is>
-      </c>
-      <c r="F3" s="665" t="n"/>
-      <c r="G3" s="665" t="n"/>
-      <c r="H3" s="665" t="n"/>
+      <c r="E3" s="674" t="inlineStr">
+        <is>
+          <t>00:23:29</t>
+        </is>
+      </c>
+      <c r="F3" s="674" t="n"/>
+      <c r="G3" s="674" t="n"/>
+      <c r="H3" s="674" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
     </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="665" t="n"/>
-      <c r="B4" s="665" t="inlineStr">
-        <is>
-          <t>4039-96</t>
-        </is>
-      </c>
-      <c r="C4" s="665" t="inlineStr">
-        <is>
-          <t>3.3535-2X2500X1250</t>
-        </is>
-      </c>
-      <c r="D4" s="665" t="n">
+    <row r="4" ht="12.00188976377953" customHeight="1">
+      <c r="A4" s="674" t="n"/>
+      <c r="B4" s="674" t="inlineStr">
+        <is>
+          <t>4040-02</t>
+        </is>
+      </c>
+      <c r="C4" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D4" s="674" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="665" t="inlineStr">
-        <is>
-          <t>00:03:09</t>
-        </is>
-      </c>
-      <c r="F4" s="665" t="n"/>
-      <c r="G4" s="665" t="n"/>
-      <c r="H4" s="665" t="n"/>
+      <c r="E4" s="674" t="inlineStr">
+        <is>
+          <t>00:23:39</t>
+        </is>
+      </c>
+      <c r="F4" s="674" t="n"/>
+      <c r="G4" s="674" t="n"/>
+      <c r="H4" s="674" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
     </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="665" t="n"/>
-      <c r="B5" s="665" t="inlineStr">
-        <is>
-          <t>4039-97</t>
-        </is>
-      </c>
-      <c r="C5" s="665" t="inlineStr">
+    <row r="5" ht="12.00188976377953" customHeight="1">
+      <c r="A5" s="674" t="n"/>
+      <c r="B5" s="674" t="inlineStr">
+        <is>
+          <t>4040-03</t>
+        </is>
+      </c>
+      <c r="C5" s="674" t="inlineStr">
         <is>
           <t>-----</t>
         </is>
       </c>
-      <c r="D5" s="665" t="n">
+      <c r="D5" s="674" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="665" t="inlineStr">
-        <is>
-          <t>00:03:56</t>
-        </is>
-      </c>
-      <c r="F5" s="665" t="n"/>
-      <c r="G5" s="665" t="n"/>
-      <c r="H5" s="665" t="n"/>
+      <c r="E5" s="674" t="inlineStr">
+        <is>
+          <t>00:19:01</t>
+        </is>
+      </c>
+      <c r="F5" s="674" t="n"/>
+      <c r="G5" s="674" t="n"/>
+      <c r="H5" s="674" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
     </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="665" t="n"/>
-      <c r="B6" s="665" t="inlineStr">
-        <is>
-          <t>4039-98</t>
-        </is>
-      </c>
-      <c r="C6" s="665" t="inlineStr">
+    <row r="6" ht="12.00188976377953" customHeight="1">
+      <c r="A6" s="674" t="n"/>
+      <c r="B6" s="674" t="inlineStr">
+        <is>
+          <t>4040-04</t>
+        </is>
+      </c>
+      <c r="C6" s="674" t="inlineStr">
         <is>
           <t>-----</t>
         </is>
       </c>
-      <c r="D6" s="665" t="n">
+      <c r="D6" s="674" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="665" t="inlineStr">
-        <is>
-          <t>00:03:02</t>
-        </is>
-      </c>
-      <c r="F6" s="665" t="n"/>
-      <c r="G6" s="665" t="n"/>
-      <c r="H6" s="665" t="n"/>
+      <c r="E6" s="674" t="inlineStr">
+        <is>
+          <t>00:17:26</t>
+        </is>
+      </c>
+      <c r="F6" s="674" t="n"/>
+      <c r="G6" s="674" t="n"/>
+      <c r="H6" s="674" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
     </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="665" t="n"/>
-      <c r="B7" s="665" t="inlineStr">
-        <is>
-          <t>4039-99</t>
-        </is>
-      </c>
-      <c r="C7" s="665" t="inlineStr">
-        <is>
-          <t>3.3535-2X3000X1500</t>
-        </is>
-      </c>
-      <c r="D7" s="665" t="n">
+    <row r="7" ht="12.00188976377953" customHeight="1">
+      <c r="A7" s="674" t="n"/>
+      <c r="B7" s="674" t="inlineStr">
+        <is>
+          <t>4040-05</t>
+        </is>
+      </c>
+      <c r="C7" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D7" s="674" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="665" t="inlineStr">
-        <is>
-          <t>00:02:44</t>
-        </is>
-      </c>
-      <c r="F7" s="665" t="n"/>
-      <c r="G7" s="665" t="n"/>
-      <c r="H7" s="665" t="n"/>
+      <c r="E7" s="674" t="inlineStr">
+        <is>
+          <t>00:33:03</t>
+        </is>
+      </c>
+      <c r="F7" s="674" t="n"/>
+      <c r="G7" s="674" t="n"/>
+      <c r="H7" s="674" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
     </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="665" t="n"/>
-      <c r="B8" s="665" t="n"/>
-      <c r="C8" s="665" t="n"/>
-      <c r="D8" s="665" t="n"/>
-      <c r="E8" s="665" t="n"/>
-      <c r="F8" s="665" t="n"/>
-      <c r="G8" s="665" t="n"/>
-      <c r="H8" s="665" t="n"/>
+    <row r="8" ht="12.00188976377953" customHeight="1">
+      <c r="A8" s="674" t="n"/>
+      <c r="B8" s="674" t="inlineStr">
+        <is>
+          <t>4041-05</t>
+        </is>
+      </c>
+      <c r="C8" s="674" t="inlineStr">
+        <is>
+          <t>3.3535SPECIAL-3X3000X1500</t>
+        </is>
+      </c>
+      <c r="D8" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="674" t="inlineStr">
+        <is>
+          <t>00:04:40</t>
+        </is>
+      </c>
+      <c r="F8" s="674" t="n"/>
+      <c r="G8" s="674" t="n"/>
+      <c r="H8" s="674" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
     </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="665" t="n"/>
-      <c r="B9" s="665" t="n"/>
-      <c r="C9" s="665" t="n"/>
-      <c r="D9" s="665" t="n"/>
-      <c r="E9" s="665" t="n"/>
-      <c r="F9" s="665" t="n"/>
-      <c r="G9" s="665" t="n"/>
-      <c r="H9" s="665" t="n"/>
+    <row r="9" ht="12.00188976377953" customHeight="1">
+      <c r="A9" s="674" t="n"/>
+      <c r="B9" s="674" t="inlineStr">
+        <is>
+          <t>4041-06</t>
+        </is>
+      </c>
+      <c r="C9" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D9" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="674" t="inlineStr">
+        <is>
+          <t>00:12:06</t>
+        </is>
+      </c>
+      <c r="F9" s="674" t="n"/>
+      <c r="G9" s="674" t="n"/>
+      <c r="H9" s="674" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
     </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="665" t="n"/>
-      <c r="B10" s="665" t="n"/>
-      <c r="C10" s="665" t="n"/>
-      <c r="D10" s="665" t="n"/>
-      <c r="E10" s="665" t="n"/>
-      <c r="F10" s="665" t="n"/>
-      <c r="G10" s="665" t="n"/>
-      <c r="H10" s="665" t="n"/>
+    <row r="10" ht="12.00188976377953" customHeight="1">
+      <c r="A10" s="674" t="n"/>
+      <c r="B10" s="674" t="inlineStr">
+        <is>
+          <t>4041-07</t>
+        </is>
+      </c>
+      <c r="C10" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D10" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="674" t="inlineStr">
+        <is>
+          <t>00:12:19</t>
+        </is>
+      </c>
+      <c r="F10" s="674" t="n"/>
+      <c r="G10" s="674" t="n"/>
+      <c r="H10" s="674" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="665" t="n"/>
-      <c r="B11" s="665" t="n"/>
-      <c r="C11" s="665" t="n"/>
-      <c r="D11" s="665" t="n"/>
-      <c r="E11" s="665" t="n"/>
-      <c r="F11" s="665" t="n"/>
-      <c r="G11" s="665" t="n"/>
-      <c r="H11" s="665" t="n"/>
+    <row r="11" ht="12.00188976377953" customHeight="1">
+      <c r="A11" s="674" t="n"/>
+      <c r="B11" s="674" t="inlineStr">
+        <is>
+          <t>4042-07</t>
+        </is>
+      </c>
+      <c r="C11" s="674" t="inlineStr">
+        <is>
+          <t>3.3535-4X2500X1250</t>
+        </is>
+      </c>
+      <c r="D11" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="674" t="inlineStr">
+        <is>
+          <t>00:07:28</t>
+        </is>
+      </c>
+      <c r="F11" s="674" t="n"/>
+      <c r="G11" s="674" t="n"/>
+      <c r="H11" s="674" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
     </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="665" t="n"/>
-      <c r="B12" s="665" t="n"/>
-      <c r="C12" s="665" t="n"/>
-      <c r="D12" s="665" t="n"/>
-      <c r="E12" s="665" t="n"/>
-      <c r="F12" s="665" t="n"/>
-      <c r="G12" s="665" t="n"/>
-      <c r="H12" s="665" t="n"/>
+    <row r="12" ht="12.00188976377953" customHeight="1">
+      <c r="A12" s="674" t="n"/>
+      <c r="B12" s="674" t="inlineStr">
+        <is>
+          <t>4042-08</t>
+        </is>
+      </c>
+      <c r="C12" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D12" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="674" t="inlineStr">
+        <is>
+          <t>00:10:04</t>
+        </is>
+      </c>
+      <c r="F12" s="674" t="n"/>
+      <c r="G12" s="674" t="n"/>
+      <c r="H12" s="674" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="665" t="n"/>
-      <c r="B13" s="665" t="n"/>
-      <c r="C13" s="665" t="n"/>
-      <c r="D13" s="665" t="n"/>
-      <c r="E13" s="665" t="n"/>
-      <c r="F13" s="665" t="n"/>
-      <c r="G13" s="665" t="n"/>
-      <c r="H13" s="665" t="n"/>
+    <row r="13" ht="12.00188976377953" customHeight="1">
+      <c r="A13" s="674" t="n"/>
+      <c r="B13" s="674" t="inlineStr">
+        <is>
+          <t>4043-09</t>
+        </is>
+      </c>
+      <c r="C13" s="674" t="inlineStr">
+        <is>
+          <t>3.3535-1X2500X1250</t>
+        </is>
+      </c>
+      <c r="D13" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="674" t="inlineStr">
+        <is>
+          <t>00:07:32</t>
+        </is>
+      </c>
+      <c r="F13" s="674" t="n"/>
+      <c r="G13" s="674" t="n"/>
+      <c r="H13" s="674" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
     </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="665" t="n"/>
-      <c r="B14" s="665" t="n"/>
-      <c r="C14" s="665" t="n"/>
-      <c r="D14" s="665" t="n"/>
-      <c r="E14" s="665" t="n"/>
-      <c r="F14" s="665" t="n"/>
-      <c r="G14" s="665" t="n"/>
-      <c r="H14" s="665" t="n"/>
+    <row r="14" ht="12.00188976377953" customHeight="1">
+      <c r="A14" s="674" t="n"/>
+      <c r="B14" s="674" t="inlineStr">
+        <is>
+          <t>4043-10</t>
+        </is>
+      </c>
+      <c r="C14" s="674" t="inlineStr">
+        <is>
+          <t>3.3535-1X3000X1500</t>
+        </is>
+      </c>
+      <c r="D14" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="674" t="inlineStr">
+        <is>
+          <t>00:04:19</t>
+        </is>
+      </c>
+      <c r="F14" s="674" t="n"/>
+      <c r="G14" s="674" t="n"/>
+      <c r="H14" s="674" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="665" t="n"/>
-      <c r="B15" s="665" t="n"/>
-      <c r="C15" s="665" t="n"/>
-      <c r="D15" s="665" t="n"/>
-      <c r="E15" s="665" t="n"/>
-      <c r="F15" s="665" t="n"/>
-      <c r="G15" s="665" t="n"/>
-      <c r="H15" s="665" t="n"/>
+    <row r="15" ht="12.00188976377953" customHeight="1">
+      <c r="A15" s="674" t="n"/>
+      <c r="B15" s="674" t="inlineStr">
+        <is>
+          <t>4044-11</t>
+        </is>
+      </c>
+      <c r="C15" s="674" t="inlineStr">
+        <is>
+          <t>1.0037-3X3000X1500</t>
+        </is>
+      </c>
+      <c r="D15" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="674" t="inlineStr">
+        <is>
+          <t>00:10:17</t>
+        </is>
+      </c>
+      <c r="F15" s="674" t="n"/>
+      <c r="G15" s="674" t="n"/>
+      <c r="H15" s="674" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
     </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="665" t="n"/>
-      <c r="B16" s="665" t="n"/>
-      <c r="C16" s="665" t="n"/>
-      <c r="D16" s="665" t="n"/>
-      <c r="E16" s="665" t="n"/>
-      <c r="F16" s="665" t="n"/>
-      <c r="G16" s="665" t="n"/>
-      <c r="H16" s="665" t="n"/>
+    <row r="16" ht="12.00188976377953" customHeight="1">
+      <c r="A16" s="674" t="n"/>
+      <c r="B16" s="674" t="inlineStr">
+        <is>
+          <t>4044-12</t>
+        </is>
+      </c>
+      <c r="C16" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D16" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="674" t="inlineStr">
+        <is>
+          <t>00:06:31</t>
+        </is>
+      </c>
+      <c r="F16" s="674" t="n"/>
+      <c r="G16" s="674" t="n"/>
+      <c r="H16" s="674" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
     </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="665" t="n"/>
-      <c r="B17" s="665" t="n"/>
-      <c r="C17" s="665" t="n"/>
-      <c r="D17" s="665" t="n"/>
-      <c r="E17" s="665" t="n"/>
-      <c r="F17" s="665" t="n"/>
-      <c r="G17" s="665" t="n"/>
-      <c r="H17" s="665" t="n"/>
+    <row r="17" ht="12.00188976377953" customHeight="1">
+      <c r="A17" s="674" t="n"/>
+      <c r="B17" s="674" t="inlineStr">
+        <is>
+          <t>4044-13</t>
+        </is>
+      </c>
+      <c r="C17" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D17" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="674" t="inlineStr">
+        <is>
+          <t>00:06:21</t>
+        </is>
+      </c>
+      <c r="F17" s="674" t="n"/>
+      <c r="G17" s="674" t="n"/>
+      <c r="H17" s="674" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n"/>
     </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="665" t="n"/>
-      <c r="B18" s="665" t="n"/>
-      <c r="C18" s="665" t="n"/>
-      <c r="D18" s="665" t="n"/>
-      <c r="E18" s="665" t="n"/>
-      <c r="F18" s="665" t="n"/>
-      <c r="G18" s="665" t="n"/>
-      <c r="H18" s="665" t="n"/>
+    <row r="18" ht="12.00188976377953" customHeight="1">
+      <c r="A18" s="674" t="n"/>
+      <c r="B18" s="674" t="inlineStr">
+        <is>
+          <t>4045-14</t>
+        </is>
+      </c>
+      <c r="C18" s="674" t="inlineStr">
+        <is>
+          <t>1.0037-2X3000X1500</t>
+        </is>
+      </c>
+      <c r="D18" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="674" t="inlineStr">
+        <is>
+          <t>00:07:47</t>
+        </is>
+      </c>
+      <c r="F18" s="674" t="n"/>
+      <c r="G18" s="674" t="n"/>
+      <c r="H18" s="674" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
     </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="665" t="n"/>
-      <c r="B19" s="665" t="n"/>
-      <c r="C19" s="665" t="n"/>
-      <c r="D19" s="665" t="n"/>
-      <c r="E19" s="665" t="n"/>
-      <c r="F19" s="665" t="n"/>
-      <c r="G19" s="665" t="n"/>
-      <c r="H19" s="665" t="n"/>
+    <row r="19" ht="12.00188976377953" customHeight="1">
+      <c r="A19" s="674" t="n"/>
+      <c r="B19" s="674" t="inlineStr">
+        <is>
+          <t>4046-15</t>
+        </is>
+      </c>
+      <c r="C19" s="674" t="inlineStr">
+        <is>
+          <t>1.0037-5X3000X1500</t>
+        </is>
+      </c>
+      <c r="D19" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="674" t="inlineStr">
+        <is>
+          <t>00:07:53</t>
+        </is>
+      </c>
+      <c r="F19" s="674" t="n"/>
+      <c r="G19" s="674" t="n"/>
+      <c r="H19" s="674" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
     </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="665" t="n"/>
-      <c r="B20" s="665" t="n"/>
-      <c r="C20" s="665" t="n"/>
-      <c r="D20" s="665" t="n"/>
-      <c r="E20" s="665" t="n"/>
-      <c r="F20" s="665" t="n"/>
-      <c r="G20" s="665" t="n"/>
-      <c r="H20" s="665" t="n"/>
+    <row r="20" ht="12.00188976377953" customHeight="1">
+      <c r="A20" s="674" t="n"/>
+      <c r="B20" s="674" t="inlineStr">
+        <is>
+          <t>4046-16</t>
+        </is>
+      </c>
+      <c r="C20" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D20" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="674" t="inlineStr">
+        <is>
+          <t>00:19:31</t>
+        </is>
+      </c>
+      <c r="F20" s="674" t="n"/>
+      <c r="G20" s="674" t="n"/>
+      <c r="H20" s="674" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
     </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="665" t="n"/>
-      <c r="B21" s="665" t="n"/>
-      <c r="C21" s="665" t="n"/>
-      <c r="D21" s="665" t="n"/>
-      <c r="E21" s="665" t="n"/>
-      <c r="F21" s="665" t="n"/>
-      <c r="G21" s="665" t="n"/>
-      <c r="H21" s="665" t="n"/>
+    <row r="21" ht="12.00188976377953" customHeight="1">
+      <c r="A21" s="674" t="n"/>
+      <c r="B21" s="674" t="inlineStr">
+        <is>
+          <t>4046-17</t>
+        </is>
+      </c>
+      <c r="C21" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D21" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="674" t="inlineStr">
+        <is>
+          <t>00:24:45</t>
+        </is>
+      </c>
+      <c r="F21" s="674" t="n"/>
+      <c r="G21" s="674" t="n"/>
+      <c r="H21" s="674" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
     </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="665" t="n"/>
-      <c r="B22" s="665" t="n"/>
-      <c r="C22" s="665" t="n"/>
-      <c r="D22" s="665" t="n"/>
-      <c r="E22" s="665" t="n"/>
-      <c r="F22" s="665" t="n"/>
-      <c r="G22" s="665" t="n"/>
-      <c r="H22" s="665" t="n"/>
+    <row r="22" ht="12.00188976377953" customHeight="1">
+      <c r="A22" s="674" t="n"/>
+      <c r="B22" s="674" t="inlineStr">
+        <is>
+          <t>4046-18</t>
+        </is>
+      </c>
+      <c r="C22" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D22" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="674" t="inlineStr">
+        <is>
+          <t>00:26:48</t>
+        </is>
+      </c>
+      <c r="F22" s="674" t="n"/>
+      <c r="G22" s="674" t="n"/>
+      <c r="H22" s="674" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
     </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="665" t="n"/>
-      <c r="B23" s="665" t="n"/>
-      <c r="C23" s="665" t="n"/>
-      <c r="D23" s="665" t="n"/>
-      <c r="E23" s="665" t="n"/>
-      <c r="F23" s="665" t="n"/>
-      <c r="G23" s="665" t="n"/>
-      <c r="H23" s="665" t="n"/>
+    <row r="23" ht="12.00188976377953" customHeight="1">
+      <c r="A23" s="674" t="n"/>
+      <c r="B23" s="674" t="inlineStr">
+        <is>
+          <t>4047-19</t>
+        </is>
+      </c>
+      <c r="C23" s="674" t="inlineStr">
+        <is>
+          <t>3.3535-2X2500X1250</t>
+        </is>
+      </c>
+      <c r="D23" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="674" t="inlineStr">
+        <is>
+          <t>00:00:48</t>
+        </is>
+      </c>
+      <c r="F23" s="674" t="n"/>
+      <c r="G23" s="674" t="n"/>
+      <c r="H23" s="674" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
     </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="665" t="n"/>
-      <c r="B24" s="665" t="n"/>
-      <c r="C24" s="665" t="n"/>
-      <c r="D24" s="665" t="n"/>
-      <c r="E24" s="665" t="n"/>
-      <c r="F24" s="665" t="n"/>
-      <c r="G24" s="665" t="n"/>
-      <c r="H24" s="665" t="n"/>
+    <row r="24" ht="12.00188976377953" customHeight="1">
+      <c r="A24" s="674" t="n"/>
+      <c r="B24" s="674" t="inlineStr">
+        <is>
+          <t>4049-22</t>
+        </is>
+      </c>
+      <c r="C24" s="674" t="inlineStr">
+        <is>
+          <t>1.0037-3X3000X1500</t>
+        </is>
+      </c>
+      <c r="D24" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="674" t="inlineStr">
+        <is>
+          <t>00:06:01</t>
+        </is>
+      </c>
+      <c r="F24" s="674" t="n"/>
+      <c r="G24" s="674" t="n"/>
+      <c r="H24" s="674" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
     </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="665" t="n"/>
-      <c r="B25" s="665" t="n"/>
-      <c r="C25" s="665" t="n"/>
-      <c r="D25" s="665" t="n"/>
-      <c r="E25" s="665" t="n"/>
-      <c r="F25" s="665" t="n"/>
-      <c r="G25" s="665" t="n"/>
-      <c r="H25" s="665" t="n"/>
+    <row r="25" ht="12.00188976377953" customHeight="1">
+      <c r="A25" s="674" t="n"/>
+      <c r="B25" s="674" t="inlineStr">
+        <is>
+          <t>4049-23</t>
+        </is>
+      </c>
+      <c r="C25" s="674" t="inlineStr">
+        <is>
+          <t>1.0037-3X1950X1500</t>
+        </is>
+      </c>
+      <c r="D25" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="674" t="inlineStr">
+        <is>
+          <t>00:04:01</t>
+        </is>
+      </c>
+      <c r="F25" s="674" t="n"/>
+      <c r="G25" s="674" t="n"/>
+      <c r="H25" s="674" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
     </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="665" t="n"/>
-      <c r="B26" s="665" t="n"/>
-      <c r="C26" s="665" t="n"/>
-      <c r="D26" s="665" t="n"/>
-      <c r="E26" s="665" t="n"/>
-      <c r="F26" s="665" t="n"/>
-      <c r="G26" s="665" t="n"/>
-      <c r="H26" s="665" t="n"/>
+    <row r="26" ht="12.00188976377953" customHeight="1">
+      <c r="A26" s="674" t="n"/>
+      <c r="B26" s="674" t="inlineStr">
+        <is>
+          <t>4049-24</t>
+        </is>
+      </c>
+      <c r="C26" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D26" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="674" t="inlineStr">
+        <is>
+          <t>00:03:19</t>
+        </is>
+      </c>
+      <c r="F26" s="674" t="n"/>
+      <c r="G26" s="674" t="n"/>
+      <c r="H26" s="674" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
     </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="665" t="n"/>
-      <c r="B27" s="665" t="n"/>
-      <c r="C27" s="665" t="n"/>
-      <c r="D27" s="665" t="n"/>
-      <c r="E27" s="665" t="n"/>
-      <c r="F27" s="665" t="n"/>
-      <c r="G27" s="665" t="n"/>
-      <c r="H27" s="665" t="n"/>
+    <row r="27" ht="12.00188976377953" customHeight="1">
+      <c r="A27" s="674" t="n"/>
+      <c r="B27" s="674" t="inlineStr">
+        <is>
+          <t>4049-25</t>
+        </is>
+      </c>
+      <c r="C27" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D27" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="674" t="inlineStr">
+        <is>
+          <t>00:05:11</t>
+        </is>
+      </c>
+      <c r="F27" s="674" t="n"/>
+      <c r="G27" s="674" t="n"/>
+      <c r="H27" s="674" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
     </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="665" t="n"/>
-      <c r="B28" s="665" t="n"/>
-      <c r="C28" s="665" t="n"/>
-      <c r="D28" s="665" t="n"/>
-      <c r="E28" s="665" t="n"/>
-      <c r="F28" s="665" t="n"/>
-      <c r="G28" s="665" t="n"/>
-      <c r="H28" s="665" t="n"/>
+    <row r="28" ht="12.00188976377953" customHeight="1">
+      <c r="A28" s="674" t="n"/>
+      <c r="B28" s="674" t="inlineStr">
+        <is>
+          <t>4049-26</t>
+        </is>
+      </c>
+      <c r="C28" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D28" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="674" t="inlineStr">
+        <is>
+          <t>00:04:11</t>
+        </is>
+      </c>
+      <c r="F28" s="674" t="n"/>
+      <c r="G28" s="674" t="n"/>
+      <c r="H28" s="674" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="665" t="n"/>
-      <c r="B29" s="665" t="n"/>
-      <c r="C29" s="665" t="n"/>
-      <c r="D29" s="665" t="n"/>
-      <c r="E29" s="665" t="n"/>
-      <c r="F29" s="665" t="n"/>
-      <c r="G29" s="665" t="n"/>
-      <c r="H29" s="665" t="n"/>
+    <row r="29" ht="12.00188976377953" customHeight="1">
+      <c r="A29" s="674" t="n"/>
+      <c r="B29" s="674" t="inlineStr">
+        <is>
+          <t>4049-27</t>
+        </is>
+      </c>
+      <c r="C29" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D29" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="674" t="inlineStr">
+        <is>
+          <t>00:08:25</t>
+        </is>
+      </c>
+      <c r="F29" s="674" t="n"/>
+      <c r="G29" s="674" t="n"/>
+      <c r="H29" s="674" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
     </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="665" t="n"/>
-      <c r="B30" s="665" t="n"/>
-      <c r="C30" s="665" t="n"/>
-      <c r="D30" s="665" t="n"/>
-      <c r="E30" s="665" t="n"/>
-      <c r="F30" s="665" t="n"/>
-      <c r="G30" s="665" t="n"/>
-      <c r="H30" s="665" t="n"/>
+    <row r="30" ht="12.00188976377953" customHeight="1">
+      <c r="A30" s="674" t="n"/>
+      <c r="B30" s="674" t="inlineStr">
+        <is>
+          <t>4052-28</t>
+        </is>
+      </c>
+      <c r="C30" s="674" t="inlineStr">
+        <is>
+          <t>1.0037-3X3000X1500</t>
+        </is>
+      </c>
+      <c r="D30" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="674" t="inlineStr">
+        <is>
+          <t>00:02:50</t>
+        </is>
+      </c>
+      <c r="F30" s="674" t="n"/>
+      <c r="G30" s="674" t="n"/>
+      <c r="H30" s="674" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="665" t="n"/>
-      <c r="B31" s="665" t="n"/>
-      <c r="C31" s="665" t="n"/>
-      <c r="D31" s="665" t="n"/>
-      <c r="E31" s="665" t="n"/>
-      <c r="F31" s="665" t="n"/>
-      <c r="G31" s="665" t="n"/>
-      <c r="H31" s="665" t="n"/>
+    <row r="31" ht="12.00188976377953" customHeight="1">
+      <c r="A31" s="674" t="n"/>
+      <c r="B31" s="674" t="inlineStr">
+        <is>
+          <t>4052-29</t>
+        </is>
+      </c>
+      <c r="C31" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D31" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="674" t="inlineStr">
+        <is>
+          <t>00:02:40</t>
+        </is>
+      </c>
+      <c r="F31" s="674" t="n"/>
+      <c r="G31" s="674" t="n"/>
+      <c r="H31" s="674" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
     </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="665" t="n"/>
-      <c r="B32" s="665" t="n"/>
-      <c r="C32" s="665" t="n"/>
-      <c r="D32" s="665" t="n"/>
-      <c r="E32" s="665" t="n"/>
-      <c r="F32" s="665" t="n"/>
-      <c r="G32" s="665" t="n"/>
-      <c r="H32" s="665" t="n"/>
+    <row r="32" ht="12.00188976377953" customHeight="1">
+      <c r="A32" s="674" t="n"/>
+      <c r="B32" s="674" t="inlineStr">
+        <is>
+          <t>4052-30</t>
+        </is>
+      </c>
+      <c r="C32" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D32" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="674" t="inlineStr">
+        <is>
+          <t>00:03:10</t>
+        </is>
+      </c>
+      <c r="F32" s="674" t="n"/>
+      <c r="G32" s="674" t="n"/>
+      <c r="H32" s="674" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
     </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="665" t="n"/>
-      <c r="B33" s="665" t="n"/>
-      <c r="C33" s="665" t="n"/>
-      <c r="D33" s="665" t="n"/>
-      <c r="E33" s="665" t="n"/>
-      <c r="F33" s="665" t="n"/>
-      <c r="G33" s="665" t="n"/>
-      <c r="H33" s="665" t="n"/>
+    <row r="33" ht="12.00188976377953" customHeight="1">
+      <c r="A33" s="674" t="n"/>
+      <c r="B33" s="674" t="inlineStr">
+        <is>
+          <t>4052-31</t>
+        </is>
+      </c>
+      <c r="C33" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D33" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="674" t="inlineStr">
+        <is>
+          <t>00:04:35</t>
+        </is>
+      </c>
+      <c r="F33" s="674" t="n"/>
+      <c r="G33" s="674" t="n"/>
+      <c r="H33" s="674" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
     </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="665" t="n"/>
-      <c r="B34" s="665" t="n"/>
-      <c r="C34" s="665" t="n"/>
-      <c r="D34" s="665" t="n"/>
-      <c r="E34" s="665" t="n"/>
-      <c r="F34" s="665" t="n"/>
-      <c r="G34" s="665" t="n"/>
-      <c r="H34" s="665" t="n"/>
+    <row r="34" ht="12.00188976377953" customHeight="1">
+      <c r="A34" s="674" t="n"/>
+      <c r="B34" s="674" t="inlineStr">
+        <is>
+          <t>4052-32</t>
+        </is>
+      </c>
+      <c r="C34" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D34" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="674" t="inlineStr">
+        <is>
+          <t>00:03:57</t>
+        </is>
+      </c>
+      <c r="F34" s="674" t="n"/>
+      <c r="G34" s="674" t="n"/>
+      <c r="H34" s="674" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
     </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="665" t="n"/>
-      <c r="B35" s="665" t="n"/>
-      <c r="C35" s="665" t="n"/>
-      <c r="D35" s="665" t="n"/>
-      <c r="E35" s="665" t="n"/>
-      <c r="F35" s="665" t="n"/>
-      <c r="G35" s="665" t="n"/>
-      <c r="H35" s="665" t="n"/>
+    <row r="35" ht="12.00188976377953" customHeight="1">
+      <c r="A35" s="674" t="n"/>
+      <c r="B35" s="674" t="inlineStr">
+        <is>
+          <t>4052-33</t>
+        </is>
+      </c>
+      <c r="C35" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D35" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="674" t="inlineStr">
+        <is>
+          <t>00:04:35</t>
+        </is>
+      </c>
+      <c r="F35" s="674" t="n"/>
+      <c r="G35" s="674" t="n"/>
+      <c r="H35" s="674" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="665" t="n"/>
-      <c r="B36" s="665" t="n"/>
-      <c r="C36" s="665" t="n"/>
-      <c r="D36" s="665" t="n"/>
-      <c r="E36" s="665" t="n"/>
-      <c r="F36" s="665" t="n"/>
-      <c r="G36" s="665" t="n"/>
-      <c r="H36" s="665" t="n"/>
+    <row r="36" ht="12.00188976377953" customHeight="1">
+      <c r="A36" s="674" t="n"/>
+      <c r="B36" s="674" t="inlineStr">
+        <is>
+          <t>4052-34</t>
+        </is>
+      </c>
+      <c r="C36" s="674" t="inlineStr">
+        <is>
+          <t>1.0037-3X1950X1500</t>
+        </is>
+      </c>
+      <c r="D36" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="674" t="inlineStr">
+        <is>
+          <t>00:02:32</t>
+        </is>
+      </c>
+      <c r="F36" s="674" t="n"/>
+      <c r="G36" s="674" t="n"/>
+      <c r="H36" s="674" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="665" t="n"/>
-      <c r="B37" s="665" t="n"/>
-      <c r="C37" s="665" t="n"/>
-      <c r="D37" s="665" t="n"/>
-      <c r="E37" s="665" t="n"/>
-      <c r="F37" s="665" t="n"/>
-      <c r="G37" s="665" t="n"/>
-      <c r="H37" s="665" t="n"/>
+    <row r="37" ht="12.00188976377953" customHeight="1">
+      <c r="A37" s="674" t="n"/>
+      <c r="B37" s="674" t="inlineStr">
+        <is>
+          <t>4052-35</t>
+        </is>
+      </c>
+      <c r="C37" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D37" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="674" t="inlineStr">
+        <is>
+          <t>00:01:12</t>
+        </is>
+      </c>
+      <c r="F37" s="674" t="n"/>
+      <c r="G37" s="674" t="n"/>
+      <c r="H37" s="674" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
     </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="665" t="n"/>
-      <c r="B38" s="665" t="n"/>
-      <c r="C38" s="665" t="n"/>
-      <c r="D38" s="665" t="n"/>
-      <c r="E38" s="665" t="n"/>
-      <c r="F38" s="665" t="n"/>
-      <c r="G38" s="665" t="n"/>
-      <c r="H38" s="665" t="n"/>
+    <row r="38" ht="12.00188976377953" customHeight="1">
+      <c r="A38" s="674" t="n"/>
+      <c r="B38" s="674" t="inlineStr">
+        <is>
+          <t>4053-35</t>
+        </is>
+      </c>
+      <c r="C38" s="674" t="inlineStr">
+        <is>
+          <t>1.0037-4X3000X1500</t>
+        </is>
+      </c>
+      <c r="D38" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="674" t="inlineStr">
+        <is>
+          <t>00:32:21</t>
+        </is>
+      </c>
+      <c r="F38" s="674" t="n"/>
+      <c r="G38" s="674" t="n"/>
+      <c r="H38" s="674" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="665" t="n"/>
-      <c r="B39" s="665" t="n"/>
-      <c r="C39" s="665" t="n"/>
-      <c r="D39" s="665" t="n"/>
-      <c r="E39" s="665" t="n"/>
-      <c r="F39" s="665" t="n"/>
-      <c r="G39" s="665" t="n"/>
-      <c r="H39" s="665" t="n"/>
+    <row r="39" ht="12.00188976377953" customHeight="1">
+      <c r="A39" s="674" t="n"/>
+      <c r="B39" s="674" t="inlineStr">
+        <is>
+          <t>4053-36</t>
+        </is>
+      </c>
+      <c r="C39" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D39" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="674" t="inlineStr">
+        <is>
+          <t>00:10:34</t>
+        </is>
+      </c>
+      <c r="F39" s="674" t="n"/>
+      <c r="G39" s="674" t="n"/>
+      <c r="H39" s="674" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n"/>
     </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="665" t="n"/>
-      <c r="B40" s="665" t="n"/>
-      <c r="C40" s="665" t="n"/>
-      <c r="D40" s="665" t="n"/>
-      <c r="E40" s="665" t="n"/>
-      <c r="F40" s="665" t="n"/>
-      <c r="G40" s="665" t="n"/>
-      <c r="H40" s="665" t="n"/>
+    <row r="40" ht="12.00188976377953" customHeight="1">
+      <c r="A40" s="674" t="n"/>
+      <c r="B40" s="674" t="inlineStr">
+        <is>
+          <t>4053-37</t>
+        </is>
+      </c>
+      <c r="C40" s="674" t="inlineStr">
+        <is>
+          <t>-----</t>
+        </is>
+      </c>
+      <c r="D40" s="674" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="674" t="inlineStr">
+        <is>
+          <t>00:11:02</t>
+        </is>
+      </c>
+      <c r="F40" s="674" t="n"/>
+      <c r="G40" s="674" t="n"/>
+      <c r="H40" s="674" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.2" footer="0.2"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -3098,514 +3587,468 @@
       <c r="I1" s="3" t="n"/>
       <c r="J1" s="3" t="n"/>
     </row>
-    <row r="2">
+    <row r="2" ht="12.00188976377953" customHeight="1">
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
     </row>
-    <row r="3">
-      <c r="A3" s="666" t="inlineStr">
-        <is>
-          <t>15.07.2026</t>
-        </is>
-      </c>
-      <c r="B3" s="666" t="inlineStr">
-        <is>
-          <t>4039-95</t>
-        </is>
-      </c>
-      <c r="C3" s="666" t="inlineStr">
-        <is>
-          <t>1.0026-2X2500X1250</t>
-        </is>
-      </c>
-      <c r="D3" s="666" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="666" t="inlineStr">
-        <is>
-          <t>00:04:03</t>
-        </is>
-      </c>
-      <c r="F3" s="666" t="n"/>
-      <c r="G3" s="666" t="n"/>
-      <c r="H3" s="666" t="n"/>
+    <row r="3" ht="12.00188976377953" customHeight="1">
+      <c r="A3" s="675" t="n"/>
+      <c r="B3" s="675" t="n"/>
+      <c r="C3" s="675" t="n"/>
+      <c r="D3" s="675" t="n"/>
+      <c r="E3" s="675" t="n"/>
+      <c r="F3" s="675" t="n"/>
+      <c r="G3" s="675" t="n"/>
+      <c r="H3" s="675" t="n"/>
       <c r="I3" s="3" t="n"/>
       <c r="J3" s="3" t="n"/>
     </row>
-    <row r="4">
-      <c r="A4" s="666" t="n"/>
-      <c r="B4" s="666" t="inlineStr">
-        <is>
-          <t>4039-96</t>
-        </is>
-      </c>
-      <c r="C4" s="666" t="inlineStr">
-        <is>
-          <t>3.3535-2X2500X1250</t>
-        </is>
-      </c>
-      <c r="D4" s="666" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="666" t="inlineStr">
-        <is>
-          <t>00:03:09</t>
-        </is>
-      </c>
-      <c r="F4" s="666" t="n"/>
-      <c r="G4" s="666" t="n"/>
-      <c r="H4" s="666" t="n"/>
+    <row r="4" ht="12.00188976377953" customHeight="1">
+      <c r="A4" s="675" t="n"/>
+      <c r="B4" s="675" t="n"/>
+      <c r="C4" s="675" t="n"/>
+      <c r="D4" s="675" t="n"/>
+      <c r="E4" s="675" t="n"/>
+      <c r="F4" s="675" t="n"/>
+      <c r="G4" s="675" t="n"/>
+      <c r="H4" s="675" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
     </row>
-    <row r="5">
-      <c r="A5" s="666" t="n"/>
-      <c r="B5" s="666" t="inlineStr">
-        <is>
-          <t>4039-97</t>
-        </is>
-      </c>
-      <c r="C5" s="666" t="inlineStr">
-        <is>
-          <t>-----</t>
-        </is>
-      </c>
-      <c r="D5" s="666" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="666" t="inlineStr">
-        <is>
-          <t>00:03:56</t>
-        </is>
-      </c>
-      <c r="F5" s="666" t="n"/>
-      <c r="G5" s="666" t="n"/>
-      <c r="H5" s="666" t="n"/>
+    <row r="5" ht="12.00188976377953" customHeight="1">
+      <c r="A5" s="675" t="n"/>
+      <c r="B5" s="675" t="n"/>
+      <c r="C5" s="675" t="n"/>
+      <c r="D5" s="675" t="n"/>
+      <c r="E5" s="675" t="n"/>
+      <c r="F5" s="675" t="n"/>
+      <c r="G5" s="675" t="n"/>
+      <c r="H5" s="675" t="n"/>
       <c r="I5" s="3" t="n"/>
       <c r="J5" s="3" t="n"/>
     </row>
-    <row r="6">
-      <c r="A6" s="666" t="n"/>
-      <c r="B6" s="666" t="n"/>
-      <c r="C6" s="666" t="n"/>
-      <c r="D6" s="666" t="n"/>
-      <c r="E6" s="666" t="n"/>
-      <c r="F6" s="666" t="n"/>
-      <c r="G6" s="666" t="n"/>
-      <c r="H6" s="666" t="n"/>
+    <row r="6" ht="12.00188976377953" customHeight="1">
+      <c r="A6" s="675" t="n"/>
+      <c r="B6" s="675" t="n"/>
+      <c r="C6" s="675" t="n"/>
+      <c r="D6" s="675" t="n"/>
+      <c r="E6" s="675" t="n"/>
+      <c r="F6" s="675" t="n"/>
+      <c r="G6" s="675" t="n"/>
+      <c r="H6" s="675" t="n"/>
       <c r="I6" s="3" t="n"/>
       <c r="J6" s="3" t="n"/>
     </row>
-    <row r="7">
-      <c r="A7" s="666" t="n"/>
-      <c r="B7" s="666" t="n"/>
-      <c r="C7" s="666" t="n"/>
-      <c r="D7" s="666" t="n"/>
-      <c r="E7" s="666" t="n"/>
-      <c r="F7" s="666" t="n"/>
-      <c r="G7" s="666" t="n"/>
-      <c r="H7" s="666" t="n"/>
+    <row r="7" ht="12.00188976377953" customHeight="1">
+      <c r="A7" s="675" t="n"/>
+      <c r="B7" s="675" t="n"/>
+      <c r="C7" s="675" t="n"/>
+      <c r="D7" s="675" t="n"/>
+      <c r="E7" s="675" t="n"/>
+      <c r="F7" s="675" t="n"/>
+      <c r="G7" s="675" t="n"/>
+      <c r="H7" s="675" t="n"/>
       <c r="I7" s="3" t="n"/>
       <c r="J7" s="3" t="n"/>
     </row>
-    <row r="8">
-      <c r="A8" s="666" t="n"/>
-      <c r="B8" s="666" t="n"/>
-      <c r="C8" s="666" t="n"/>
-      <c r="D8" s="666" t="n"/>
-      <c r="E8" s="666" t="n"/>
-      <c r="F8" s="666" t="n"/>
-      <c r="G8" s="666" t="n"/>
-      <c r="H8" s="666" t="n"/>
+    <row r="8" ht="12.00188976377953" customHeight="1">
+      <c r="A8" s="675" t="n"/>
+      <c r="B8" s="675" t="n"/>
+      <c r="C8" s="675" t="n"/>
+      <c r="D8" s="675" t="n"/>
+      <c r="E8" s="675" t="n"/>
+      <c r="F8" s="675" t="n"/>
+      <c r="G8" s="675" t="n"/>
+      <c r="H8" s="675" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
     </row>
-    <row r="9">
-      <c r="A9" s="666" t="n"/>
-      <c r="B9" s="666" t="n"/>
-      <c r="C9" s="666" t="n"/>
-      <c r="D9" s="666" t="n"/>
-      <c r="E9" s="666" t="n"/>
-      <c r="F9" s="666" t="n"/>
-      <c r="G9" s="666" t="n"/>
-      <c r="H9" s="666" t="n"/>
+    <row r="9" ht="12.00188976377953" customHeight="1">
+      <c r="A9" s="675" t="n"/>
+      <c r="B9" s="675" t="n"/>
+      <c r="C9" s="675" t="n"/>
+      <c r="D9" s="675" t="n"/>
+      <c r="E9" s="675" t="n"/>
+      <c r="F9" s="675" t="n"/>
+      <c r="G9" s="675" t="n"/>
+      <c r="H9" s="675" t="n"/>
       <c r="I9" s="3" t="n"/>
       <c r="J9" s="3" t="n"/>
     </row>
-    <row r="10">
-      <c r="A10" s="666" t="n"/>
-      <c r="B10" s="666" t="n"/>
-      <c r="C10" s="666" t="n"/>
-      <c r="D10" s="666" t="n"/>
-      <c r="E10" s="666" t="n"/>
-      <c r="F10" s="666" t="n"/>
-      <c r="G10" s="666" t="n"/>
-      <c r="H10" s="666" t="n"/>
+    <row r="10" ht="12.00188976377953" customHeight="1">
+      <c r="A10" s="675" t="n"/>
+      <c r="B10" s="675" t="n"/>
+      <c r="C10" s="675" t="n"/>
+      <c r="D10" s="675" t="n"/>
+      <c r="E10" s="675" t="n"/>
+      <c r="F10" s="675" t="n"/>
+      <c r="G10" s="675" t="n"/>
+      <c r="H10" s="675" t="n"/>
       <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="n"/>
     </row>
-    <row r="11">
-      <c r="A11" s="666" t="n"/>
-      <c r="B11" s="666" t="n"/>
-      <c r="C11" s="666" t="n"/>
-      <c r="D11" s="666" t="n"/>
-      <c r="E11" s="666" t="n"/>
-      <c r="F11" s="666" t="n"/>
-      <c r="G11" s="666" t="n"/>
-      <c r="H11" s="666" t="n"/>
+    <row r="11" ht="12.00188976377953" customHeight="1">
+      <c r="A11" s="675" t="n"/>
+      <c r="B11" s="675" t="n"/>
+      <c r="C11" s="675" t="n"/>
+      <c r="D11" s="675" t="n"/>
+      <c r="E11" s="675" t="n"/>
+      <c r="F11" s="675" t="n"/>
+      <c r="G11" s="675" t="n"/>
+      <c r="H11" s="675" t="n"/>
       <c r="I11" s="3" t="n"/>
       <c r="J11" s="3" t="n"/>
     </row>
-    <row r="12">
-      <c r="A12" s="666" t="n"/>
-      <c r="B12" s="666" t="n"/>
-      <c r="C12" s="666" t="n"/>
-      <c r="D12" s="666" t="n"/>
-      <c r="E12" s="666" t="n"/>
-      <c r="F12" s="666" t="n"/>
-      <c r="G12" s="666" t="n"/>
-      <c r="H12" s="666" t="n"/>
+    <row r="12" ht="12.00188976377953" customHeight="1">
+      <c r="A12" s="675" t="n"/>
+      <c r="B12" s="675" t="n"/>
+      <c r="C12" s="675" t="n"/>
+      <c r="D12" s="675" t="n"/>
+      <c r="E12" s="675" t="n"/>
+      <c r="F12" s="675" t="n"/>
+      <c r="G12" s="675" t="n"/>
+      <c r="H12" s="675" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
     </row>
-    <row r="13">
-      <c r="A13" s="666" t="n"/>
-      <c r="B13" s="666" t="n"/>
-      <c r="C13" s="666" t="n"/>
-      <c r="D13" s="666" t="n"/>
-      <c r="E13" s="666" t="n"/>
-      <c r="F13" s="666" t="n"/>
-      <c r="G13" s="666" t="n"/>
-      <c r="H13" s="666" t="n"/>
+    <row r="13" ht="12.00188976377953" customHeight="1">
+      <c r="A13" s="675" t="n"/>
+      <c r="B13" s="675" t="n"/>
+      <c r="C13" s="675" t="n"/>
+      <c r="D13" s="675" t="n"/>
+      <c r="E13" s="675" t="n"/>
+      <c r="F13" s="675" t="n"/>
+      <c r="G13" s="675" t="n"/>
+      <c r="H13" s="675" t="n"/>
       <c r="I13" s="3" t="n"/>
       <c r="J13" s="3" t="n"/>
     </row>
-    <row r="14">
-      <c r="A14" s="666" t="n"/>
-      <c r="B14" s="666" t="n"/>
-      <c r="C14" s="666" t="n"/>
-      <c r="D14" s="666" t="n"/>
-      <c r="E14" s="666" t="n"/>
-      <c r="F14" s="666" t="n"/>
-      <c r="G14" s="666" t="n"/>
-      <c r="H14" s="666" t="n"/>
+    <row r="14" ht="12.00188976377953" customHeight="1">
+      <c r="A14" s="675" t="n"/>
+      <c r="B14" s="675" t="n"/>
+      <c r="C14" s="675" t="n"/>
+      <c r="D14" s="675" t="n"/>
+      <c r="E14" s="675" t="n"/>
+      <c r="F14" s="675" t="n"/>
+      <c r="G14" s="675" t="n"/>
+      <c r="H14" s="675" t="n"/>
       <c r="I14" s="3" t="n"/>
       <c r="J14" s="3" t="n"/>
     </row>
-    <row r="15">
-      <c r="A15" s="666" t="n"/>
-      <c r="B15" s="666" t="n"/>
-      <c r="C15" s="666" t="n"/>
-      <c r="D15" s="666" t="n"/>
-      <c r="E15" s="666" t="n"/>
-      <c r="F15" s="666" t="n"/>
-      <c r="G15" s="666" t="n"/>
-      <c r="H15" s="666" t="n"/>
+    <row r="15" ht="12.00188976377953" customHeight="1">
+      <c r="A15" s="675" t="n"/>
+      <c r="B15" s="675" t="n"/>
+      <c r="C15" s="675" t="n"/>
+      <c r="D15" s="675" t="n"/>
+      <c r="E15" s="675" t="n"/>
+      <c r="F15" s="675" t="n"/>
+      <c r="G15" s="675" t="n"/>
+      <c r="H15" s="675" t="n"/>
       <c r="I15" s="3" t="n"/>
       <c r="J15" s="3" t="n"/>
     </row>
-    <row r="16">
-      <c r="A16" s="666" t="n"/>
-      <c r="B16" s="666" t="n"/>
-      <c r="C16" s="666" t="n"/>
-      <c r="D16" s="666" t="n"/>
-      <c r="E16" s="666" t="n"/>
-      <c r="F16" s="666" t="n"/>
-      <c r="G16" s="666" t="n"/>
-      <c r="H16" s="666" t="n"/>
+    <row r="16" ht="12.00188976377953" customHeight="1">
+      <c r="A16" s="675" t="n"/>
+      <c r="B16" s="675" t="n"/>
+      <c r="C16" s="675" t="n"/>
+      <c r="D16" s="675" t="n"/>
+      <c r="E16" s="675" t="n"/>
+      <c r="F16" s="675" t="n"/>
+      <c r="G16" s="675" t="n"/>
+      <c r="H16" s="675" t="n"/>
       <c r="I16" s="3" t="n"/>
       <c r="J16" s="3" t="n"/>
     </row>
-    <row r="17">
-      <c r="A17" s="666" t="n"/>
-      <c r="B17" s="666" t="n"/>
-      <c r="C17" s="666" t="n"/>
-      <c r="D17" s="666" t="n"/>
-      <c r="E17" s="666" t="n"/>
-      <c r="F17" s="666" t="n"/>
-      <c r="G17" s="666" t="n"/>
-      <c r="H17" s="666" t="n"/>
+    <row r="17" ht="12.00188976377953" customHeight="1">
+      <c r="A17" s="675" t="n"/>
+      <c r="B17" s="675" t="n"/>
+      <c r="C17" s="675" t="n"/>
+      <c r="D17" s="675" t="n"/>
+      <c r="E17" s="675" t="n"/>
+      <c r="F17" s="675" t="n"/>
+      <c r="G17" s="675" t="n"/>
+      <c r="H17" s="675" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="3" t="n"/>
     </row>
-    <row r="18">
-      <c r="A18" s="666" t="n"/>
-      <c r="B18" s="666" t="n"/>
-      <c r="C18" s="666" t="n"/>
-      <c r="D18" s="666" t="n"/>
-      <c r="E18" s="666" t="n"/>
-      <c r="F18" s="666" t="n"/>
-      <c r="G18" s="666" t="n"/>
-      <c r="H18" s="666" t="n"/>
+    <row r="18" ht="12.00188976377953" customHeight="1">
+      <c r="A18" s="675" t="n"/>
+      <c r="B18" s="675" t="n"/>
+      <c r="C18" s="675" t="n"/>
+      <c r="D18" s="675" t="n"/>
+      <c r="E18" s="675" t="n"/>
+      <c r="F18" s="675" t="n"/>
+      <c r="G18" s="675" t="n"/>
+      <c r="H18" s="675" t="n"/>
       <c r="I18" s="3" t="n"/>
       <c r="J18" s="3" t="n"/>
     </row>
-    <row r="19">
-      <c r="A19" s="666" t="n"/>
-      <c r="B19" s="666" t="n"/>
-      <c r="C19" s="666" t="n"/>
-      <c r="D19" s="666" t="n"/>
-      <c r="E19" s="666" t="n"/>
-      <c r="F19" s="666" t="n"/>
-      <c r="G19" s="666" t="n"/>
-      <c r="H19" s="666" t="n"/>
+    <row r="19" ht="12.00188976377953" customHeight="1">
+      <c r="A19" s="675" t="n"/>
+      <c r="B19" s="675" t="n"/>
+      <c r="C19" s="675" t="n"/>
+      <c r="D19" s="675" t="n"/>
+      <c r="E19" s="675" t="n"/>
+      <c r="F19" s="675" t="n"/>
+      <c r="G19" s="675" t="n"/>
+      <c r="H19" s="675" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
     </row>
-    <row r="20">
-      <c r="A20" s="666" t="n"/>
-      <c r="B20" s="666" t="n"/>
-      <c r="C20" s="666" t="n"/>
-      <c r="D20" s="666" t="n"/>
-      <c r="E20" s="666" t="n"/>
-      <c r="F20" s="666" t="n"/>
-      <c r="G20" s="666" t="n"/>
-      <c r="H20" s="666" t="n"/>
+    <row r="20" ht="12.00188976377953" customHeight="1">
+      <c r="A20" s="675" t="n"/>
+      <c r="B20" s="675" t="n"/>
+      <c r="C20" s="675" t="n"/>
+      <c r="D20" s="675" t="n"/>
+      <c r="E20" s="675" t="n"/>
+      <c r="F20" s="675" t="n"/>
+      <c r="G20" s="675" t="n"/>
+      <c r="H20" s="675" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="3" t="n"/>
     </row>
-    <row r="21">
-      <c r="A21" s="666" t="n"/>
-      <c r="B21" s="666" t="n"/>
-      <c r="C21" s="666" t="n"/>
-      <c r="D21" s="666" t="n"/>
-      <c r="E21" s="666" t="n"/>
-      <c r="F21" s="666" t="n"/>
-      <c r="G21" s="666" t="n"/>
-      <c r="H21" s="666" t="n"/>
+    <row r="21" ht="12.00188976377953" customHeight="1">
+      <c r="A21" s="675" t="n"/>
+      <c r="B21" s="675" t="n"/>
+      <c r="C21" s="675" t="n"/>
+      <c r="D21" s="675" t="n"/>
+      <c r="E21" s="675" t="n"/>
+      <c r="F21" s="675" t="n"/>
+      <c r="G21" s="675" t="n"/>
+      <c r="H21" s="675" t="n"/>
       <c r="I21" s="3" t="n"/>
       <c r="J21" s="3" t="n"/>
     </row>
-    <row r="22">
-      <c r="A22" s="666" t="n"/>
-      <c r="B22" s="666" t="n"/>
-      <c r="C22" s="666" t="n"/>
-      <c r="D22" s="666" t="n"/>
-      <c r="E22" s="666" t="n"/>
-      <c r="F22" s="666" t="n"/>
-      <c r="G22" s="666" t="n"/>
-      <c r="H22" s="666" t="n"/>
+    <row r="22" ht="12.00188976377953" customHeight="1">
+      <c r="A22" s="675" t="n"/>
+      <c r="B22" s="675" t="n"/>
+      <c r="C22" s="675" t="n"/>
+      <c r="D22" s="675" t="n"/>
+      <c r="E22" s="675" t="n"/>
+      <c r="F22" s="675" t="n"/>
+      <c r="G22" s="675" t="n"/>
+      <c r="H22" s="675" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
     </row>
-    <row r="23">
-      <c r="A23" s="666" t="n"/>
-      <c r="B23" s="666" t="n"/>
-      <c r="C23" s="666" t="n"/>
-      <c r="D23" s="666" t="n"/>
-      <c r="E23" s="666" t="n"/>
-      <c r="F23" s="666" t="n"/>
-      <c r="G23" s="666" t="n"/>
-      <c r="H23" s="666" t="n"/>
+    <row r="23" ht="12.00188976377953" customHeight="1">
+      <c r="A23" s="675" t="n"/>
+      <c r="B23" s="675" t="n"/>
+      <c r="C23" s="675" t="n"/>
+      <c r="D23" s="675" t="n"/>
+      <c r="E23" s="675" t="n"/>
+      <c r="F23" s="675" t="n"/>
+      <c r="G23" s="675" t="n"/>
+      <c r="H23" s="675" t="n"/>
       <c r="I23" s="3" t="n"/>
       <c r="J23" s="3" t="n"/>
     </row>
-    <row r="24">
-      <c r="A24" s="666" t="n"/>
-      <c r="B24" s="666" t="n"/>
-      <c r="C24" s="666" t="n"/>
-      <c r="D24" s="666" t="n"/>
-      <c r="E24" s="666" t="n"/>
-      <c r="F24" s="666" t="n"/>
-      <c r="G24" s="666" t="n"/>
-      <c r="H24" s="666" t="n"/>
+    <row r="24" ht="12.00188976377953" customHeight="1">
+      <c r="A24" s="675" t="n"/>
+      <c r="B24" s="675" t="n"/>
+      <c r="C24" s="675" t="n"/>
+      <c r="D24" s="675" t="n"/>
+      <c r="E24" s="675" t="n"/>
+      <c r="F24" s="675" t="n"/>
+      <c r="G24" s="675" t="n"/>
+      <c r="H24" s="675" t="n"/>
       <c r="I24" s="3" t="n"/>
       <c r="J24" s="3" t="n"/>
     </row>
-    <row r="25">
-      <c r="A25" s="666" t="n"/>
-      <c r="B25" s="666" t="n"/>
-      <c r="C25" s="666" t="n"/>
-      <c r="D25" s="666" t="n"/>
-      <c r="E25" s="666" t="n"/>
-      <c r="F25" s="666" t="n"/>
-      <c r="G25" s="666" t="n"/>
-      <c r="H25" s="666" t="n"/>
+    <row r="25" ht="12.00188976377953" customHeight="1">
+      <c r="A25" s="675" t="n"/>
+      <c r="B25" s="675" t="n"/>
+      <c r="C25" s="675" t="n"/>
+      <c r="D25" s="675" t="n"/>
+      <c r="E25" s="675" t="n"/>
+      <c r="F25" s="675" t="n"/>
+      <c r="G25" s="675" t="n"/>
+      <c r="H25" s="675" t="n"/>
       <c r="I25" s="3" t="n"/>
       <c r="J25" s="3" t="n"/>
     </row>
-    <row r="26">
-      <c r="A26" s="666" t="n"/>
-      <c r="B26" s="666" t="n"/>
-      <c r="C26" s="666" t="n"/>
-      <c r="D26" s="666" t="n"/>
-      <c r="E26" s="666" t="n"/>
-      <c r="F26" s="666" t="n"/>
-      <c r="G26" s="666" t="n"/>
-      <c r="H26" s="666" t="n"/>
+    <row r="26" ht="12.00188976377953" customHeight="1">
+      <c r="A26" s="675" t="n"/>
+      <c r="B26" s="675" t="n"/>
+      <c r="C26" s="675" t="n"/>
+      <c r="D26" s="675" t="n"/>
+      <c r="E26" s="675" t="n"/>
+      <c r="F26" s="675" t="n"/>
+      <c r="G26" s="675" t="n"/>
+      <c r="H26" s="675" t="n"/>
       <c r="I26" s="3" t="n"/>
       <c r="J26" s="3" t="n"/>
     </row>
-    <row r="27">
-      <c r="A27" s="666" t="n"/>
-      <c r="B27" s="666" t="n"/>
-      <c r="C27" s="666" t="n"/>
-      <c r="D27" s="666" t="n"/>
-      <c r="E27" s="666" t="n"/>
-      <c r="F27" s="666" t="n"/>
-      <c r="G27" s="666" t="n"/>
-      <c r="H27" s="666" t="n"/>
+    <row r="27" ht="12.00188976377953" customHeight="1">
+      <c r="A27" s="675" t="n"/>
+      <c r="B27" s="675" t="n"/>
+      <c r="C27" s="675" t="n"/>
+      <c r="D27" s="675" t="n"/>
+      <c r="E27" s="675" t="n"/>
+      <c r="F27" s="675" t="n"/>
+      <c r="G27" s="675" t="n"/>
+      <c r="H27" s="675" t="n"/>
       <c r="I27" s="3" t="n"/>
       <c r="J27" s="3" t="n"/>
     </row>
-    <row r="28">
-      <c r="A28" s="666" t="n"/>
-      <c r="B28" s="666" t="n"/>
-      <c r="C28" s="666" t="n"/>
-      <c r="D28" s="666" t="n"/>
-      <c r="E28" s="666" t="n"/>
-      <c r="F28" s="666" t="n"/>
-      <c r="G28" s="666" t="n"/>
-      <c r="H28" s="666" t="n"/>
+    <row r="28" ht="12.00188976377953" customHeight="1">
+      <c r="A28" s="675" t="n"/>
+      <c r="B28" s="675" t="n"/>
+      <c r="C28" s="675" t="n"/>
+      <c r="D28" s="675" t="n"/>
+      <c r="E28" s="675" t="n"/>
+      <c r="F28" s="675" t="n"/>
+      <c r="G28" s="675" t="n"/>
+      <c r="H28" s="675" t="n"/>
       <c r="I28" s="3" t="n"/>
       <c r="J28" s="3" t="n"/>
     </row>
-    <row r="29">
-      <c r="A29" s="666" t="n"/>
-      <c r="B29" s="666" t="n"/>
-      <c r="C29" s="666" t="n"/>
-      <c r="D29" s="666" t="n"/>
-      <c r="E29" s="666" t="n"/>
-      <c r="F29" s="666" t="n"/>
-      <c r="G29" s="666" t="n"/>
-      <c r="H29" s="666" t="n"/>
+    <row r="29" ht="12.00188976377953" customHeight="1">
+      <c r="A29" s="675" t="n"/>
+      <c r="B29" s="675" t="n"/>
+      <c r="C29" s="675" t="n"/>
+      <c r="D29" s="675" t="n"/>
+      <c r="E29" s="675" t="n"/>
+      <c r="F29" s="675" t="n"/>
+      <c r="G29" s="675" t="n"/>
+      <c r="H29" s="675" t="n"/>
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
     </row>
-    <row r="30">
-      <c r="A30" s="666" t="n"/>
-      <c r="B30" s="666" t="n"/>
-      <c r="C30" s="666" t="n"/>
-      <c r="D30" s="666" t="n"/>
-      <c r="E30" s="666" t="n"/>
-      <c r="F30" s="666" t="n"/>
-      <c r="G30" s="666" t="n"/>
-      <c r="H30" s="666" t="n"/>
+    <row r="30" ht="12.00188976377953" customHeight="1">
+      <c r="A30" s="675" t="n"/>
+      <c r="B30" s="675" t="n"/>
+      <c r="C30" s="675" t="n"/>
+      <c r="D30" s="675" t="n"/>
+      <c r="E30" s="675" t="n"/>
+      <c r="F30" s="675" t="n"/>
+      <c r="G30" s="675" t="n"/>
+      <c r="H30" s="675" t="n"/>
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
     </row>
-    <row r="31">
-      <c r="A31" s="666" t="n"/>
-      <c r="B31" s="666" t="n"/>
-      <c r="C31" s="666" t="n"/>
-      <c r="D31" s="666" t="n"/>
-      <c r="E31" s="666" t="n"/>
-      <c r="F31" s="666" t="n"/>
-      <c r="G31" s="666" t="n"/>
-      <c r="H31" s="666" t="n"/>
+    <row r="31" ht="12.00188976377953" customHeight="1">
+      <c r="A31" s="675" t="n"/>
+      <c r="B31" s="675" t="n"/>
+      <c r="C31" s="675" t="n"/>
+      <c r="D31" s="675" t="n"/>
+      <c r="E31" s="675" t="n"/>
+      <c r="F31" s="675" t="n"/>
+      <c r="G31" s="675" t="n"/>
+      <c r="H31" s="675" t="n"/>
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
     </row>
-    <row r="32">
-      <c r="A32" s="666" t="n"/>
-      <c r="B32" s="666" t="n"/>
-      <c r="C32" s="666" t="n"/>
-      <c r="D32" s="666" t="n"/>
-      <c r="E32" s="666" t="n"/>
-      <c r="F32" s="666" t="n"/>
-      <c r="G32" s="666" t="n"/>
-      <c r="H32" s="666" t="n"/>
+    <row r="32" ht="12.00188976377953" customHeight="1">
+      <c r="A32" s="675" t="n"/>
+      <c r="B32" s="675" t="n"/>
+      <c r="C32" s="675" t="n"/>
+      <c r="D32" s="675" t="n"/>
+      <c r="E32" s="675" t="n"/>
+      <c r="F32" s="675" t="n"/>
+      <c r="G32" s="675" t="n"/>
+      <c r="H32" s="675" t="n"/>
       <c r="I32" s="3" t="n"/>
       <c r="J32" s="3" t="n"/>
     </row>
-    <row r="33">
-      <c r="A33" s="666" t="n"/>
-      <c r="B33" s="666" t="n"/>
-      <c r="C33" s="666" t="n"/>
-      <c r="D33" s="666" t="n"/>
-      <c r="E33" s="666" t="n"/>
-      <c r="F33" s="666" t="n"/>
-      <c r="G33" s="666" t="n"/>
-      <c r="H33" s="666" t="n"/>
+    <row r="33" ht="12.00188976377953" customHeight="1">
+      <c r="A33" s="675" t="n"/>
+      <c r="B33" s="675" t="n"/>
+      <c r="C33" s="675" t="n"/>
+      <c r="D33" s="675" t="n"/>
+      <c r="E33" s="675" t="n"/>
+      <c r="F33" s="675" t="n"/>
+      <c r="G33" s="675" t="n"/>
+      <c r="H33" s="675" t="n"/>
       <c r="I33" s="3" t="n"/>
       <c r="J33" s="3" t="n"/>
     </row>
-    <row r="34">
-      <c r="A34" s="666" t="n"/>
-      <c r="B34" s="666" t="n"/>
-      <c r="C34" s="666" t="n"/>
-      <c r="D34" s="666" t="n"/>
-      <c r="E34" s="666" t="n"/>
-      <c r="F34" s="666" t="n"/>
-      <c r="G34" s="666" t="n"/>
-      <c r="H34" s="666" t="n"/>
+    <row r="34" ht="12.00188976377953" customHeight="1">
+      <c r="A34" s="675" t="n"/>
+      <c r="B34" s="675" t="n"/>
+      <c r="C34" s="675" t="n"/>
+      <c r="D34" s="675" t="n"/>
+      <c r="E34" s="675" t="n"/>
+      <c r="F34" s="675" t="n"/>
+      <c r="G34" s="675" t="n"/>
+      <c r="H34" s="675" t="n"/>
       <c r="I34" s="3" t="n"/>
       <c r="J34" s="3" t="n"/>
     </row>
-    <row r="35">
-      <c r="A35" s="666" t="n"/>
-      <c r="B35" s="666" t="n"/>
-      <c r="C35" s="666" t="n"/>
-      <c r="D35" s="666" t="n"/>
-      <c r="E35" s="666" t="n"/>
-      <c r="F35" s="666" t="n"/>
-      <c r="G35" s="666" t="n"/>
-      <c r="H35" s="666" t="n"/>
+    <row r="35" ht="12.00188976377953" customHeight="1">
+      <c r="A35" s="675" t="n"/>
+      <c r="B35" s="675" t="n"/>
+      <c r="C35" s="675" t="n"/>
+      <c r="D35" s="675" t="n"/>
+      <c r="E35" s="675" t="n"/>
+      <c r="F35" s="675" t="n"/>
+      <c r="G35" s="675" t="n"/>
+      <c r="H35" s="675" t="n"/>
       <c r="I35" s="3" t="n"/>
       <c r="J35" s="3" t="n"/>
     </row>
-    <row r="36">
-      <c r="A36" s="666" t="n"/>
-      <c r="B36" s="666" t="n"/>
-      <c r="C36" s="666" t="n"/>
-      <c r="D36" s="666" t="n"/>
-      <c r="E36" s="666" t="n"/>
-      <c r="F36" s="666" t="n"/>
-      <c r="G36" s="666" t="n"/>
-      <c r="H36" s="666" t="n"/>
+    <row r="36" ht="12.00188976377953" customHeight="1">
+      <c r="A36" s="675" t="n"/>
+      <c r="B36" s="675" t="n"/>
+      <c r="C36" s="675" t="n"/>
+      <c r="D36" s="675" t="n"/>
+      <c r="E36" s="675" t="n"/>
+      <c r="F36" s="675" t="n"/>
+      <c r="G36" s="675" t="n"/>
+      <c r="H36" s="675" t="n"/>
       <c r="I36" s="3" t="n"/>
       <c r="J36" s="3" t="n"/>
     </row>
-    <row r="37">
-      <c r="A37" s="666" t="n"/>
-      <c r="B37" s="666" t="n"/>
-      <c r="C37" s="666" t="n"/>
-      <c r="D37" s="666" t="n"/>
-      <c r="E37" s="666" t="n"/>
-      <c r="F37" s="666" t="n"/>
-      <c r="G37" s="666" t="n"/>
-      <c r="H37" s="666" t="n"/>
+    <row r="37" ht="12.00188976377953" customHeight="1">
+      <c r="A37" s="675" t="n"/>
+      <c r="B37" s="675" t="n"/>
+      <c r="C37" s="675" t="n"/>
+      <c r="D37" s="675" t="n"/>
+      <c r="E37" s="675" t="n"/>
+      <c r="F37" s="675" t="n"/>
+      <c r="G37" s="675" t="n"/>
+      <c r="H37" s="675" t="n"/>
       <c r="I37" s="3" t="n"/>
       <c r="J37" s="3" t="n"/>
     </row>
-    <row r="38">
-      <c r="A38" s="666" t="n"/>
-      <c r="B38" s="666" t="n"/>
-      <c r="C38" s="666" t="n"/>
-      <c r="D38" s="666" t="n"/>
-      <c r="E38" s="666" t="n"/>
-      <c r="F38" s="666" t="n"/>
-      <c r="G38" s="666" t="n"/>
-      <c r="H38" s="666" t="n"/>
+    <row r="38" ht="12.00188976377953" customHeight="1">
+      <c r="A38" s="675" t="n"/>
+      <c r="B38" s="675" t="n"/>
+      <c r="C38" s="675" t="n"/>
+      <c r="D38" s="675" t="n"/>
+      <c r="E38" s="675" t="n"/>
+      <c r="F38" s="675" t="n"/>
+      <c r="G38" s="675" t="n"/>
+      <c r="H38" s="675" t="n"/>
       <c r="I38" s="3" t="n"/>
       <c r="J38" s="3" t="n"/>
     </row>
-    <row r="39">
-      <c r="A39" s="666" t="n"/>
-      <c r="B39" s="666" t="n"/>
-      <c r="C39" s="666" t="n"/>
-      <c r="D39" s="666" t="n"/>
-      <c r="E39" s="666" t="n"/>
-      <c r="F39" s="666" t="n"/>
-      <c r="G39" s="666" t="n"/>
-      <c r="H39" s="666" t="n"/>
+    <row r="39" ht="12.00188976377953" customHeight="1">
+      <c r="A39" s="675" t="n"/>
+      <c r="B39" s="675" t="n"/>
+      <c r="C39" s="675" t="n"/>
+      <c r="D39" s="675" t="n"/>
+      <c r="E39" s="675" t="n"/>
+      <c r="F39" s="675" t="n"/>
+      <c r="G39" s="675" t="n"/>
+      <c r="H39" s="675" t="n"/>
       <c r="I39" s="3" t="n"/>
       <c r="J39" s="3" t="n"/>
     </row>
-    <row r="40">
-      <c r="A40" s="666" t="n"/>
-      <c r="B40" s="666" t="n"/>
-      <c r="C40" s="666" t="n"/>
-      <c r="D40" s="666" t="n"/>
-      <c r="E40" s="666" t="n"/>
-      <c r="F40" s="666" t="n"/>
-      <c r="G40" s="666" t="n"/>
-      <c r="H40" s="666" t="n"/>
+    <row r="40" ht="12.00188976377953" customHeight="1">
+      <c r="A40" s="675" t="n"/>
+      <c r="B40" s="675" t="n"/>
+      <c r="C40" s="675" t="n"/>
+      <c r="D40" s="675" t="n"/>
+      <c r="E40" s="675" t="n"/>
+      <c r="F40" s="675" t="n"/>
+      <c r="G40" s="675" t="n"/>
+      <c r="H40" s="675" t="n"/>
       <c r="I40" s="3" t="n"/>
       <c r="J40" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.2" footer="0.2"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>